<commit_message>
Refactor orb mechanics to introduce new orb types and enhance gameplay dynamics
- Replaced the previous chaos orb types (Shadow, Poison, Electric) with new orbs (Ghost, Rot, Conduit) that launch from the summoning circle at level start, improving strategic options and elemental interactions.
- Updated project structure to reflect the new orb organization under `entities/orbs/`, enhancing clarity and maintainability.
- Revised `level.gd` to manage the spawning and behavior of the new orbs, ensuring they follow the intended gameplay mechanics.
- Adjusted relevant documentation in `DECISIONS.md`, `GAME_BRIEF.md`, and `PROJECT_MAP.md` to reflect the introduction of new orb types and their implications for player strategy and interactions.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,19 +8,21 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\One Last Bullet\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0E309ADC-E0E7-46B8-B514-9A5D577E2EFA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B59C5EA-C6FF-4C4E-AD42-1A985500D97F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="5430" yWindow="4515" windowWidth="28800" windowHeight="15345" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
-    <sheet name="objects_OLD" sheetId="3" state="hidden" r:id="rId2"/>
-    <sheet name="input" sheetId="13" r:id="rId3"/>
-    <sheet name="schema" sheetId="14" r:id="rId4"/>
+    <sheet name="glyphs" sheetId="15" r:id="rId2"/>
+    <sheet name="motion" sheetId="16" r:id="rId3"/>
+    <sheet name="objects_OLD" sheetId="3" state="hidden" r:id="rId4"/>
+    <sheet name="input" sheetId="13" r:id="rId5"/>
+    <sheet name="schema" sheetId="14" r:id="rId6"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">objects_OLD!$A$1:$U$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">orbs!$A$1:$H$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">objects_OLD!$A$1:$U$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">orbs!$A$1:$R$44</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="419" uniqueCount="170">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="216">
   <si>
     <t>id</t>
   </si>
@@ -54,12 +56,6 @@
     <t>type</t>
   </si>
   <si>
-    <t>action_1</t>
-  </si>
-  <si>
-    <t>action_2</t>
-  </si>
-  <si>
     <t>effect</t>
   </si>
   <si>
@@ -375,42 +371,9 @@
     <t>hanging_meat</t>
   </si>
   <si>
-    <t>tag_1</t>
-  </si>
-  <si>
-    <t>tag_2</t>
-  </si>
-  <si>
-    <t>tag_3</t>
-  </si>
-  <si>
-    <t>effect_desc</t>
-  </si>
-  <si>
-    <t>level_value_1</t>
-  </si>
-  <si>
-    <t>level_value_2</t>
-  </si>
-  <si>
-    <t>level_value_3</t>
-  </si>
-  <si>
-    <t>req_room_adjacency</t>
-  </si>
-  <si>
-    <t>room_size_cap</t>
-  </si>
-  <si>
-    <t>placeable_budget</t>
-  </si>
-  <si>
     <t>scene_path</t>
   </si>
   <si>
-    <t>res://areas/rooms/bedroom/cozy_cot.tscn</t>
-  </si>
-  <si>
     <t>fun</t>
   </si>
   <si>
@@ -432,131 +395,308 @@
     <t>+1 decor for every plant in the room</t>
   </si>
   <si>
-    <t>input_item_1</t>
-  </si>
-  <si>
-    <t>input_item_1_quantity</t>
-  </si>
-  <si>
-    <t>input_item_2</t>
-  </si>
-  <si>
-    <t>input_item_2_quantity</t>
-  </si>
-  <si>
-    <t>output_item</t>
-  </si>
-  <si>
-    <t>output_item_quantity</t>
-  </si>
-  <si>
-    <t>cook_time</t>
-  </si>
-  <si>
-    <t>base_quality</t>
-  </si>
-  <si>
-    <t>group_id</t>
-  </si>
-  <si>
-    <t>stage</t>
-  </si>
-  <si>
-    <t>trigger_condition</t>
-  </si>
-  <si>
-    <t>progress_condition</t>
-  </si>
-  <si>
-    <t>progress_goal</t>
-  </si>
-  <si>
-    <t>flavor_text</t>
-  </si>
-  <si>
-    <t>satisfaction</t>
-  </si>
-  <si>
-    <t>effect_1</t>
-  </si>
-  <si>
-    <t>effect_2</t>
-  </si>
-  <si>
-    <t>effect_3</t>
-  </si>
-  <si>
-    <t>duration_hours</t>
-  </si>
-  <si>
-    <t>additive</t>
-  </si>
-  <si>
-    <t>slot</t>
-  </si>
-  <si>
-    <t>typical_sources</t>
-  </si>
-  <si>
-    <t>objects</t>
-  </si>
-  <si>
     <t>sheet</t>
   </si>
   <si>
     <t>column</t>
   </si>
   <si>
-    <t>rooms</t>
-  </si>
-  <si>
     <t>string</t>
   </si>
   <si>
     <t>int</t>
   </si>
   <si>
-    <t>dict</t>
-  </si>
-  <si>
     <t>boolean</t>
   </si>
   <si>
-    <t>recipes</t>
-  </si>
-  <si>
     <t>float</t>
   </si>
   <si>
-    <t>foods</t>
-  </si>
-  <si>
-    <t>room_tags</t>
-  </si>
-  <si>
-    <t>actions</t>
-  </si>
-  <si>
-    <t>memories</t>
-  </si>
-  <si>
-    <t>statuses</t>
-  </si>
-  <si>
     <t>orbs</t>
   </si>
   <si>
-    <t>basic_orb</t>
-  </si>
-  <si>
     <t>Standard orb with no effect</t>
+  </si>
+  <si>
+    <t>Burn on enemy hit</t>
+  </si>
+  <si>
+    <t>Fire</t>
+  </si>
+  <si>
+    <t>Damage</t>
+  </si>
+  <si>
+    <t>On hit, that % of the damage also hits nearby enemies</t>
+  </si>
+  <si>
+    <t>Chill enemy on hit</t>
+  </si>
+  <si>
+    <t>Water</t>
+  </si>
+  <si>
+    <t>This orb deals less damage to players</t>
+  </si>
+  <si>
+    <t>Mana drop chance from enemies</t>
+  </si>
+  <si>
+    <t>Shock on enemy hit</t>
+  </si>
+  <si>
+    <t>Air</t>
+  </si>
+  <si>
+    <t>Critical chance</t>
+  </si>
+  <si>
+    <t>Decreases speed</t>
+  </si>
+  <si>
+    <t>Poison on enemy hit</t>
+  </si>
+  <si>
+    <t>Earth</t>
+  </si>
+  <si>
+    <t>Increases weight</t>
+  </si>
+  <si>
+    <t>Critical damage</t>
+  </si>
+  <si>
+    <t>rarity_common</t>
+  </si>
+  <si>
+    <t>rarity_rare</t>
+  </si>
+  <si>
+    <t>rarity_unique</t>
+  </si>
+  <si>
+    <t>coal</t>
+  </si>
+  <si>
+    <t>fury</t>
+  </si>
+  <si>
+    <t>blast</t>
+  </si>
+  <si>
+    <t>rime</t>
+  </si>
+  <si>
+    <t>soft</t>
+  </si>
+  <si>
+    <t>bounty</t>
+  </si>
+  <si>
+    <t>static</t>
+  </si>
+  <si>
+    <t>drag</t>
+  </si>
+  <si>
+    <t>blight</t>
+  </si>
+  <si>
+    <t>dense</t>
+  </si>
+  <si>
+    <t>crush</t>
+  </si>
+  <si>
+    <t>element</t>
+  </si>
+  <si>
+    <t>shear</t>
+  </si>
+  <si>
+    <t>damage</t>
+  </si>
+  <si>
+    <t>self_damage</t>
+  </si>
+  <si>
+    <t>splash</t>
+  </si>
+  <si>
+    <t>speed</t>
+  </si>
+  <si>
+    <t>weight</t>
+  </si>
+  <si>
+    <t>crit_chance</t>
+  </si>
+  <si>
+    <t>crit_damage</t>
+  </si>
+  <si>
+    <t>crystal_drop</t>
+  </si>
+  <si>
+    <t>burn</t>
+  </si>
+  <si>
+    <t>chill</t>
+  </si>
+  <si>
+    <t>shock</t>
+  </si>
+  <si>
+    <t>poison</t>
+  </si>
+  <si>
+    <t>wayward</t>
+  </si>
+  <si>
+    <t>motion</t>
+  </si>
+  <si>
+    <t>Straight flight, bounce off solids</t>
+  </si>
+  <si>
+    <t>hungry</t>
+  </si>
+  <si>
+    <t>Steer toward nearest enemy</t>
+  </si>
+  <si>
+    <t>spite</t>
+  </si>
+  <si>
+    <t>Steer toward the player</t>
+  </si>
+  <si>
+    <t>rooted</t>
+  </si>
+  <si>
+    <t>Stops in place</t>
+  </si>
+  <si>
+    <t>Travels in a circle</t>
+  </si>
+  <si>
+    <t>patrol</t>
+  </si>
+  <si>
+    <t>familiar</t>
+  </si>
+  <si>
+    <t>Orbit the player</t>
+  </si>
+  <si>
+    <t>rail</t>
+  </si>
+  <si>
+    <t>Slides along walls. Goes opposite way on impact.</t>
+  </si>
+  <si>
+    <t>tide</t>
+  </si>
+  <si>
+    <t>Ping-pong between last redirect and last bounce</t>
+  </si>
+  <si>
+    <t>blink</t>
+  </si>
+  <si>
+    <t>Teleport a short hop on a timer or on wall hit</t>
+  </si>
+  <si>
+    <t>loyal</t>
+  </si>
+  <si>
+    <t>Match the player’s move vector, offset</t>
+  </si>
+  <si>
+    <t>hexed</t>
+  </si>
+  <si>
+    <t>Flee the player</t>
+  </si>
+  <si>
+    <t>stalker</t>
+  </si>
+  <si>
+    <t>Idle until an enemy or player enters range, then lunge</t>
+  </si>
+  <si>
+    <t>herd</t>
+  </si>
+  <si>
+    <t>greedy</t>
+  </si>
+  <si>
+    <t>Steers towards mana crystals</t>
+  </si>
+  <si>
+    <t>Steer towards other orbs</t>
+  </si>
+  <si>
+    <t>oathbound</t>
+  </si>
+  <si>
+    <t>Orbits the summoning circle</t>
+  </si>
+  <si>
+    <t>echo</t>
+  </si>
+  <si>
+    <t>Replay a nearby players path on a 1 s delay</t>
+  </si>
+  <si>
+    <t>phasing</t>
+  </si>
+  <si>
+    <t>Go through entities and obstacles</t>
+  </si>
+  <si>
+    <t>blank</t>
+  </si>
+  <si>
+    <t>conduit</t>
+  </si>
+  <si>
+    <t>rot</t>
+  </si>
+  <si>
+    <t>ghost</t>
+  </si>
+  <si>
+    <t>When you are within 120 meters of the orb, create a tether between you dealing 3 DPS to enemies touching it</t>
+  </si>
+  <si>
+    <t>Enters enemies and deal its impact damage per second to them. Once dead, exits in a random direction</t>
+  </si>
+  <si>
+    <t>Inflict poison on hit</t>
+  </si>
+  <si>
+    <t>glyphs</t>
+  </si>
+  <si>
+    <t>res://entities/orbs/blank/blank_orb.tscn</t>
+  </si>
+  <si>
+    <t>res://entities/orbs/conduit/conduit_orb.tscn</t>
+  </si>
+  <si>
+    <t>res://entities/orbs/rot/rot_orb.tscn</t>
+  </si>
+  <si>
+    <t>res://entities/orbs/ghost/ghost_orb.tscn</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -587,8 +727,15 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="8">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -597,7 +744,37 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor theme="7" tint="0.79998168889431442"/>
+        <fgColor theme="3" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="2" tint="-0.249977111117893"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="4" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -620,10 +797,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -633,11 +811,18 @@
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="0" xfId="1" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
   <dxfs count="6">
     <dxf>
@@ -980,18 +1165,27 @@
   <sheetPr>
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:H44"/>
+  <dimension ref="A1:R44"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" customWidth="1"/>
     <col min="2" max="2" width="17.5703125" customWidth="1"/>
-    <col min="3" max="3" width="48.85546875" customWidth="1"/>
-    <col min="4" max="4" width="30.42578125" bestFit="1" customWidth="1"/>
-    <col min="5" max="6" width="15.7109375" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="47" customWidth="1"/>
+    <col min="3" max="3" width="104.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15" customWidth="1"/>
+    <col min="5" max="5" width="10.42578125" customWidth="1"/>
+    <col min="6" max="6" width="15.42578125" customWidth="1"/>
+    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="8.5703125" customWidth="1"/>
+    <col min="9" max="9" width="9.140625" customWidth="1"/>
+    <col min="10" max="12" width="14.5703125" customWidth="1"/>
+    <col min="13" max="13" width="8.85546875" customWidth="1"/>
+    <col min="14" max="14" width="8.42578125" customWidth="1"/>
+    <col min="15" max="15" width="8.5703125" customWidth="1"/>
+    <col min="16" max="16" width="8.7109375" customWidth="1"/>
+    <col min="17" max="17" width="47" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1001,128 +1195,341 @@
       <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="7" t="s">
-        <v>115</v>
-      </c>
-      <c r="E1" s="7" t="s">
-        <v>116</v>
-      </c>
-      <c r="F1" s="7" t="s">
-        <v>117</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>121</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="D1" s="10" t="s">
+        <v>170</v>
+      </c>
+      <c r="E1" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="F1" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="G1" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="H1" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="I1" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="J1" s="9" t="s">
+        <v>162</v>
+      </c>
+      <c r="K1" s="9" t="s">
+        <v>163</v>
+      </c>
+      <c r="L1" s="9" t="s">
+        <v>164</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>165</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>166</v>
+      </c>
+      <c r="O1" s="9" t="s">
+        <v>167</v>
+      </c>
+      <c r="P1" s="9" t="s">
+        <v>168</v>
+      </c>
+      <c r="Q1" s="13" t="s">
+        <v>109</v>
+      </c>
+      <c r="R1" s="13" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>168</v>
+        <v>204</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B26" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
-        <v>Basic Orb</v>
+        <v>Blank</v>
       </c>
       <c r="C2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D2" t="s">
         <v>169</v>
       </c>
-      <c r="D2" s="6">
+      <c r="E2">
+        <v>10</v>
+      </c>
+      <c r="F2">
+        <v>8</v>
+      </c>
+      <c r="G2" s="8">
+        <v>0</v>
+      </c>
+      <c r="H2">
+        <v>100</v>
+      </c>
+      <c r="I2">
+        <v>10</v>
+      </c>
+      <c r="J2" s="8">
+        <v>0.01</v>
+      </c>
+      <c r="K2" s="8">
+        <v>2</v>
+      </c>
+      <c r="L2" s="8">
         <v>0.1</v>
       </c>
-      <c r="E2" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="F2" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="G2" t="s">
-        <v>122</v>
-      </c>
-      <c r="H2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="M2">
+        <v>0</v>
+      </c>
+      <c r="N2">
+        <v>0</v>
+      </c>
+      <c r="O2">
+        <v>0</v>
+      </c>
+      <c r="P2">
+        <v>0</v>
+      </c>
+      <c r="Q2" t="s">
+        <v>212</v>
+      </c>
+      <c r="R2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>205</v>
+      </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+        <v>Conduit</v>
+      </c>
+      <c r="C3" t="s">
+        <v>208</v>
+      </c>
+      <c r="D3" t="s">
+        <v>169</v>
+      </c>
+      <c r="E3">
+        <v>15</v>
+      </c>
+      <c r="F3">
+        <v>12</v>
+      </c>
+      <c r="G3" s="8">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>130</v>
+      </c>
+      <c r="I3">
+        <v>10</v>
+      </c>
+      <c r="J3" s="8">
+        <v>0.01</v>
+      </c>
+      <c r="K3" s="8">
+        <v>2</v>
+      </c>
+      <c r="L3" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="M3">
+        <v>0</v>
+      </c>
+      <c r="N3">
+        <v>0</v>
+      </c>
+      <c r="O3">
+        <v>3</v>
+      </c>
+      <c r="P3">
+        <v>0</v>
+      </c>
+      <c r="Q3" t="s">
+        <v>213</v>
+      </c>
+      <c r="R3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>206</v>
+      </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+        <v>Rot</v>
+      </c>
+      <c r="C4" t="s">
+        <v>210</v>
+      </c>
+      <c r="D4" t="s">
+        <v>169</v>
+      </c>
+      <c r="E4">
+        <v>10</v>
+      </c>
+      <c r="F4">
+        <v>18</v>
+      </c>
+      <c r="G4" s="8">
+        <v>0.01</v>
+      </c>
+      <c r="H4">
+        <v>80</v>
+      </c>
+      <c r="I4">
+        <v>15</v>
+      </c>
+      <c r="J4" s="8">
+        <v>0.01</v>
+      </c>
+      <c r="K4" s="8">
+        <v>2</v>
+      </c>
+      <c r="L4" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="M4">
+        <v>0</v>
+      </c>
+      <c r="N4">
+        <v>0</v>
+      </c>
+      <c r="O4">
+        <v>0</v>
+      </c>
+      <c r="P4">
+        <v>0</v>
+      </c>
+      <c r="Q4" t="s">
+        <v>214</v>
+      </c>
+      <c r="R4" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>207</v>
+      </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+        <v>Ghost</v>
+      </c>
+      <c r="C5" t="s">
+        <v>209</v>
+      </c>
+      <c r="D5" t="s">
+        <v>169</v>
+      </c>
+      <c r="E5">
+        <v>10</v>
+      </c>
+      <c r="F5">
+        <v>8</v>
+      </c>
+      <c r="G5" s="8">
+        <v>0</v>
+      </c>
+      <c r="H5">
+        <v>110</v>
+      </c>
+      <c r="I5">
+        <v>5</v>
+      </c>
+      <c r="J5" s="8">
+        <v>0.01</v>
+      </c>
+      <c r="K5" s="8">
+        <v>2</v>
+      </c>
+      <c r="L5" s="8">
+        <v>0.1</v>
+      </c>
+      <c r="M5">
+        <v>0</v>
+      </c>
+      <c r="N5">
+        <v>0</v>
+      </c>
+      <c r="O5">
+        <v>0</v>
+      </c>
+      <c r="P5">
+        <v>3</v>
+      </c>
+      <c r="Q5" t="s">
+        <v>215</v>
+      </c>
+      <c r="R5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="14" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="15" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B15" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
     </row>
-    <row r="16" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
       <c r="B16" t="str">
         <f t="shared" si="0"/>
         <v/>
@@ -1297,12 +1704,523 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H44" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:R44" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DFC42C69-7304-40C7-BA02-8A3EB2712138}">
+          <x14:formula1>
+            <xm:f>motion!$A$2:$A$30</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2:D50</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A706FF91-8AAE-4DE1-83AD-81AADC56FAFB}">
+  <sheetPr>
+    <tabColor theme="7" tint="0.59999389629810485"/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="3" max="3" width="49.85546875" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" customWidth="1"/>
+    <col min="6" max="6" width="12.85546875" customWidth="1"/>
+    <col min="7" max="7" width="15.7109375" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="G1" s="3" t="s">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>144</v>
+      </c>
+      <c r="B2" t="str">
+        <f>PROPER(A2)</f>
+        <v>Coal</v>
+      </c>
+      <c r="C2" t="s">
+        <v>125</v>
+      </c>
+      <c r="D2" t="s">
+        <v>126</v>
+      </c>
+      <c r="E2">
+        <v>1</v>
+      </c>
+      <c r="F2">
+        <v>2</v>
+      </c>
+      <c r="G2">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>145</v>
+      </c>
+      <c r="B3" t="str">
+        <f t="shared" ref="B3:B13" si="0">PROPER(A3)</f>
+        <v>Fury</v>
+      </c>
+      <c r="C3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D3" t="s">
+        <v>126</v>
+      </c>
+      <c r="E3" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="F3" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="G3" s="6">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>146</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>Blast</v>
+      </c>
+      <c r="C4" t="s">
+        <v>128</v>
+      </c>
+      <c r="D4" t="s">
+        <v>126</v>
+      </c>
+      <c r="E4" s="6">
+        <v>0.05</v>
+      </c>
+      <c r="F4" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="G4" s="6">
+        <v>0.15</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>147</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>Rime</v>
+      </c>
+      <c r="C5" t="s">
+        <v>129</v>
+      </c>
+      <c r="D5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E5">
+        <v>1</v>
+      </c>
+      <c r="F5">
+        <v>2</v>
+      </c>
+      <c r="G5">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>148</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>Soft</v>
+      </c>
+      <c r="C6" t="s">
+        <v>131</v>
+      </c>
+      <c r="D6" t="s">
+        <v>130</v>
+      </c>
+      <c r="E6" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="F6" s="6">
+        <v>0.4</v>
+      </c>
+      <c r="G6" s="6">
+        <v>0.6</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>149</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>Bounty</v>
+      </c>
+      <c r="C7" t="s">
+        <v>132</v>
+      </c>
+      <c r="D7" t="s">
+        <v>130</v>
+      </c>
+      <c r="E7">
+        <v>1</v>
+      </c>
+      <c r="F7">
+        <v>2</v>
+      </c>
+      <c r="G7">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>150</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>Static</v>
+      </c>
+      <c r="C8" t="s">
+        <v>133</v>
+      </c>
+      <c r="D8" t="s">
+        <v>134</v>
+      </c>
+      <c r="E8">
+        <v>1</v>
+      </c>
+      <c r="F8">
+        <v>2</v>
+      </c>
+      <c r="G8">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>156</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>Shear</v>
+      </c>
+      <c r="C9" t="s">
+        <v>135</v>
+      </c>
+      <c r="D9" t="s">
+        <v>134</v>
+      </c>
+      <c r="E9" s="6">
+        <v>0.01</v>
+      </c>
+      <c r="F9" s="6">
+        <v>0.02</v>
+      </c>
+      <c r="G9" s="6">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>151</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>Drag</v>
+      </c>
+      <c r="C10" t="s">
+        <v>136</v>
+      </c>
+      <c r="D10" t="s">
+        <v>134</v>
+      </c>
+      <c r="E10" s="6">
+        <v>0.1</v>
+      </c>
+      <c r="F10" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="G10" s="6">
+        <v>0.3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>152</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>Blight</v>
+      </c>
+      <c r="C11" t="s">
+        <v>137</v>
+      </c>
+      <c r="D11" t="s">
+        <v>138</v>
+      </c>
+      <c r="E11">
+        <v>1</v>
+      </c>
+      <c r="F11">
+        <v>2</v>
+      </c>
+      <c r="G11">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>153</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>Dense</v>
+      </c>
+      <c r="C12" t="s">
+        <v>139</v>
+      </c>
+      <c r="D12" t="s">
+        <v>138</v>
+      </c>
+      <c r="E12" s="6">
+        <v>0.2</v>
+      </c>
+      <c r="F12" s="6">
+        <v>0.3</v>
+      </c>
+      <c r="G12" s="6">
+        <v>0.4</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>154</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>Crush</v>
+      </c>
+      <c r="C13" t="s">
+        <v>140</v>
+      </c>
+      <c r="D13" t="s">
+        <v>138</v>
+      </c>
+      <c r="E13" s="6">
+        <v>0.01</v>
+      </c>
+      <c r="F13" s="6">
+        <v>0.02</v>
+      </c>
+      <c r="G13" s="6">
+        <v>0.03</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3C10F13-8E40-4AB2-9849-0A8DFD3352A1}">
+  <sheetPr>
+    <tabColor theme="4" tint="0.59999389629810485"/>
+  </sheetPr>
+  <dimension ref="A1:C18"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="46.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A1" s="3" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>169</v>
+      </c>
+      <c r="B2" t="str">
+        <f t="shared" ref="B2" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
+        <v>Wayward</v>
+      </c>
+      <c r="C2" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>172</v>
+      </c>
+      <c r="C3" t="s">
+        <v>173</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>174</v>
+      </c>
+      <c r="C4" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>176</v>
+      </c>
+      <c r="C5" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>179</v>
+      </c>
+      <c r="C6" t="s">
+        <v>178</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>180</v>
+      </c>
+      <c r="C7" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>182</v>
+      </c>
+      <c r="C8" t="s">
+        <v>183</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>184</v>
+      </c>
+      <c r="C9" t="s">
+        <v>185</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>186</v>
+      </c>
+      <c r="C10" t="s">
+        <v>187</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>188</v>
+      </c>
+      <c r="C11" t="s">
+        <v>189</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>190</v>
+      </c>
+      <c r="C12" t="s">
+        <v>191</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>192</v>
+      </c>
+      <c r="C13" t="s">
+        <v>193</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>194</v>
+      </c>
+      <c r="C14" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>195</v>
+      </c>
+      <c r="C15" t="s">
+        <v>196</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>198</v>
+      </c>
+      <c r="C16" t="s">
+        <v>199</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>200</v>
+      </c>
+      <c r="C17" t="s">
+        <v>201</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>202</v>
+      </c>
+      <c r="C18" t="s">
+        <v>203</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="8" tint="0.59999389629810485"/>
@@ -1340,139 +2258,139 @@
         <v>3</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>110</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>111</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>112</v>
+      </c>
+      <c r="I1" s="4" t="s">
+        <v>113</v>
+      </c>
+      <c r="J1" s="4" t="s">
+        <v>62</v>
+      </c>
+      <c r="K1" s="4" t="s">
+        <v>114</v>
+      </c>
+      <c r="L1" s="4" t="s">
+        <v>5</v>
+      </c>
+      <c r="M1" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="F1" s="4" t="s">
-        <v>123</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>124</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>125</v>
-      </c>
-      <c r="I1" s="4" t="s">
-        <v>126</v>
-      </c>
-      <c r="J1" s="4" t="s">
-        <v>64</v>
-      </c>
-      <c r="K1" s="4" t="s">
-        <v>127</v>
-      </c>
-      <c r="L1" s="4" t="s">
+      <c r="N1" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="M1" s="4" t="s">
+      <c r="O1" s="3" t="s">
         <v>8</v>
       </c>
-      <c r="N1" s="4" t="s">
+      <c r="P1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="O1" s="3" t="s">
+      <c r="Q1" s="3" t="s">
         <v>10</v>
       </c>
-      <c r="P1" s="3" t="s">
+      <c r="R1" s="3" t="s">
         <v>11</v>
       </c>
-      <c r="Q1" s="3" t="s">
+      <c r="S1" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="R1" s="3" t="s">
+      <c r="T1" s="4" t="s">
         <v>13</v>
       </c>
-      <c r="S1" s="4" t="s">
+      <c r="U1" s="3" t="s">
         <v>14</v>
-      </c>
-      <c r="T1" s="4" t="s">
-        <v>15</v>
-      </c>
-      <c r="U1" s="3" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B33" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Reception Desk</v>
       </c>
       <c r="C2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D2" t="s">
+        <v>17</v>
+      </c>
+      <c r="F2" s="2">
+        <v>0</v>
+      </c>
+      <c r="G2" s="2">
+        <v>0</v>
+      </c>
+      <c r="H2" s="2">
+        <v>0</v>
+      </c>
+      <c r="I2" s="2">
+        <v>0</v>
+      </c>
+      <c r="J2" s="2">
+        <v>0</v>
+      </c>
+      <c r="K2" s="2">
+        <v>0</v>
+      </c>
+      <c r="L2" t="s">
         <v>18</v>
-      </c>
-      <c r="D2" t="s">
-        <v>19</v>
-      </c>
-      <c r="F2" s="2">
-        <v>0</v>
-      </c>
-      <c r="G2" s="2">
-        <v>0</v>
-      </c>
-      <c r="H2" s="2">
-        <v>0</v>
-      </c>
-      <c r="I2" s="2">
-        <v>0</v>
-      </c>
-      <c r="J2" s="2">
-        <v>0</v>
-      </c>
-      <c r="K2" s="2">
-        <v>0</v>
-      </c>
-      <c r="L2" t="s">
-        <v>20</v>
       </c>
       <c r="O2">
         <v>2</v>
       </c>
       <c r="T2" t="s">
+        <v>19</v>
+      </c>
+      <c r="U2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A3" s="7" t="s">
+        <v>20</v>
+      </c>
+      <c r="B3" t="str">
+        <f t="shared" si="0"/>
+        <v>Straw Pallet</v>
+      </c>
+      <c r="C3" t="s">
         <v>21</v>
       </c>
-      <c r="U2" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="3" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A3" s="8" t="s">
+      <c r="D3" t="s">
         <v>22</v>
       </c>
-      <c r="B3" t="str">
-        <f t="shared" si="0"/>
-        <v>Straw Pallet</v>
-      </c>
-      <c r="C3" t="s">
+      <c r="F3" s="2">
+        <v>1</v>
+      </c>
+      <c r="G3" s="2">
+        <v>0</v>
+      </c>
+      <c r="H3" s="2">
+        <v>1</v>
+      </c>
+      <c r="I3" s="2">
+        <v>0</v>
+      </c>
+      <c r="J3" s="2">
+        <v>0</v>
+      </c>
+      <c r="K3" s="2">
+        <v>0</v>
+      </c>
+      <c r="L3" t="s">
+        <v>18</v>
+      </c>
+      <c r="M3" t="s">
         <v>23</v>
-      </c>
-      <c r="D3" t="s">
-        <v>24</v>
-      </c>
-      <c r="F3" s="2">
-        <v>1</v>
-      </c>
-      <c r="G3" s="2">
-        <v>0</v>
-      </c>
-      <c r="H3" s="2">
-        <v>1</v>
-      </c>
-      <c r="I3" s="2">
-        <v>0</v>
-      </c>
-      <c r="J3" s="2">
-        <v>0</v>
-      </c>
-      <c r="K3" s="2">
-        <v>0</v>
-      </c>
-      <c r="L3" t="s">
-        <v>20</v>
-      </c>
-      <c r="M3" t="s">
-        <v>25</v>
       </c>
       <c r="O3">
         <v>2</v>
@@ -1486,17 +2404,17 @@
     </row>
     <row r="4" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Wood Frame Bed</v>
       </c>
       <c r="C4" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D4" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F4" s="2">
         <v>0</v>
@@ -1517,10 +2435,10 @@
         <v>0</v>
       </c>
       <c r="L4" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M4" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O4">
         <v>2</v>
@@ -1529,10 +2447,10 @@
         <v>0</v>
       </c>
       <c r="S4" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
       <c r="T4" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="U4" t="b">
         <v>1</v>
@@ -1540,17 +2458,17 @@
     </row>
     <row r="5" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Bunk Bed</v>
       </c>
       <c r="C5" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D5" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F5" s="2">
         <v>0</v>
@@ -1571,10 +2489,10 @@
         <v>0</v>
       </c>
       <c r="L5" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M5" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O5">
         <v>2</v>
@@ -1583,28 +2501,28 @@
         <v>1</v>
       </c>
       <c r="S5" t="s">
+        <v>30</v>
+      </c>
+      <c r="T5" t="s">
+        <v>31</v>
+      </c>
+      <c r="U5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A6" s="7" t="s">
         <v>32</v>
       </c>
-      <c r="T5" t="s">
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>Canopy Bed</v>
+      </c>
+      <c r="C6" t="s">
         <v>33</v>
       </c>
-      <c r="U5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A6" s="8" t="s">
-        <v>34</v>
-      </c>
-      <c r="B6" t="str">
-        <f t="shared" si="0"/>
-        <v>Canopy Bed</v>
-      </c>
-      <c r="C6" t="s">
-        <v>35</v>
-      </c>
       <c r="D6" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
       <c r="F6" s="2">
         <v>0</v>
@@ -1625,10 +2543,10 @@
         <v>0</v>
       </c>
       <c r="L6" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M6" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O6">
         <v>2</v>
@@ -1642,17 +2560,17 @@
     </row>
     <row r="7" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>34</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>Budget Wardrobe</v>
+      </c>
+      <c r="C7" t="s">
+        <v>35</v>
+      </c>
+      <c r="D7" t="s">
         <v>36</v>
-      </c>
-      <c r="B7" t="str">
-        <f t="shared" si="0"/>
-        <v>Budget Wardrobe</v>
-      </c>
-      <c r="C7" t="s">
-        <v>37</v>
-      </c>
-      <c r="D7" t="s">
-        <v>38</v>
       </c>
       <c r="F7" s="2">
         <v>0</v>
@@ -1673,10 +2591,10 @@
         <v>2</v>
       </c>
       <c r="L7" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M7" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O7">
         <v>3</v>
@@ -1685,10 +2603,10 @@
         <v>0</v>
       </c>
       <c r="S7" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="T7" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="U7" t="b">
         <v>1</v>
@@ -1696,17 +2614,17 @@
     </row>
     <row r="8" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>Fine Wardrobe</v>
       </c>
       <c r="C8" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D8" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="F8" s="2">
         <v>0</v>
@@ -1727,10 +2645,10 @@
         <v>4</v>
       </c>
       <c r="L8" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M8" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O8">
         <v>3</v>
@@ -1739,10 +2657,10 @@
         <v>0</v>
       </c>
       <c r="S8" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="T8" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="U8" t="b">
         <v>1</v>
@@ -1750,17 +2668,17 @@
     </row>
     <row r="9" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>Ornate Wardrobe</v>
       </c>
       <c r="D9" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="E9" t="s">
-        <v>128</v>
+        <v>115</v>
       </c>
       <c r="F9" s="2">
         <v>0</v>
@@ -1781,10 +2699,10 @@
         <v>7</v>
       </c>
       <c r="L9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M9" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O9">
         <v>3</v>
@@ -1793,67 +2711,67 @@
         <v>0</v>
       </c>
       <c r="S9" t="s">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="T9" t="s">
+        <v>43</v>
+      </c>
+      <c r="U9" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A10" s="7" t="s">
+        <v>44</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>Night Stand</v>
+      </c>
+      <c r="F10" s="2">
+        <v>0</v>
+      </c>
+      <c r="G10" s="2">
+        <v>0</v>
+      </c>
+      <c r="H10" s="2">
+        <v>0</v>
+      </c>
+      <c r="I10" s="2">
+        <v>0</v>
+      </c>
+      <c r="J10" s="2">
+        <v>0</v>
+      </c>
+      <c r="K10" s="2">
+        <v>0</v>
+      </c>
+      <c r="L10" t="s">
+        <v>18</v>
+      </c>
+      <c r="M10" t="s">
+        <v>23</v>
+      </c>
+      <c r="O10">
+        <v>1</v>
+      </c>
+      <c r="R10" t="b">
+        <v>0</v>
+      </c>
+      <c r="U10" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A11" s="7" t="s">
         <v>45</v>
       </c>
-      <c r="U9" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="10" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A10" s="8" t="s">
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>Wash Basin</v>
+      </c>
+      <c r="E11" t="s">
         <v>46</v>
-      </c>
-      <c r="B10" t="str">
-        <f t="shared" si="0"/>
-        <v>Night Stand</v>
-      </c>
-      <c r="F10" s="2">
-        <v>0</v>
-      </c>
-      <c r="G10" s="2">
-        <v>0</v>
-      </c>
-      <c r="H10" s="2">
-        <v>0</v>
-      </c>
-      <c r="I10" s="2">
-        <v>0</v>
-      </c>
-      <c r="J10" s="2">
-        <v>0</v>
-      </c>
-      <c r="K10" s="2">
-        <v>0</v>
-      </c>
-      <c r="L10" t="s">
-        <v>20</v>
-      </c>
-      <c r="M10" t="s">
-        <v>25</v>
-      </c>
-      <c r="O10">
-        <v>1</v>
-      </c>
-      <c r="R10" t="b">
-        <v>0</v>
-      </c>
-      <c r="U10" t="b">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="11" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A11" s="8" t="s">
-        <v>47</v>
-      </c>
-      <c r="B11" t="str">
-        <f t="shared" si="0"/>
-        <v>Wash Basin</v>
-      </c>
-      <c r="E11" t="s">
-        <v>48</v>
       </c>
       <c r="F11" s="2">
         <v>0</v>
@@ -1874,10 +2792,10 @@
         <v>0</v>
       </c>
       <c r="L11" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M11" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O11">
         <v>1</v>
@@ -1890,15 +2808,15 @@
       </c>
     </row>
     <row r="12" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A12" s="8" t="s">
-        <v>49</v>
+      <c r="A12" s="7" t="s">
+        <v>47</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Artisan Rug</v>
       </c>
       <c r="E12" t="s">
-        <v>50</v>
+        <v>48</v>
       </c>
       <c r="F12" s="2">
         <v>0</v>
@@ -1919,7 +2837,7 @@
         <v>4</v>
       </c>
       <c r="L12" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="O12">
         <v>2</v>
@@ -1932,15 +2850,15 @@
       </c>
     </row>
     <row r="13" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A13" s="8" t="s">
-        <v>51</v>
+      <c r="A13" s="7" t="s">
+        <v>49</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>Mirror</v>
       </c>
       <c r="E13" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F13" s="2">
         <v>0</v>
@@ -1961,10 +2879,10 @@
         <v>3</v>
       </c>
       <c r="L13" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M13" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O13">
         <v>1</v>
@@ -1977,15 +2895,15 @@
       </c>
     </row>
     <row r="14" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A14" s="8" t="s">
-        <v>53</v>
+      <c r="A14" s="7" t="s">
+        <v>51</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v>Trunk</v>
       </c>
       <c r="C14" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="F14" s="2">
         <v>0</v>
@@ -2006,10 +2924,10 @@
         <v>1</v>
       </c>
       <c r="L14" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M14" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O14">
         <v>2</v>
@@ -2022,8 +2940,8 @@
       </c>
     </row>
     <row r="15" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A15" s="8" t="s">
-        <v>55</v>
+      <c r="A15" s="7" t="s">
+        <v>53</v>
       </c>
       <c r="B15" t="str">
         <f t="shared" si="0"/>
@@ -2048,7 +2966,7 @@
         <v>0</v>
       </c>
       <c r="L15" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="O15">
         <v>3</v>
@@ -2061,8 +2979,8 @@
       </c>
     </row>
     <row r="16" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A16" s="8" t="s">
-        <v>56</v>
+      <c r="A16" s="7" t="s">
+        <v>54</v>
       </c>
       <c r="B16" t="str">
         <f t="shared" si="0"/>
@@ -2087,10 +3005,10 @@
         <v>0</v>
       </c>
       <c r="L16" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M16" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="O16">
         <v>1</v>
@@ -2104,14 +3022,14 @@
     </row>
     <row r="17" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v>Small Houseplant</v>
       </c>
       <c r="D17" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="F17" s="2">
         <v>0</v>
@@ -2132,7 +3050,7 @@
         <v>4</v>
       </c>
       <c r="L17" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="O17">
         <v>1</v>
@@ -2141,25 +3059,25 @@
         <v>0</v>
       </c>
       <c r="S17" t="s">
+        <v>57</v>
+      </c>
+      <c r="T17" t="s">
+        <v>58</v>
+      </c>
+      <c r="U17" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A18" s="7" t="s">
         <v>59</v>
       </c>
-      <c r="T17" t="s">
-        <v>60</v>
-      </c>
-      <c r="U17" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="18" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A18" s="8" t="s">
-        <v>61</v>
-      </c>
       <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v>Big Houseplant</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>129</v>
+        <v>116</v>
       </c>
       <c r="F18" s="2">
         <v>0</v>
@@ -2180,7 +3098,7 @@
         <v>6</v>
       </c>
       <c r="L18" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="O18">
         <v>2</v>
@@ -2193,15 +3111,15 @@
       </c>
     </row>
     <row r="19" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A19" s="8" t="s">
-        <v>62</v>
+      <c r="A19" s="7" t="s">
+        <v>60</v>
       </c>
       <c r="B19" t="str">
         <f t="shared" si="0"/>
         <v>Chamber Pot</v>
       </c>
       <c r="C19" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="F19" s="2">
         <v>0</v>
@@ -2222,10 +3140,10 @@
         <v>0</v>
       </c>
       <c r="L19" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M19" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="O19">
         <v>1</v>
@@ -2239,41 +3157,41 @@
     </row>
     <row r="20" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
+        <v>63</v>
+      </c>
+      <c r="B20" t="str">
+        <f t="shared" si="0"/>
+        <v>Cooking Order Desk</v>
+      </c>
+      <c r="C20" t="s">
+        <v>64</v>
+      </c>
+      <c r="D20" t="s">
         <v>65</v>
       </c>
-      <c r="B20" t="str">
-        <f t="shared" si="0"/>
-        <v>Cooking Order Desk</v>
-      </c>
-      <c r="C20" t="s">
+      <c r="F20" s="2">
+        <v>0</v>
+      </c>
+      <c r="G20" s="2">
+        <v>0</v>
+      </c>
+      <c r="H20" s="2">
+        <v>0</v>
+      </c>
+      <c r="I20" s="2">
+        <v>0</v>
+      </c>
+      <c r="J20" s="2">
+        <v>0</v>
+      </c>
+      <c r="K20" s="2">
+        <v>0</v>
+      </c>
+      <c r="L20" t="s">
+        <v>18</v>
+      </c>
+      <c r="M20" t="s">
         <v>66</v>
-      </c>
-      <c r="D20" t="s">
-        <v>67</v>
-      </c>
-      <c r="F20" s="2">
-        <v>0</v>
-      </c>
-      <c r="G20" s="2">
-        <v>0</v>
-      </c>
-      <c r="H20" s="2">
-        <v>0</v>
-      </c>
-      <c r="I20" s="2">
-        <v>0</v>
-      </c>
-      <c r="J20" s="2">
-        <v>0</v>
-      </c>
-      <c r="K20" s="2">
-        <v>0</v>
-      </c>
-      <c r="L20" t="s">
-        <v>20</v>
-      </c>
-      <c r="M20" t="s">
-        <v>68</v>
       </c>
       <c r="O20">
         <v>2</v>
@@ -2282,10 +3200,10 @@
         <v>0</v>
       </c>
       <c r="S20" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="T20" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="U20" t="b">
         <v>1</v>
@@ -2293,41 +3211,41 @@
     </row>
     <row r="21" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
+        <v>69</v>
+      </c>
+      <c r="B21" t="str">
+        <f t="shared" si="0"/>
+        <v>Cooking Couldron</v>
+      </c>
+      <c r="C21" t="s">
+        <v>70</v>
+      </c>
+      <c r="D21" t="s">
         <v>71</v>
       </c>
-      <c r="B21" t="str">
-        <f t="shared" si="0"/>
-        <v>Cooking Couldron</v>
-      </c>
-      <c r="C21" t="s">
+      <c r="F21" s="2">
+        <v>0</v>
+      </c>
+      <c r="G21" s="2">
+        <v>0</v>
+      </c>
+      <c r="H21" s="2">
+        <v>0</v>
+      </c>
+      <c r="I21" s="2">
+        <v>0</v>
+      </c>
+      <c r="J21" s="2">
+        <v>0</v>
+      </c>
+      <c r="K21" s="2">
+        <v>0</v>
+      </c>
+      <c r="L21" t="s">
+        <v>18</v>
+      </c>
+      <c r="M21" t="s">
         <v>72</v>
-      </c>
-      <c r="D21" t="s">
-        <v>73</v>
-      </c>
-      <c r="F21" s="2">
-        <v>0</v>
-      </c>
-      <c r="G21" s="2">
-        <v>0</v>
-      </c>
-      <c r="H21" s="2">
-        <v>0</v>
-      </c>
-      <c r="I21" s="2">
-        <v>0</v>
-      </c>
-      <c r="J21" s="2">
-        <v>0</v>
-      </c>
-      <c r="K21" s="2">
-        <v>0</v>
-      </c>
-      <c r="L21" t="s">
-        <v>20</v>
-      </c>
-      <c r="M21" t="s">
-        <v>74</v>
       </c>
       <c r="O21">
         <v>2</v>
@@ -2336,10 +3254,10 @@
         <v>0</v>
       </c>
       <c r="S21" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="T21" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="U21" t="b">
         <v>1</v>
@@ -2347,14 +3265,14 @@
     </row>
     <row r="22" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>77</v>
+        <v>75</v>
       </c>
       <c r="B22" t="str">
         <f t="shared" si="0"/>
         <v>Small Seating Table</v>
       </c>
       <c r="D22" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="F22" s="2">
         <v>0</v>
@@ -2375,10 +3293,10 @@
         <v>0</v>
       </c>
       <c r="L22" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M22" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="O22">
         <v>2</v>
@@ -2387,10 +3305,10 @@
         <v>0</v>
       </c>
       <c r="S22" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="T22" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
       <c r="U22" t="b">
         <v>1</v>
@@ -2398,18 +3316,18 @@
     </row>
     <row r="23" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
+        <v>79</v>
+      </c>
+      <c r="B23" t="str">
+        <f t="shared" si="0"/>
+        <v>Pass Table</v>
+      </c>
+      <c r="C23" t="s">
+        <v>80</v>
+      </c>
+      <c r="D23" t="s">
         <v>81</v>
       </c>
-      <c r="B23" t="str">
-        <f t="shared" si="0"/>
-        <v>Pass Table</v>
-      </c>
-      <c r="C23" t="s">
-        <v>82</v>
-      </c>
-      <c r="D23" t="s">
-        <v>83</v>
-      </c>
       <c r="F23" s="2">
         <v>0</v>
       </c>
@@ -2429,10 +3347,10 @@
         <v>1</v>
       </c>
       <c r="L23" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M23" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="O23">
         <v>2</v>
@@ -2441,10 +3359,10 @@
         <v>0</v>
       </c>
       <c r="S23" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="T23" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="U23" t="b">
         <v>1</v>
@@ -2452,18 +3370,18 @@
     </row>
     <row r="24" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
+        <v>84</v>
+      </c>
+      <c r="B24" t="str">
+        <f t="shared" si="0"/>
+        <v>Crate</v>
+      </c>
+      <c r="C24" t="s">
+        <v>85</v>
+      </c>
+      <c r="D24" t="s">
         <v>86</v>
       </c>
-      <c r="B24" t="str">
-        <f t="shared" si="0"/>
-        <v>Crate</v>
-      </c>
-      <c r="C24" t="s">
-        <v>87</v>
-      </c>
-      <c r="D24" t="s">
-        <v>88</v>
-      </c>
       <c r="F24" s="2">
         <v>0</v>
       </c>
@@ -2483,7 +3401,7 @@
         <v>0</v>
       </c>
       <c r="L24" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="O24">
         <v>2</v>
@@ -2492,28 +3410,28 @@
         <v>0</v>
       </c>
       <c r="S24" t="s">
+        <v>87</v>
+      </c>
+      <c r="T24" t="s">
+        <v>88</v>
+      </c>
+      <c r="U24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
+      <c r="A25" s="7" t="s">
         <v>89</v>
       </c>
-      <c r="T24" t="s">
-        <v>90</v>
-      </c>
-      <c r="U24" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:21" x14ac:dyDescent="0.25">
-      <c r="A25" s="8" t="s">
-        <v>91</v>
-      </c>
       <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v>Barrel</v>
       </c>
       <c r="C25" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="D25" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="F25" s="2">
         <v>0</v>
@@ -2534,7 +3452,7 @@
         <v>0</v>
       </c>
       <c r="L25" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="O25">
         <v>2</v>
@@ -2543,10 +3461,10 @@
         <v>0</v>
       </c>
       <c r="S25" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="T25" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="U25" t="b">
         <v>1</v>
@@ -2554,38 +3472,38 @@
     </row>
     <row r="26" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
+        <v>92</v>
+      </c>
+      <c r="B26" t="str">
+        <f t="shared" si="0"/>
+        <v>Wall Torch</v>
+      </c>
+      <c r="C26" t="s">
+        <v>93</v>
+      </c>
+      <c r="D26" t="s">
         <v>94</v>
       </c>
-      <c r="B26" t="str">
-        <f t="shared" si="0"/>
-        <v>Wall Torch</v>
-      </c>
-      <c r="C26" t="s">
+      <c r="F26" s="2">
+        <v>0</v>
+      </c>
+      <c r="G26" s="2">
+        <v>0</v>
+      </c>
+      <c r="H26" s="2">
+        <v>0</v>
+      </c>
+      <c r="I26" s="2">
+        <v>0</v>
+      </c>
+      <c r="J26" s="2">
+        <v>0</v>
+      </c>
+      <c r="K26" s="2">
+        <v>0</v>
+      </c>
+      <c r="L26" t="s">
         <v>95</v>
-      </c>
-      <c r="D26" t="s">
-        <v>96</v>
-      </c>
-      <c r="F26" s="2">
-        <v>0</v>
-      </c>
-      <c r="G26" s="2">
-        <v>0</v>
-      </c>
-      <c r="H26" s="2">
-        <v>0</v>
-      </c>
-      <c r="I26" s="2">
-        <v>0</v>
-      </c>
-      <c r="J26" s="2">
-        <v>0</v>
-      </c>
-      <c r="K26" s="2">
-        <v>0</v>
-      </c>
-      <c r="L26" t="s">
-        <v>97</v>
       </c>
       <c r="O26">
         <v>0</v>
@@ -2597,10 +3515,10 @@
         <v>0</v>
       </c>
       <c r="S26" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="T26" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="U26" t="b">
         <v>1</v>
@@ -2608,17 +3526,17 @@
     </row>
     <row r="27" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
+        <v>98</v>
+      </c>
+      <c r="B27" t="str">
+        <f t="shared" si="0"/>
+        <v>Condiment Shelf</v>
+      </c>
+      <c r="C27" t="s">
+        <v>99</v>
+      </c>
+      <c r="D27" t="s">
         <v>100</v>
-      </c>
-      <c r="B27" t="str">
-        <f t="shared" si="0"/>
-        <v>Condiment Shelf</v>
-      </c>
-      <c r="C27" t="s">
-        <v>101</v>
-      </c>
-      <c r="D27" t="s">
-        <v>102</v>
       </c>
       <c r="F27" s="2">
         <v>0</v>
@@ -2639,10 +3557,10 @@
         <v>2</v>
       </c>
       <c r="L27" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="M27" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="O27">
         <v>1</v>
@@ -2654,10 +3572,10 @@
         <v>0</v>
       </c>
       <c r="S27" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="T27" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="U27" t="b">
         <v>1</v>
@@ -2665,17 +3583,17 @@
     </row>
     <row r="28" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="B28" t="str">
         <f t="shared" si="0"/>
         <v>Condiment Shelf Small</v>
       </c>
       <c r="C28" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D28" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F28" s="2">
         <v>0</v>
@@ -2696,10 +3614,10 @@
         <v>1</v>
       </c>
       <c r="L28" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="M28" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="O28">
         <v>1</v>
@@ -2711,10 +3629,10 @@
         <v>0</v>
       </c>
       <c r="S28" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="T28" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="U28" t="b">
         <v>1</v>
@@ -2722,17 +3640,17 @@
     </row>
     <row r="29" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="B29" t="str">
         <f t="shared" si="0"/>
         <v>Hanging Frying Pans</v>
       </c>
       <c r="C29" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="D29" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="F29" s="2">
         <v>0</v>
@@ -2753,10 +3671,10 @@
         <v>0</v>
       </c>
       <c r="L29" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="M29" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="O29">
         <v>0</v>
@@ -2767,14 +3685,14 @@
     </row>
     <row r="30" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="B30" t="str">
         <f t="shared" si="0"/>
         <v>Butcher Table</v>
       </c>
       <c r="D30" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="F30" s="2">
         <v>0</v>
@@ -2795,10 +3713,10 @@
         <v>3</v>
       </c>
       <c r="L30" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="M30" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="O30">
         <v>2</v>
@@ -2809,14 +3727,14 @@
     </row>
     <row r="31" spans="1:21" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="B31" t="str">
         <f t="shared" si="0"/>
         <v>Hanging Meat</v>
       </c>
       <c r="D31" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
     </row>
     <row r="32" spans="1:21" x14ac:dyDescent="0.25">
@@ -2986,7 +3904,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
@@ -2996,16 +3914,16 @@
   <sheetData>
     <row r="2" spans="1:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
-        <v>167</v>
+        <v>123</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>7</v>
+        <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
       <c r="D2" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
     </row>
   </sheetData>
@@ -3013,872 +3931,337 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:C76"/>
+  <dimension ref="A1:C29"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.7109375" customWidth="1"/>
-    <col min="2" max="2" width="27.5703125" customWidth="1"/>
+    <col min="1" max="2" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
-        <v>153</v>
+        <v>117</v>
       </c>
       <c r="B1" t="s">
-        <v>154</v>
+        <v>118</v>
       </c>
       <c r="C1" t="s">
         <v>3</v>
       </c>
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
+      <c r="A2" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B2" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="C2" s="11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A3" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B3" s="11" t="s">
+        <v>1</v>
+      </c>
+      <c r="C3" s="11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A4" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A5" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B5" s="11" t="s">
+        <v>170</v>
+      </c>
+      <c r="C5" s="11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A6" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B6" s="11" t="s">
+        <v>157</v>
+      </c>
+      <c r="C6" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A7" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B7" s="11" t="s">
+        <v>158</v>
+      </c>
+      <c r="C7" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A8" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" s="11" t="s">
+        <v>159</v>
+      </c>
+      <c r="C8" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A9" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B9" s="11" t="s">
+        <v>160</v>
+      </c>
+      <c r="C9" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A10" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B10" s="11" t="s">
+        <v>161</v>
+      </c>
+      <c r="C10" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A11" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B11" s="11" t="s">
+        <v>162</v>
+      </c>
+      <c r="C11" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A12" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B12" s="11" t="s">
+        <v>163</v>
+      </c>
+      <c r="C12" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A13" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B13" s="11" t="s">
+        <v>164</v>
+      </c>
+      <c r="C13" s="11" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A14" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B14" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="C14" s="11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A15" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B15" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="C15" s="11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A16" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B16" s="11" t="s">
+        <v>167</v>
+      </c>
+      <c r="C16" s="11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B17" s="11" t="s">
+        <v>168</v>
+      </c>
+      <c r="C17" s="11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B18" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="C18" s="11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B19" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="C20" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="B21" s="12" t="s">
+        <v>1</v>
+      </c>
+      <c r="C21" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="B22" s="12" t="s">
+        <v>2</v>
+      </c>
+      <c r="C22" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="B23" s="12" t="s">
         <v>155</v>
       </c>
-      <c r="B2" t="s">
-        <v>0</v>
-      </c>
-      <c r="C2" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>155</v>
-      </c>
-      <c r="B3" t="s">
-        <v>1</v>
-      </c>
-      <c r="C3" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>155</v>
-      </c>
-      <c r="B4" t="s">
+      <c r="C23" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="B24" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="C24" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="B25" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="C25" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="12" t="s">
+        <v>211</v>
+      </c>
+      <c r="B26" s="12" t="s">
+        <v>143</v>
+      </c>
+      <c r="C26" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="B27" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C27" s="14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="B28" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C28" s="14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="14" t="s">
+        <v>170</v>
+      </c>
+      <c r="B29" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C4" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>155</v>
-      </c>
-      <c r="B5" t="s">
-        <v>111</v>
-      </c>
-      <c r="C5" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
-        <v>155</v>
-      </c>
-      <c r="B6" t="s">
-        <v>112</v>
-      </c>
-      <c r="C6" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
-        <v>155</v>
-      </c>
-      <c r="B7" t="s">
-        <v>113</v>
-      </c>
-      <c r="C7" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
-        <v>155</v>
-      </c>
-      <c r="B8" t="s">
-        <v>114</v>
-      </c>
-      <c r="C8" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>155</v>
-      </c>
-      <c r="B9" t="s">
-        <v>115</v>
-      </c>
-      <c r="C9" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>155</v>
-      </c>
-      <c r="B10" t="s">
-        <v>116</v>
-      </c>
-      <c r="C10" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>155</v>
-      </c>
-      <c r="B11" t="s">
-        <v>117</v>
-      </c>
-      <c r="C11" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>155</v>
-      </c>
-      <c r="B12" t="s">
-        <v>118</v>
-      </c>
-      <c r="C12" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B13" t="s">
+      <c r="C29" s="14" t="s">
         <v>119</v>
       </c>
-      <c r="C13" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
-        <v>155</v>
-      </c>
-      <c r="B14" t="s">
-        <v>120</v>
-      </c>
-      <c r="C14" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
-        <v>155</v>
-      </c>
-      <c r="B15" t="s">
-        <v>121</v>
-      </c>
-      <c r="C15" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
-        <v>155</v>
-      </c>
-      <c r="B16" t="s">
-        <v>16</v>
-      </c>
-      <c r="C16" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
-        <v>152</v>
-      </c>
-      <c r="B17" t="s">
-        <v>0</v>
-      </c>
-      <c r="C17" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
-        <v>152</v>
-      </c>
-      <c r="B18" t="s">
-        <v>1</v>
-      </c>
-      <c r="C18" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
-        <v>152</v>
-      </c>
-      <c r="B19" t="s">
-        <v>2</v>
-      </c>
-      <c r="C19" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
-        <v>152</v>
-      </c>
-      <c r="B20" t="s">
-        <v>3</v>
-      </c>
-      <c r="C20" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
-        <v>152</v>
-      </c>
-      <c r="B21" t="s">
-        <v>4</v>
-      </c>
-      <c r="C21" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
-        <v>152</v>
-      </c>
-      <c r="B22" t="s">
-        <v>5</v>
-      </c>
-      <c r="C22" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
-        <v>152</v>
-      </c>
-      <c r="B23" t="s">
-        <v>6</v>
-      </c>
-      <c r="C23" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
-        <v>152</v>
-      </c>
-      <c r="B24" t="s">
-        <v>7</v>
-      </c>
-      <c r="C24" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A25" t="s">
-        <v>152</v>
-      </c>
-      <c r="B25" t="s">
-        <v>8</v>
-      </c>
-      <c r="C25" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A26" t="s">
-        <v>152</v>
-      </c>
-      <c r="B26" t="s">
-        <v>9</v>
-      </c>
-      <c r="C26" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" t="s">
-        <v>152</v>
-      </c>
-      <c r="B27" t="s">
-        <v>10</v>
-      </c>
-      <c r="C27" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" t="s">
-        <v>152</v>
-      </c>
-      <c r="B28" t="s">
-        <v>11</v>
-      </c>
-      <c r="C28" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" t="s">
-        <v>152</v>
-      </c>
-      <c r="B29" t="s">
-        <v>12</v>
-      </c>
-      <c r="C29" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" t="s">
-        <v>152</v>
-      </c>
-      <c r="B30" t="s">
-        <v>13</v>
-      </c>
-      <c r="C30" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" t="s">
-        <v>152</v>
-      </c>
-      <c r="B31" t="s">
-        <v>14</v>
-      </c>
-      <c r="C31" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A32" t="s">
-        <v>152</v>
-      </c>
-      <c r="B32" t="s">
-        <v>15</v>
-      </c>
-      <c r="C32" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A33" t="s">
-        <v>152</v>
-      </c>
-      <c r="B33" t="s">
-        <v>16</v>
-      </c>
-      <c r="C33" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A34" t="s">
-        <v>160</v>
-      </c>
-      <c r="B34" t="s">
-        <v>0</v>
-      </c>
-      <c r="C34" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A35" t="s">
-        <v>160</v>
-      </c>
-      <c r="B35" t="s">
-        <v>1</v>
-      </c>
-      <c r="C35" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A36" t="s">
-        <v>160</v>
-      </c>
-      <c r="B36" t="s">
-        <v>2</v>
-      </c>
-      <c r="C36" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A37" t="s">
-        <v>160</v>
-      </c>
-      <c r="B37" t="s">
-        <v>130</v>
-      </c>
-      <c r="C37" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A38" t="s">
-        <v>160</v>
-      </c>
-      <c r="B38" t="s">
-        <v>131</v>
-      </c>
-      <c r="C38" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" t="s">
-        <v>160</v>
-      </c>
-      <c r="B39" t="s">
-        <v>132</v>
-      </c>
-      <c r="C39" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A40" t="s">
-        <v>160</v>
-      </c>
-      <c r="B40" t="s">
-        <v>133</v>
-      </c>
-      <c r="C40" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A41" t="s">
-        <v>160</v>
-      </c>
-      <c r="B41" t="s">
-        <v>134</v>
-      </c>
-      <c r="C41" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A42" t="s">
-        <v>160</v>
-      </c>
-      <c r="B42" t="s">
-        <v>135</v>
-      </c>
-      <c r="C42" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A43" t="s">
-        <v>160</v>
-      </c>
-      <c r="B43" t="s">
-        <v>136</v>
-      </c>
-      <c r="C43" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A44" t="s">
-        <v>162</v>
-      </c>
-      <c r="B44" t="s">
-        <v>0</v>
-      </c>
-      <c r="C44" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A45" t="s">
-        <v>162</v>
-      </c>
-      <c r="B45" t="s">
-        <v>1</v>
-      </c>
-      <c r="C45" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A46" t="s">
-        <v>162</v>
-      </c>
-      <c r="B46" t="s">
-        <v>2</v>
-      </c>
-      <c r="C46" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A47" t="s">
-        <v>162</v>
-      </c>
-      <c r="B47" t="s">
-        <v>6</v>
-      </c>
-      <c r="C47" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A48" t="s">
-        <v>162</v>
-      </c>
-      <c r="B48" t="s">
-        <v>137</v>
-      </c>
-      <c r="C48" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A49" t="s">
-        <v>162</v>
-      </c>
-      <c r="B49" t="s">
-        <v>15</v>
-      </c>
-      <c r="C49" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A50" t="s">
-        <v>163</v>
-      </c>
-      <c r="B50" t="s">
-        <v>0</v>
-      </c>
-      <c r="C50" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A51" t="s">
-        <v>163</v>
-      </c>
-      <c r="B51" t="s">
-        <v>1</v>
-      </c>
-      <c r="C51" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A52" t="s">
-        <v>163</v>
-      </c>
-      <c r="B52" t="s">
-        <v>2</v>
-      </c>
-      <c r="C52" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A53" t="s">
-        <v>164</v>
-      </c>
-      <c r="B53" t="s">
-        <v>0</v>
-      </c>
-      <c r="C53" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A54" t="s">
-        <v>164</v>
-      </c>
-      <c r="B54" t="s">
-        <v>1</v>
-      </c>
-      <c r="C54" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A55" t="s">
-        <v>164</v>
-      </c>
-      <c r="B55" t="s">
-        <v>2</v>
-      </c>
-      <c r="C55" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A56" t="s">
-        <v>165</v>
-      </c>
-      <c r="B56" t="s">
-        <v>0</v>
-      </c>
-      <c r="C56" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A57" t="s">
-        <v>165</v>
-      </c>
-      <c r="B57" t="s">
-        <v>1</v>
-      </c>
-      <c r="C57" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A58" t="s">
-        <v>165</v>
-      </c>
-      <c r="B58" t="s">
-        <v>138</v>
-      </c>
-      <c r="C58" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A59" t="s">
-        <v>165</v>
-      </c>
-      <c r="B59" t="s">
-        <v>139</v>
-      </c>
-      <c r="C59" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A60" t="s">
-        <v>165</v>
-      </c>
-      <c r="B60" t="s">
-        <v>2</v>
-      </c>
-      <c r="C60" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A61" t="s">
-        <v>165</v>
-      </c>
-      <c r="B61" t="s">
-        <v>140</v>
-      </c>
-      <c r="C61" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A62" t="s">
-        <v>165</v>
-      </c>
-      <c r="B62" t="s">
-        <v>141</v>
-      </c>
-      <c r="C62" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A63" t="s">
-        <v>165</v>
-      </c>
-      <c r="B63" t="s">
-        <v>142</v>
-      </c>
-      <c r="C63" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A64" t="s">
-        <v>165</v>
-      </c>
-      <c r="B64" t="s">
-        <v>143</v>
-      </c>
-      <c r="C64" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" t="s">
-        <v>165</v>
-      </c>
-      <c r="B65" t="s">
-        <v>144</v>
-      </c>
-      <c r="C65" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A66" t="s">
-        <v>165</v>
-      </c>
-      <c r="B66" t="s">
-        <v>16</v>
-      </c>
-      <c r="C66" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A67" t="s">
-        <v>166</v>
-      </c>
-      <c r="B67" t="s">
-        <v>0</v>
-      </c>
-      <c r="C67" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A68" t="s">
-        <v>166</v>
-      </c>
-      <c r="B68" t="s">
-        <v>1</v>
-      </c>
-      <c r="C68" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A69" t="s">
-        <v>166</v>
-      </c>
-      <c r="B69" t="s">
-        <v>145</v>
-      </c>
-      <c r="C69" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A70" t="s">
-        <v>166</v>
-      </c>
-      <c r="B70" t="s">
-        <v>146</v>
-      </c>
-      <c r="C70" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A71" t="s">
-        <v>166</v>
-      </c>
-      <c r="B71" t="s">
-        <v>147</v>
-      </c>
-      <c r="C71" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A72" t="s">
-        <v>166</v>
-      </c>
-      <c r="B72" t="s">
-        <v>148</v>
-      </c>
-      <c r="C72" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A73" t="s">
-        <v>166</v>
-      </c>
-      <c r="B73" t="s">
-        <v>149</v>
-      </c>
-      <c r="C73" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A74" t="s">
-        <v>166</v>
-      </c>
-      <c r="B74" t="s">
-        <v>150</v>
-      </c>
-      <c r="C74" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A75" t="s">
-        <v>166</v>
-      </c>
-      <c r="B75" t="s">
-        <v>151</v>
-      </c>
-      <c r="C75" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A76" t="s">
-        <v>166</v>
-      </c>
-      <c r="B76" t="s">
-        <v>16</v>
-      </c>
-      <c r="C76" t="s">
-        <v>159</v>
-      </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="B16">
-    <cfRule type="containsText" dxfId="4" priority="1" operator="containsText" text="aether">
-      <formula>NOT(ISERROR(SEARCH("aether",B16)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="3" priority="2" operator="containsText" text="breach">
-      <formula>NOT(ISERROR(SEARCH("breach",B16)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="2" priority="3" operator="containsText" text="bio">
-      <formula>NOT(ISERROR(SEARCH("bio",B16)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="1" priority="4" operator="containsText" text="industry">
-      <formula>NOT(ISERROR(SEARCH("industry",B16)))</formula>
-    </cfRule>
-    <cfRule type="containsText" dxfId="0" priority="5" operator="containsText" text="bastion">
-      <formula>NOT(ISERROR(SEARCH("bastion",B16)))</formula>
-    </cfRule>
-  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Implement Excel to JSON game data pipeline and update project structure
- Introduced a new system for managing game data by exporting from an Excel workbook (`game_data.xlsx`) to a JSON format (`game_data.json`), allowing for easier content authoring and integration.
- Added a `GameData` autoload script to facilitate generic data lookups for orbs, glyphs, and motion, enhancing the flexibility of data management.
- Updated project structure to reflect the new data organization, including the addition of export scripts and documentation for the new pipeline.
- Revised `DECISIONS.md` and `PROJECT_MAP.md` to document the new data management approach and its implications for future content integration.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\One Last Bullet\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4B59C5EA-C6FF-4C4E-AD42-1A985500D97F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D7BEB2E-7BB9-4C5F-8AC8-3DDCD3F0E501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -824,42 +824,7 @@
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="4" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="7" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor theme="9" tint="0.59996337778862885"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FFFA8A8A"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill>
-          <bgColor rgb="FF918CEC"/>
-        </patternFill>
-      </fill>
-    </dxf>
+  <dxfs count="1">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -1403,7 +1368,7 @@
         <v>0</v>
       </c>
       <c r="P4">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="Q4" t="s">
         <v>214</v>
@@ -1460,7 +1425,7 @@
         <v>0</v>
       </c>
       <c r="P5">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="Q5" t="s">
         <v>215</v>
@@ -3884,7 +3849,7 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="F2:K104">
-    <cfRule type="cellIs" dxfId="5" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>0</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>

<commit_message>
Enhance orb mechanics and status effects for improved gameplay dynamics
- Updated orb mechanics to include new core stats and status effects, allowing orbs to apply damage and effects such as Poison, Shock, Burn, and Chill based on GameData.
- Revised `DECISIONS.md` to document the new orb stats and their interactions, ensuring clarity on gameplay mechanics and strategic implications.
- Enhanced `GAME_BRIEF.md` to reflect the updated orb behaviors and their impact on player strategy.
- Adjusted `PROJECT_MAP.md` to include new components and their roles in the game, improving project organization and clarity.
- Implemented changes in `level.gd` to manage the new orb behaviors and ensure consistent gameplay experience.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\One Last Bullet\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D7BEB2E-7BB9-4C5F-8AC8-3DDCD3F0E501}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6625C04-3EB8-47AA-A0C0-8EF213B78D4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-28800" yWindow="240" windowWidth="28800" windowHeight="15345" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -1233,7 +1233,7 @@
         <v>100</v>
       </c>
       <c r="I2">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J2" s="8">
         <v>0.01</v>
@@ -1278,7 +1278,7 @@
         <v>169</v>
       </c>
       <c r="E3">
-        <v>15</v>
+        <v>10</v>
       </c>
       <c r="F3">
         <v>12</v>
@@ -1290,7 +1290,7 @@
         <v>130</v>
       </c>
       <c r="I3">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="J3" s="8">
         <v>0.01</v>
@@ -1335,7 +1335,7 @@
         <v>169</v>
       </c>
       <c r="E4">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="F4">
         <v>18</v>
@@ -1347,7 +1347,7 @@
         <v>80</v>
       </c>
       <c r="I4">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="J4" s="8">
         <v>0.01</v>
@@ -1404,7 +1404,7 @@
         <v>110</v>
       </c>
       <c r="I5">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="J5" s="8">
         <v>0.01</v>

</xml_diff>

<commit_message>
Implement glyph mechanics and update inventory system for enhanced gameplay
- Introduced glyphs as a replacement for mana crystals, allowing enemies to drop glyphs with varying rarities and attributes, enhancing strategic gameplay.
- Updated the summoning circle mechanics to include a ritual menu for orb customization, separating mana delivery from orb upgrades.
- Revised `GAME_BRIEF.md` to reflect the new glyph mechanics and their impact on player strategy.
- Adjusted `PROJECT_MAP.md` to include new glyph components and their roles in the game, improving project organization.
- Modified `level.gd` to manage glyph spawning and integrate with the new inventory system, ensuring a cohesive gameplay experience.
- Updated relevant components to support the new item handling and interactions, enhancing overall game dynamics.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\One Last Bullet\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D6625C04-3EB8-47AA-A0C0-8EF213B78D4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BB5C189-4D38-4857-BCD1-73C15634FD1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28800" yWindow="240" windowWidth="28800" windowHeight="15345" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7125" yWindow="4230" windowWidth="28800" windowHeight="15345" tabRatio="696" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -42,7 +42,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="381" uniqueCount="216">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="217">
   <si>
     <t>id</t>
   </si>
@@ -440,9 +440,6 @@
     <t>This orb deals less damage to players</t>
   </si>
   <si>
-    <t>Mana drop chance from enemies</t>
-  </si>
-  <si>
     <t>Shock on enemy hit</t>
   </si>
   <si>
@@ -536,9 +533,6 @@
     <t>crit_damage</t>
   </si>
   <si>
-    <t>crystal_drop</t>
-  </si>
-  <si>
     <t>burn</t>
   </si>
   <si>
@@ -690,6 +684,15 @@
   </si>
   <si>
     <t>res://entities/orbs/ghost/ghost_orb.tscn</t>
+  </si>
+  <si>
+    <t>attribute</t>
+  </si>
+  <si>
+    <t>glyph_drop</t>
+  </si>
+  <si>
+    <t>Glyph drop chance from enemies</t>
   </si>
 </sst>
 </file>
@@ -1161,43 +1164,43 @@
         <v>2</v>
       </c>
       <c r="D1" s="10" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E1" s="9" t="s">
+        <v>156</v>
+      </c>
+      <c r="F1" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="G1" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="H1" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="I1" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="9" t="s">
+        <v>215</v>
+      </c>
+      <c r="M1" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="L1" s="9" t="s">
+      <c r="N1" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="M1" s="9" t="s">
+      <c r="O1" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="P1" s="9" t="s">
         <v>166</v>
-      </c>
-      <c r="O1" s="9" t="s">
-        <v>167</v>
-      </c>
-      <c r="P1" s="9" t="s">
-        <v>168</v>
       </c>
       <c r="Q1" s="13" t="s">
         <v>109</v>
@@ -1208,7 +1211,7 @@
     </row>
     <row r="2" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B26" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
@@ -1218,7 +1221,7 @@
         <v>124</v>
       </c>
       <c r="D2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E2">
         <v>10</v>
@@ -1257,7 +1260,7 @@
         <v>0</v>
       </c>
       <c r="Q2" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="R2" t="b">
         <v>1</v>
@@ -1265,17 +1268,17 @@
     </row>
     <row r="3" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Conduit</v>
       </c>
       <c r="C3" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E3">
         <v>10</v>
@@ -1314,7 +1317,7 @@
         <v>0</v>
       </c>
       <c r="Q3" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="R3" t="b">
         <v>1</v>
@@ -1322,17 +1325,17 @@
     </row>
     <row r="4" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Rot</v>
       </c>
       <c r="C4" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E4">
         <v>5</v>
@@ -1371,7 +1374,7 @@
         <v>3</v>
       </c>
       <c r="Q4" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="R4" t="b">
         <v>1</v>
@@ -1379,17 +1382,17 @@
     </row>
     <row r="5" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>205</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>Ghost</v>
+      </c>
+      <c r="C5" t="s">
         <v>207</v>
       </c>
-      <c r="B5" t="str">
-        <f t="shared" si="0"/>
-        <v>Ghost</v>
-      </c>
-      <c r="C5" t="s">
-        <v>209</v>
-      </c>
       <c r="D5" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E5">
         <v>10</v>
@@ -1428,7 +1431,7 @@
         <v>0</v>
       </c>
       <c r="Q5" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="R5" t="b">
         <v>1</v>
@@ -1691,16 +1694,17 @@
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:G13"/>
+  <dimension ref="A1:H13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="49.85546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="16.85546875" customWidth="1"/>
-    <col min="6" max="6" width="12.85546875" customWidth="1"/>
-    <col min="7" max="7" width="15.7109375" customWidth="1"/>
+    <col min="5" max="5" width="13.5703125" customWidth="1"/>
+    <col min="6" max="6" width="16.85546875" customWidth="1"/>
+    <col min="7" max="7" width="12.85546875" customWidth="1"/>
+    <col min="8" max="8" width="15.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
@@ -1711,21 +1715,24 @@
         <v>2</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E1" s="3" t="s">
+        <v>214</v>
+      </c>
+      <c r="F1" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="G1" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="F1" s="3" t="s">
+      <c r="H1" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="G1" s="3" t="s">
+    </row>
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
         <v>143</v>
-      </c>
-    </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A2" t="s">
-        <v>144</v>
       </c>
       <c r="B2" t="str">
         <f>PROPER(A2)</f>
@@ -1737,19 +1744,22 @@
       <c r="D2" t="s">
         <v>126</v>
       </c>
-      <c r="E2">
-        <v>1</v>
+      <c r="E2" t="s">
+        <v>163</v>
       </c>
       <c r="F2">
+        <v>1</v>
+      </c>
+      <c r="G2">
         <v>2</v>
       </c>
-      <c r="G2">
+      <c r="H2">
         <v>3</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" ref="B3:B13" si="0">PROPER(A3)</f>
@@ -1761,19 +1771,22 @@
       <c r="D3" t="s">
         <v>126</v>
       </c>
-      <c r="E3" s="6">
-        <v>0.1</v>
-      </c>
-      <c r="F3" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="G3" s="6">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E3" t="s">
+        <v>156</v>
+      </c>
+      <c r="F3">
+        <v>5</v>
+      </c>
+      <c r="G3">
+        <v>10</v>
+      </c>
+      <c r="H3">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
@@ -1785,19 +1798,22 @@
       <c r="D4" t="s">
         <v>126</v>
       </c>
-      <c r="E4" s="6">
+      <c r="E4" t="s">
+        <v>158</v>
+      </c>
+      <c r="F4" s="6">
         <v>0.05</v>
       </c>
-      <c r="F4" s="6">
+      <c r="G4" s="6">
         <v>0.1</v>
       </c>
-      <c r="G4" s="6">
+      <c r="H4" s="6">
         <v>0.15</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
@@ -1809,19 +1825,22 @@
       <c r="D5" t="s">
         <v>130</v>
       </c>
-      <c r="E5">
-        <v>1</v>
+      <c r="E5" t="s">
+        <v>164</v>
       </c>
       <c r="F5">
+        <v>1</v>
+      </c>
+      <c r="G5">
         <v>2</v>
       </c>
-      <c r="G5">
+      <c r="H5">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
@@ -1833,181 +1852,205 @@
       <c r="D6" t="s">
         <v>130</v>
       </c>
-      <c r="E6" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="F6" s="6">
-        <v>0.4</v>
-      </c>
-      <c r="G6" s="6">
-        <v>0.6</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="E6" t="s">
+        <v>157</v>
+      </c>
+      <c r="F6">
+        <v>-10</v>
+      </c>
+      <c r="G6">
+        <v>-20</v>
+      </c>
+      <c r="H6">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Bounty</v>
       </c>
       <c r="C7" t="s">
-        <v>132</v>
+        <v>216</v>
       </c>
       <c r="D7" t="s">
         <v>130</v>
       </c>
-      <c r="E7">
-        <v>1</v>
-      </c>
-      <c r="F7">
+      <c r="E7" t="s">
+        <v>215</v>
+      </c>
+      <c r="F7" s="8">
+        <v>0.01</v>
+      </c>
+      <c r="G7" s="8">
+        <v>0.02</v>
+      </c>
+      <c r="H7" s="8">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>149</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>Static</v>
+      </c>
+      <c r="C8" t="s">
+        <v>132</v>
+      </c>
+      <c r="D8" t="s">
+        <v>133</v>
+      </c>
+      <c r="E8" t="s">
+        <v>165</v>
+      </c>
+      <c r="F8">
+        <v>1</v>
+      </c>
+      <c r="G8">
         <v>2</v>
       </c>
-      <c r="G7">
+      <c r="H8">
         <v>3</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>155</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>Shear</v>
+      </c>
+      <c r="C9" t="s">
+        <v>134</v>
+      </c>
+      <c r="D9" t="s">
+        <v>133</v>
+      </c>
+      <c r="E9" t="s">
+        <v>161</v>
+      </c>
+      <c r="F9" s="6">
+        <v>0.01</v>
+      </c>
+      <c r="G9" s="6">
+        <v>0.02</v>
+      </c>
+      <c r="H9" s="6">
+        <v>0.03</v>
+      </c>
+    </row>
+    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
         <v>150</v>
       </c>
-      <c r="B8" t="str">
-        <f t="shared" si="0"/>
-        <v>Static</v>
-      </c>
-      <c r="C8" t="s">
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>Drag</v>
+      </c>
+      <c r="C10" t="s">
+        <v>135</v>
+      </c>
+      <c r="D10" t="s">
         <v>133</v>
       </c>
-      <c r="D8" t="s">
-        <v>134</v>
-      </c>
-      <c r="E8">
-        <v>1</v>
-      </c>
-      <c r="F8">
+      <c r="E10" t="s">
+        <v>159</v>
+      </c>
+      <c r="F10">
+        <v>-10</v>
+      </c>
+      <c r="G10">
+        <v>-20</v>
+      </c>
+      <c r="H10">
+        <v>-30</v>
+      </c>
+    </row>
+    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>151</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>Blight</v>
+      </c>
+      <c r="C11" t="s">
+        <v>136</v>
+      </c>
+      <c r="D11" t="s">
+        <v>137</v>
+      </c>
+      <c r="E11" t="s">
+        <v>166</v>
+      </c>
+      <c r="F11">
+        <v>1</v>
+      </c>
+      <c r="G11">
         <v>2</v>
       </c>
-      <c r="G8">
+      <c r="H11">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
-        <v>156</v>
-      </c>
-      <c r="B9" t="str">
-        <f t="shared" si="0"/>
-        <v>Shear</v>
-      </c>
-      <c r="C9" t="s">
-        <v>135</v>
-      </c>
-      <c r="D9" t="s">
-        <v>134</v>
-      </c>
-      <c r="E9" s="6">
+    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>152</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>Dense</v>
+      </c>
+      <c r="C12" t="s">
+        <v>138</v>
+      </c>
+      <c r="D12" t="s">
+        <v>137</v>
+      </c>
+      <c r="E12" t="s">
+        <v>160</v>
+      </c>
+      <c r="F12">
+        <v>1</v>
+      </c>
+      <c r="G12">
+        <v>2</v>
+      </c>
+      <c r="H12">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>153</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>Crush</v>
+      </c>
+      <c r="C13" t="s">
+        <v>139</v>
+      </c>
+      <c r="D13" t="s">
+        <v>137</v>
+      </c>
+      <c r="E13" t="s">
+        <v>162</v>
+      </c>
+      <c r="F13" s="6">
         <v>0.01</v>
       </c>
-      <c r="F9" s="6">
+      <c r="G13" s="6">
         <v>0.02</v>
       </c>
-      <c r="G9" s="6">
-        <v>0.03</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
-        <v>151</v>
-      </c>
-      <c r="B10" t="str">
-        <f t="shared" si="0"/>
-        <v>Drag</v>
-      </c>
-      <c r="C10" t="s">
-        <v>136</v>
-      </c>
-      <c r="D10" t="s">
-        <v>134</v>
-      </c>
-      <c r="E10" s="6">
-        <v>0.1</v>
-      </c>
-      <c r="F10" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="G10" s="6">
-        <v>0.3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
-        <v>152</v>
-      </c>
-      <c r="B11" t="str">
-        <f t="shared" si="0"/>
-        <v>Blight</v>
-      </c>
-      <c r="C11" t="s">
-        <v>137</v>
-      </c>
-      <c r="D11" t="s">
-        <v>138</v>
-      </c>
-      <c r="E11">
-        <v>1</v>
-      </c>
-      <c r="F11">
-        <v>2</v>
-      </c>
-      <c r="G11">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
-        <v>153</v>
-      </c>
-      <c r="B12" t="str">
-        <f t="shared" si="0"/>
-        <v>Dense</v>
-      </c>
-      <c r="C12" t="s">
-        <v>139</v>
-      </c>
-      <c r="D12" t="s">
-        <v>138</v>
-      </c>
-      <c r="E12" s="6">
-        <v>0.2</v>
-      </c>
-      <c r="F12" s="6">
-        <v>0.3</v>
-      </c>
-      <c r="G12" s="6">
-        <v>0.4</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
-        <v>154</v>
-      </c>
-      <c r="B13" t="str">
-        <f t="shared" si="0"/>
-        <v>Crush</v>
-      </c>
-      <c r="C13" t="s">
-        <v>140</v>
-      </c>
-      <c r="D13" t="s">
-        <v>138</v>
-      </c>
-      <c r="E13" s="6">
-        <v>0.01</v>
-      </c>
-      <c r="F13" s="6">
-        <v>0.02</v>
-      </c>
-      <c r="G13" s="6">
+      <c r="H13" s="6">
         <v>0.03</v>
       </c>
     </row>
@@ -2042,142 +2085,142 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Wayward</v>
       </c>
       <c r="C2" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="C3" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="C4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="C5" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="C6" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="C7" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="C8" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="C9" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="C10" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="C11" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="C12" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="C13" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="C14" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="C15" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="C16" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="C17" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="C18" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -3901,7 +3944,7 @@
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C30"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="14.7109375" customWidth="1"/>
@@ -3956,7 +3999,7 @@
         <v>123</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>119</v>
@@ -3967,7 +4010,7 @@
         <v>123</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>122</v>
@@ -3978,7 +4021,7 @@
         <v>123</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>122</v>
@@ -3989,7 +4032,7 @@
         <v>123</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>122</v>
@@ -4000,7 +4043,7 @@
         <v>123</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>122</v>
@@ -4011,7 +4054,7 @@
         <v>123</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>122</v>
@@ -4022,7 +4065,7 @@
         <v>123</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>122</v>
@@ -4033,7 +4076,7 @@
         <v>123</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>122</v>
@@ -4044,7 +4087,7 @@
         <v>123</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>164</v>
+        <v>215</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>122</v>
@@ -4055,7 +4098,7 @@
         <v>123</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>165</v>
+        <v>163</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>120</v>
@@ -4066,7 +4109,7 @@
         <v>123</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>120</v>
@@ -4077,7 +4120,7 @@
         <v>123</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>120</v>
@@ -4088,7 +4131,7 @@
         <v>123</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>120</v>
@@ -4118,7 +4161,7 @@
     </row>
     <row r="20" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A20" s="12" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B20" s="12" t="s">
         <v>0</v>
@@ -4129,7 +4172,7 @@
     </row>
     <row r="21" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A21" s="12" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B21" s="12" t="s">
         <v>1</v>
@@ -4140,7 +4183,7 @@
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A22" s="12" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B22" s="12" t="s">
         <v>2</v>
@@ -4151,10 +4194,10 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>119</v>
@@ -4162,21 +4205,21 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>141</v>
+        <v>214</v>
       </c>
       <c r="C24" s="12" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="C25" s="12" t="s">
         <v>122</v>
@@ -4184,32 +4227,32 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="C26" s="12" t="s">
         <v>122</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A27" s="14" t="s">
-        <v>170</v>
-      </c>
-      <c r="B27" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="C27" s="14" t="s">
-        <v>119</v>
+      <c r="A27" s="12" t="s">
+        <v>209</v>
+      </c>
+      <c r="B27" s="12" t="s">
+        <v>142</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>122</v>
       </c>
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="14" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B28" s="14" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C28" s="14" t="s">
         <v>119</v>
@@ -4217,12 +4260,23 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="14" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B29" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C29" s="14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="14" t="s">
+        <v>168</v>
+      </c>
+      <c r="B30" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C29" s="14" t="s">
+      <c r="C30" s="14" t="s">
         <v>119</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update ritual menu and orb mechanics for improved gameplay experience
- Revised `desert.tscn` to update the ritual menu resource reference, ensuring consistency in scene management.
- Enhanced `orb_tether_component.gd` to improve connection handling and clarify owner exit logic.
- Adjusted `game_data.json` to modify rarity and self-damage values for orbs, balancing gameplay dynamics.
- Refactored `blank_orb.gd` to incorporate new capture mechanics and streamline physics interactions.
- Updated `ritual_menu.gd` to enhance stat display and formatting, improving user interface clarity.
- Made structural changes to `ritual_menu.tscn` for better organization and layout consistency.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\One Last Bullet\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5BB5C189-4D38-4857-BCD1-73C15634FD1A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E966BF6-55EF-4B8C-95B8-116087FE6D6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7125" yWindow="4230" windowWidth="28800" windowHeight="15345" tabRatio="696" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7125" yWindow="4230" windowWidth="28800" windowHeight="15345" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -1227,7 +1227,7 @@
         <v>10</v>
       </c>
       <c r="F2">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G2" s="8">
         <v>0</v>
@@ -1245,7 +1245,7 @@
         <v>2</v>
       </c>
       <c r="L2" s="8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M2">
         <v>0</v>
@@ -1284,7 +1284,7 @@
         <v>10</v>
       </c>
       <c r="F3">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="G3" s="8">
         <v>0</v>
@@ -1302,7 +1302,7 @@
         <v>2</v>
       </c>
       <c r="L3" s="8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M3">
         <v>0</v>
@@ -1341,7 +1341,7 @@
         <v>5</v>
       </c>
       <c r="F4">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="G4" s="8">
         <v>0.01</v>
@@ -1359,7 +1359,7 @@
         <v>2</v>
       </c>
       <c r="L4" s="8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M4">
         <v>0</v>
@@ -1398,7 +1398,7 @@
         <v>10</v>
       </c>
       <c r="F5">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G5" s="8">
         <v>0</v>
@@ -1416,7 +1416,7 @@
         <v>2</v>
       </c>
       <c r="L5" s="8">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="M5">
         <v>0</v>
@@ -2045,13 +2045,13 @@
         <v>162</v>
       </c>
       <c r="F13" s="6">
-        <v>0.01</v>
+        <v>0.1</v>
       </c>
       <c r="G13" s="6">
-        <v>0.02</v>
+        <v>0.2</v>
       </c>
       <c r="H13" s="6">
-        <v>0.03</v>
+        <v>0.3</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Enhance desert level and ritual menu for improved gameplay dynamics
- Added new enemy resources in `desert.tscn` to diversify enemy encounters and enhance gameplay variety.
- Updated `level.gd` to include a placeholder for a new orb scene, improving future orb integration.
- Expanded `game_data.json` with new attunements for orbs, enriching gameplay mechanics and strategic options.
- Refined `ritual_menu.gd` to center the panel dynamically, enhancing user interface experience.
- Made structural adjustments in `ritual_menu.tscn` for better organization and layout consistency.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,21 +8,22 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\One Last Bullet\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E966BF6-55EF-4B8C-95B8-116087FE6D6E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2511F6C2-22E4-4F9C-BBC2-CF77A815396F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="7125" yWindow="4230" windowWidth="28800" windowHeight="15345" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
     <sheet name="glyphs" sheetId="15" r:id="rId2"/>
-    <sheet name="motion" sheetId="16" r:id="rId3"/>
-    <sheet name="objects_OLD" sheetId="3" state="hidden" r:id="rId4"/>
-    <sheet name="input" sheetId="13" r:id="rId5"/>
-    <sheet name="schema" sheetId="14" r:id="rId6"/>
+    <sheet name="attunements" sheetId="17" r:id="rId3"/>
+    <sheet name="motion" sheetId="16" r:id="rId4"/>
+    <sheet name="objects_OLD" sheetId="3" state="hidden" r:id="rId5"/>
+    <sheet name="input" sheetId="13" r:id="rId6"/>
+    <sheet name="schema" sheetId="14" r:id="rId7"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">objects_OLD!$A$1:$U$53</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">orbs!$A$1:$R$44</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">objects_OLD!$A$1:$U$53</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">orbs!$A$1:$W$44</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -42,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="397" uniqueCount="217">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="236">
   <si>
     <t>id</t>
   </si>
@@ -554,9 +555,6 @@
     <t>Straight flight, bounce off solids</t>
   </si>
   <si>
-    <t>hungry</t>
-  </si>
-  <si>
     <t>Steer toward nearest enemy</t>
   </si>
   <si>
@@ -665,9 +663,6 @@
     <t>When you are within 120 meters of the orb, create a tether between you dealing 3 DPS to enemies touching it</t>
   </si>
   <si>
-    <t>Enters enemies and deal its impact damage per second to them. Once dead, exits in a random direction</t>
-  </si>
-  <si>
     <t>Inflict poison on hit</t>
   </si>
   <si>
@@ -693,6 +688,69 @@
   </si>
   <si>
     <t>Glyph drop chance from enemies</t>
+  </si>
+  <si>
+    <t>elements</t>
+  </si>
+  <si>
+    <t>element_1</t>
+  </si>
+  <si>
+    <t>element_2</t>
+  </si>
+  <si>
+    <t>element_3</t>
+  </si>
+  <si>
+    <t>unique?</t>
+  </si>
+  <si>
+    <t>haunt</t>
+  </si>
+  <si>
+    <t>orb_id</t>
+  </si>
+  <si>
+    <t>attunements</t>
+  </si>
+  <si>
+    <t>Enters and haunts enemies and deal its impact damage per second to them. Once dead, exits in a random direction</t>
+  </si>
+  <si>
+    <t>possesion</t>
+  </si>
+  <si>
+    <t>attracted</t>
+  </si>
+  <si>
+    <t>Changes Motion to Attracted</t>
+  </si>
+  <si>
+    <t>Makes haunted enemy attack other enemies</t>
+  </si>
+  <si>
+    <t>inferno</t>
+  </si>
+  <si>
+    <t>Leaves a trail of fire after the orb for 2 seconds, inflicting 1 Burn on enemies</t>
+  </si>
+  <si>
+    <t>trail</t>
+  </si>
+  <si>
+    <t>Fire trail lasts 4 seconds</t>
+  </si>
+  <si>
+    <t>kindling</t>
+  </si>
+  <si>
+    <t>Dashing through a fire trail extends it</t>
+  </si>
+  <si>
+    <t>When colliding with another orb, a fire trail is made</t>
+  </si>
+  <si>
+    <t>spark</t>
   </si>
 </sst>
 </file>
@@ -804,7 +862,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -822,12 +880,14 @@
     <xf numFmtId="0" fontId="0" fillId="5" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="1">
+  <dxfs count="13">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -849,10 +909,96 @@
         </bottom>
       </border>
     </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF7C80"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCA8914"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF7C80"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCA8914"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="3" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFFF7C80"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor theme="4" tint="0.59996337778862885"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill>
+          <bgColor rgb="FFCA8914"/>
+        </patternFill>
+      </fill>
+    </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
     <mruColors>
+      <color rgb="FFCA8914"/>
+      <color rgb="FFFF7C80"/>
       <color rgb="FF00FFCC"/>
     </mruColors>
   </colors>
@@ -1133,27 +1279,32 @@
   <sheetPr>
     <tabColor theme="9" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:R44"/>
+  <dimension ref="A1:W98"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="19.42578125" customWidth="1"/>
     <col min="2" max="2" width="17.5703125" customWidth="1"/>
     <col min="3" max="3" width="104.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15" customWidth="1"/>
-    <col min="5" max="5" width="10.42578125" customWidth="1"/>
-    <col min="6" max="6" width="15.42578125" customWidth="1"/>
-    <col min="7" max="7" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="8.5703125" customWidth="1"/>
-    <col min="9" max="9" width="9.140625" customWidth="1"/>
-    <col min="10" max="12" width="14.5703125" customWidth="1"/>
-    <col min="13" max="13" width="8.85546875" customWidth="1"/>
-    <col min="14" max="14" width="8.42578125" customWidth="1"/>
-    <col min="15" max="15" width="8.5703125" customWidth="1"/>
-    <col min="16" max="16" width="8.7109375" customWidth="1"/>
-    <col min="17" max="17" width="47" customWidth="1"/>
+    <col min="4" max="4" width="16.7109375" customWidth="1"/>
+    <col min="5" max="5" width="10.5703125" customWidth="1"/>
+    <col min="6" max="6" width="13.42578125" customWidth="1"/>
+    <col min="7" max="7" width="20" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="20" customWidth="1"/>
+    <col min="9" max="9" width="15" customWidth="1"/>
+    <col min="10" max="10" width="10.42578125" customWidth="1"/>
+    <col min="11" max="11" width="15.42578125" customWidth="1"/>
+    <col min="12" max="12" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="8.5703125" customWidth="1"/>
+    <col min="14" max="14" width="9.140625" customWidth="1"/>
+    <col min="15" max="17" width="14.5703125" customWidth="1"/>
+    <col min="18" max="18" width="8.85546875" customWidth="1"/>
+    <col min="19" max="19" width="8.42578125" customWidth="1"/>
+    <col min="20" max="20" width="8.5703125" customWidth="1"/>
+    <col min="21" max="21" width="8.7109375" customWidth="1"/>
+    <col min="22" max="22" width="47" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -1163,55 +1314,67 @@
       <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="10" t="s">
+      <c r="D1" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="H1" s="4" t="s">
+        <v>219</v>
+      </c>
+      <c r="I1" s="10" t="s">
         <v>168</v>
       </c>
-      <c r="E1" s="9" t="s">
+      <c r="J1" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="F1" s="9" t="s">
+      <c r="K1" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="G1" s="9" t="s">
+      <c r="L1" s="9" t="s">
         <v>158</v>
       </c>
-      <c r="H1" s="9" t="s">
+      <c r="M1" s="9" t="s">
         <v>159</v>
       </c>
-      <c r="I1" s="9" t="s">
+      <c r="N1" s="9" t="s">
         <v>160</v>
       </c>
-      <c r="J1" s="9" t="s">
+      <c r="O1" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="P1" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="L1" s="9" t="s">
-        <v>215</v>
-      </c>
-      <c r="M1" s="9" t="s">
+      <c r="Q1" s="9" t="s">
+        <v>213</v>
+      </c>
+      <c r="R1" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="N1" s="9" t="s">
+      <c r="S1" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="O1" s="9" t="s">
+      <c r="T1" s="9" t="s">
         <v>165</v>
       </c>
-      <c r="P1" s="9" t="s">
+      <c r="U1" s="9" t="s">
         <v>166</v>
       </c>
-      <c r="Q1" s="13" t="s">
+      <c r="V1" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="R1" s="13" t="s">
+      <c r="W1" s="13" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="2" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B26" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
@@ -1220,468 +1383,1452 @@
       <c r="C2" t="s">
         <v>124</v>
       </c>
-      <c r="D2" t="s">
+      <c r="H2" t="str">
+        <f t="shared" ref="H2:H5" si="1">IF(ISBLANK(F2),"",IF(COUNTIF($G$2:$G$101,G2)=1,"Yes","No"))</f>
+        <v/>
+      </c>
+      <c r="I2" t="s">
         <v>167</v>
       </c>
-      <c r="E2">
+      <c r="J2">
         <v>10</v>
       </c>
-      <c r="F2">
+      <c r="K2">
         <v>10</v>
       </c>
-      <c r="G2" s="8">
-        <v>0</v>
-      </c>
-      <c r="H2">
+      <c r="L2" s="8">
+        <v>0</v>
+      </c>
+      <c r="M2">
         <v>100</v>
       </c>
-      <c r="I2">
+      <c r="N2">
         <v>5</v>
       </c>
-      <c r="J2" s="8">
+      <c r="O2" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="P2" s="8">
+        <v>2</v>
+      </c>
+      <c r="Q2" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="R2">
+        <v>0</v>
+      </c>
+      <c r="S2">
+        <v>0</v>
+      </c>
+      <c r="T2">
+        <v>0</v>
+      </c>
+      <c r="U2">
+        <v>0</v>
+      </c>
+      <c r="V2" t="s">
+        <v>208</v>
+      </c>
+      <c r="W2" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="3" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>202</v>
+      </c>
+      <c r="B3" t="str">
+        <f t="shared" si="0"/>
+        <v>Conduit</v>
+      </c>
+      <c r="C3" t="s">
+        <v>205</v>
+      </c>
+      <c r="D3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E3" t="s">
+        <v>133</v>
+      </c>
+      <c r="F3" t="s">
+        <v>126</v>
+      </c>
+      <c r="G3" t="str">
+        <f>_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(D3:F3))</f>
+        <v>Air|Air|Fire</v>
+      </c>
+      <c r="H3" t="str">
+        <f t="shared" si="1"/>
+        <v>Yes</v>
+      </c>
+      <c r="I3" t="s">
+        <v>167</v>
+      </c>
+      <c r="J3">
+        <v>10</v>
+      </c>
+      <c r="K3">
+        <v>10</v>
+      </c>
+      <c r="L3" s="8">
+        <v>0</v>
+      </c>
+      <c r="M3">
+        <v>130</v>
+      </c>
+      <c r="N3">
+        <v>5</v>
+      </c>
+      <c r="O3" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="P3" s="8">
+        <v>2</v>
+      </c>
+      <c r="Q3" s="8">
+        <v>0.2</v>
+      </c>
+      <c r="R3">
+        <v>0</v>
+      </c>
+      <c r="S3">
+        <v>0</v>
+      </c>
+      <c r="T3">
+        <v>3</v>
+      </c>
+      <c r="U3">
+        <v>0</v>
+      </c>
+      <c r="V3" t="s">
+        <v>209</v>
+      </c>
+      <c r="W3" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>Rot</v>
+      </c>
+      <c r="C4" t="s">
+        <v>206</v>
+      </c>
+      <c r="D4" t="s">
+        <v>137</v>
+      </c>
+      <c r="E4" t="s">
+        <v>137</v>
+      </c>
+      <c r="F4" t="s">
+        <v>130</v>
+      </c>
+      <c r="G4" t="str">
+        <f t="shared" ref="G4:G67" si="2">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(D4:F4))</f>
+        <v>Earth|Earth|Water</v>
+      </c>
+      <c r="H4" t="str">
+        <f t="shared" si="1"/>
+        <v>Yes</v>
+      </c>
+      <c r="I4" t="s">
+        <v>167</v>
+      </c>
+      <c r="J4">
+        <v>5</v>
+      </c>
+      <c r="K4">
+        <v>10</v>
+      </c>
+      <c r="L4" s="8">
         <v>0.01</v>
       </c>
-      <c r="K2" s="8">
+      <c r="M4">
+        <v>80</v>
+      </c>
+      <c r="N4">
+        <v>7</v>
+      </c>
+      <c r="O4" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="P4" s="8">
         <v>2</v>
       </c>
-      <c r="L2" s="8">
+      <c r="Q4" s="8">
         <v>0.2</v>
       </c>
-      <c r="M2">
-        <v>0</v>
-      </c>
-      <c r="N2">
-        <v>0</v>
-      </c>
-      <c r="O2">
-        <v>0</v>
-      </c>
-      <c r="P2">
-        <v>0</v>
-      </c>
-      <c r="Q2" t="s">
+      <c r="R4">
+        <v>0</v>
+      </c>
+      <c r="S4">
+        <v>0</v>
+      </c>
+      <c r="T4">
+        <v>0</v>
+      </c>
+      <c r="U4">
+        <v>3</v>
+      </c>
+      <c r="V4" t="s">
         <v>210</v>
       </c>
-      <c r="R2" t="b">
+      <c r="W4" t="b">
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A3" t="s">
-        <v>203</v>
-      </c>
-      <c r="B3" t="str">
-        <f t="shared" si="0"/>
-        <v>Conduit</v>
-      </c>
-      <c r="C3" t="s">
-        <v>206</v>
-      </c>
-      <c r="D3" t="s">
+    <row r="5" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>204</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>Ghost</v>
+      </c>
+      <c r="C5" t="s">
+        <v>223</v>
+      </c>
+      <c r="D5" t="s">
+        <v>133</v>
+      </c>
+      <c r="E5" t="s">
+        <v>133</v>
+      </c>
+      <c r="F5" t="s">
+        <v>137</v>
+      </c>
+      <c r="G5" t="str">
+        <f t="shared" si="2"/>
+        <v>Air|Air|Earth</v>
+      </c>
+      <c r="H5" t="str">
+        <f t="shared" si="1"/>
+        <v>Yes</v>
+      </c>
+      <c r="I5" t="s">
         <v>167</v>
       </c>
-      <c r="E3">
+      <c r="J5">
         <v>10</v>
       </c>
-      <c r="F3">
+      <c r="K5">
         <v>10</v>
       </c>
-      <c r="G3" s="8">
-        <v>0</v>
-      </c>
-      <c r="H3">
-        <v>130</v>
-      </c>
-      <c r="I3">
-        <v>5</v>
-      </c>
-      <c r="J3" s="8">
-        <v>0.01</v>
-      </c>
-      <c r="K3" s="8">
+      <c r="L5" s="8">
+        <v>0</v>
+      </c>
+      <c r="M5">
+        <v>110</v>
+      </c>
+      <c r="N5">
         <v>2</v>
       </c>
-      <c r="L3" s="8">
+      <c r="O5" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="P5" s="8">
+        <v>2</v>
+      </c>
+      <c r="Q5" s="8">
         <v>0.2</v>
       </c>
-      <c r="M3">
-        <v>0</v>
-      </c>
-      <c r="N3">
-        <v>0</v>
-      </c>
-      <c r="O3">
+      <c r="R5">
+        <v>0</v>
+      </c>
+      <c r="S5">
+        <v>0</v>
+      </c>
+      <c r="T5">
+        <v>0</v>
+      </c>
+      <c r="U5">
+        <v>0</v>
+      </c>
+      <c r="V5" t="s">
+        <v>211</v>
+      </c>
+      <c r="W5" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="6" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>228</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>Inferno</v>
+      </c>
+      <c r="C6" t="s">
+        <v>229</v>
+      </c>
+      <c r="D6" t="s">
+        <v>126</v>
+      </c>
+      <c r="E6" t="s">
+        <v>126</v>
+      </c>
+      <c r="F6" t="s">
+        <v>126</v>
+      </c>
+      <c r="G6" t="str">
+        <f t="shared" si="2"/>
+        <v>Fire|Fire|Fire</v>
+      </c>
+      <c r="H6" t="str">
+        <f>IF(ISBLANK(F6),"",IF(COUNTIF($G$2:$G$101,G6)=1,"Yes","No"))</f>
+        <v>Yes</v>
+      </c>
+      <c r="I6" t="s">
+        <v>167</v>
+      </c>
+      <c r="J6">
+        <v>10</v>
+      </c>
+      <c r="K6">
+        <v>15</v>
+      </c>
+      <c r="L6" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="M6">
+        <v>90</v>
+      </c>
+      <c r="N6">
         <v>3</v>
       </c>
-      <c r="P3">
-        <v>0</v>
-      </c>
-      <c r="Q3" t="s">
-        <v>211</v>
-      </c>
-      <c r="R3" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="4" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
-        <v>204</v>
-      </c>
-      <c r="B4" t="str">
-        <f t="shared" si="0"/>
-        <v>Rot</v>
-      </c>
-      <c r="C4" t="s">
-        <v>208</v>
-      </c>
-      <c r="D4" t="s">
-        <v>167</v>
-      </c>
-      <c r="E4">
-        <v>5</v>
-      </c>
-      <c r="F4">
-        <v>10</v>
-      </c>
-      <c r="G4" s="8">
-        <v>0.01</v>
-      </c>
-      <c r="H4">
-        <v>80</v>
-      </c>
-      <c r="I4">
-        <v>7</v>
-      </c>
-      <c r="J4" s="8">
-        <v>0.01</v>
-      </c>
-      <c r="K4" s="8">
+      <c r="O6" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="P6" s="8">
         <v>2</v>
       </c>
-      <c r="L4" s="8">
+      <c r="Q6" s="8">
         <v>0.2</v>
       </c>
-      <c r="M4">
-        <v>0</v>
-      </c>
-      <c r="N4">
-        <v>0</v>
-      </c>
-      <c r="O4">
-        <v>0</v>
-      </c>
-      <c r="P4">
+      <c r="R6">
         <v>3</v>
       </c>
-      <c r="Q4" t="s">
-        <v>212</v>
-      </c>
-      <c r="R4" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
-        <v>205</v>
-      </c>
-      <c r="B5" t="str">
-        <f t="shared" si="0"/>
-        <v>Ghost</v>
-      </c>
-      <c r="C5" t="s">
-        <v>207</v>
-      </c>
-      <c r="D5" t="s">
-        <v>167</v>
-      </c>
-      <c r="E5">
-        <v>10</v>
-      </c>
-      <c r="F5">
-        <v>10</v>
-      </c>
-      <c r="G5" s="8">
-        <v>0</v>
-      </c>
-      <c r="H5">
-        <v>110</v>
-      </c>
-      <c r="I5">
-        <v>2</v>
-      </c>
-      <c r="J5" s="8">
-        <v>0.01</v>
-      </c>
-      <c r="K5" s="8">
-        <v>2</v>
-      </c>
-      <c r="L5" s="8">
-        <v>0.2</v>
-      </c>
-      <c r="M5">
-        <v>0</v>
-      </c>
-      <c r="N5">
-        <v>0</v>
-      </c>
-      <c r="O5">
-        <v>0</v>
-      </c>
-      <c r="P5">
-        <v>0</v>
-      </c>
-      <c r="Q5" t="s">
-        <v>213</v>
-      </c>
-      <c r="R5" t="b">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="6" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="B6" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-    </row>
-    <row r="7" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S6" s="8">
+        <v>0</v>
+      </c>
+      <c r="T6" s="8">
+        <v>0</v>
+      </c>
+      <c r="U6" s="8">
+        <v>0</v>
+      </c>
+      <c r="W6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="8" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="G7" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H7" t="str">
+        <f t="shared" ref="H7:H70" si="3">IF(ISBLANK(F7),"",IF(COUNTIF($G$2:$G$101,G7)=1,"Yes","No"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="8" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="9" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="G8" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H8" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="9" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="10" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="G9" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H9" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="11" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="G10" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H10" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="11" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="12" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="G11" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H11" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="13" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="G12" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H12" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="14" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="G13" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H13" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="15" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="G14" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H14" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B15" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="16" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="G15" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H15" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:23" x14ac:dyDescent="0.25">
       <c r="B16" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="G16" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H16" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B17" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="18" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="G17" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H17" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B18" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="19" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="G18" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H18" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B19" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="20" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="G19" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H19" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B20" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="21" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="G20" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H20" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B21" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="22" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="G21" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H21" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B22" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="23" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="G22" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H22" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B23" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="24" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="G23" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H23" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B24" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="25" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="G24" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H24" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B25" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="26" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="G25" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H25" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B26" t="str">
         <f t="shared" si="0"/>
         <v/>
       </c>
-    </row>
-    <row r="27" spans="2:2" x14ac:dyDescent="0.25">
+      <c r="G26" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H26" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B27" t="str">
-        <f t="shared" ref="B27:B44" si="1">PROPER(SUBSTITUTE(A27,"_"," "))</f>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" ref="B27:B44" si="4">PROPER(SUBSTITUTE(A27,"_"," "))</f>
+        <v/>
+      </c>
+      <c r="G27" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H27" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B28" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G28" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H28" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B29" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G29" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H29" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B30" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="31" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G30" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H30" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B31" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="32" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G31" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H31" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B32" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="33" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G32" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H32" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B33" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="34" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G33" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H33" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B34" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="35" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G34" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H34" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B35" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="36" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G35" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H35" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B36" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="37" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G36" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H36" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="37" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B37" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="38" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G37" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H37" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B38" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="39" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G38" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H38" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B39" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="40" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G39" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H39" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="40" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B40" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="41" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G40" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H40" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B41" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="42" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G41" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H41" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B42" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="43" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G42" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H42" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B43" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="44" spans="2:2" x14ac:dyDescent="0.25">
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G43" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H43" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="2:8" x14ac:dyDescent="0.25">
       <c r="B44" t="str">
-        <f t="shared" si="1"/>
+        <f t="shared" si="4"/>
+        <v/>
+      </c>
+      <c r="G44" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H44" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="45" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="G45" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H45" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="46" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="G46" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H46" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="47" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="G47" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H47" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="48" spans="2:8" x14ac:dyDescent="0.25">
+      <c r="G48" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H48" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G49" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H49" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="50" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G50" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H50" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="51" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G51" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H51" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G52" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H52" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="53" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G53" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H53" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="54" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G54" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H54" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="55" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G55" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H55" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="56" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G56" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H56" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="57" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G57" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H57" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="58" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G58" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H58" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="59" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G59" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H59" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="60" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G60" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H60" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="61" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G61" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H61" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="62" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G62" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H62" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="63" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G63" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H63" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="64" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G64" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H64" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="65" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G65" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H65" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="66" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G66" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H66" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="67" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G67" t="str">
+        <f t="shared" si="2"/>
+        <v/>
+      </c>
+      <c r="H67" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="68" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G68" t="str">
+        <f t="shared" ref="G68:G98" si="5">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(D68:F68))</f>
+        <v/>
+      </c>
+      <c r="H68" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="69" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G69" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H69" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="70" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G70" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H70" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="71" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G71" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H71" t="str">
+        <f t="shared" ref="H71:H98" si="6">IF(ISBLANK(F71),"",IF(COUNTIF($G$2:$G$101,G71)=1,"Yes","No"))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="72" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G72" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H72" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="73" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G73" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H73" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="74" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G74" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H74" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="75" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G75" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H75" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="76" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G76" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H76" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="77" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G77" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H77" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="78" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G78" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H78" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="79" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G79" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H79" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="80" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G80" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H80" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="81" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G81" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H81" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="82" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G82" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H82" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="83" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G83" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H83" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="84" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G84" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H84" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="85" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G85" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H85" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="86" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G86" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H86" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="87" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G87" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H87" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="88" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G88" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H88" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="89" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G89" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H89" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="90" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G90" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H90" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="91" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G91" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H91" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="92" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G92" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H92" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="93" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G93" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H93" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="94" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G94" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H94" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="95" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G95" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H95" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="96" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G96" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H96" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="97" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G97" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H97" t="str">
+        <f t="shared" si="6"/>
+        <v/>
+      </c>
+    </row>
+    <row r="98" spans="7:8" x14ac:dyDescent="0.25">
+      <c r="G98" t="str">
+        <f t="shared" si="5"/>
+        <v/>
+      </c>
+      <c r="H98" t="str">
+        <f t="shared" si="6"/>
         <v/>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:R44" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:W44" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <conditionalFormatting sqref="H1 D1:F111 D112:H1048576">
+    <cfRule type="cellIs" dxfId="12" priority="1" operator="equal">
+      <formula>"Earth"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="11" priority="2" operator="equal">
+      <formula>"Water"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="10" priority="3" operator="equal">
+      <formula>"Fire"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="9" priority="4" operator="equal">
+      <formula>"Air"</formula>
+    </cfRule>
+  </conditionalFormatting>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DFC42C69-7304-40C7-BA02-8A3EB2712138}">
           <x14:formula1>
             <xm:f>motion!$A$2:$A$30</xm:f>
           </x14:formula1>
-          <xm:sqref>D2:D50</xm:sqref>
+          <xm:sqref>I2:I50</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{E5B318B9-C4FE-4359-9562-7862AB8A9B76}">
+          <x14:formula1>
+            <xm:f>input!$C$2:$F$2</xm:f>
+          </x14:formula1>
+          <xm:sqref>D2:F99</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -1705,28 +2852,28 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="B1" s="3" t="s">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="3" t="s">
+      <c r="C1" s="4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="3" t="s">
+      <c r="D1" s="4" t="s">
         <v>154</v>
       </c>
-      <c r="E1" s="3" t="s">
-        <v>214</v>
-      </c>
-      <c r="F1" s="3" t="s">
+      <c r="E1" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="G1" s="3" t="s">
+      <c r="G1" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="H1" s="3" t="s">
+      <c r="H1" s="4" t="s">
         <v>142</v>
       </c>
     </row>
@@ -1874,13 +3021,13 @@
         <v>Bounty</v>
       </c>
       <c r="C7" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D7" t="s">
         <v>130</v>
       </c>
       <c r="E7" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="F7" s="8">
         <v>0.01</v>
@@ -2060,6 +3207,847 @@
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{63A1687E-9087-4AF4-BB85-417F5711F916}">
+  <sheetPr>
+    <tabColor theme="5" tint="0.59999389629810485"/>
+  </sheetPr>
+  <dimension ref="A1:I106"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="1" max="1" width="12.7109375" customWidth="1"/>
+    <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="4" max="4" width="94.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="0" hidden="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A1" s="4" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="4" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="4" t="s">
+        <v>221</v>
+      </c>
+      <c r="D1" s="4" t="s">
+        <v>2</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>216</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>217</v>
+      </c>
+      <c r="G1" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="I1" s="16" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>220</v>
+      </c>
+      <c r="B2" t="str">
+        <f t="shared" ref="B2:B4" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
+        <v>Haunt</v>
+      </c>
+      <c r="C2" t="s">
+        <v>204</v>
+      </c>
+      <c r="D2" t="s">
+        <v>226</v>
+      </c>
+      <c r="E2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F2" t="s">
+        <v>133</v>
+      </c>
+      <c r="G2" t="s">
+        <v>130</v>
+      </c>
+      <c r="H2" t="str">
+        <f>_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(E2:G2))</f>
+        <v>Air|Air|Water</v>
+      </c>
+      <c r="I2" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>224</v>
+      </c>
+      <c r="B3" t="str">
+        <f t="shared" si="0"/>
+        <v>Possesion</v>
+      </c>
+      <c r="C3" t="s">
+        <v>204</v>
+      </c>
+      <c r="D3" t="s">
+        <v>227</v>
+      </c>
+      <c r="E3" t="s">
+        <v>126</v>
+      </c>
+      <c r="F3" t="s">
+        <v>126</v>
+      </c>
+      <c r="G3" t="s">
+        <v>133</v>
+      </c>
+      <c r="H3" t="str">
+        <f t="shared" ref="H3:H66" si="1">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(E3:G3))</f>
+        <v>Fire|Fire|Air</v>
+      </c>
+      <c r="I3" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>230</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>Trail</v>
+      </c>
+      <c r="C4" t="s">
+        <v>228</v>
+      </c>
+      <c r="D4" t="s">
+        <v>231</v>
+      </c>
+      <c r="E4" t="s">
+        <v>126</v>
+      </c>
+      <c r="F4" t="s">
+        <v>126</v>
+      </c>
+      <c r="G4" t="s">
+        <v>137</v>
+      </c>
+      <c r="H4" t="str">
+        <f t="shared" si="1"/>
+        <v>Fire|Fire|Earth</v>
+      </c>
+      <c r="I4" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
+        <v>232</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" ref="B5:B6" si="2">PROPER(SUBSTITUTE(A5,"_"," "))</f>
+        <v>Kindling</v>
+      </c>
+      <c r="C5" t="s">
+        <v>228</v>
+      </c>
+      <c r="D5" t="s">
+        <v>233</v>
+      </c>
+      <c r="E5" t="s">
+        <v>133</v>
+      </c>
+      <c r="F5" t="s">
+        <v>133</v>
+      </c>
+      <c r="G5" t="s">
+        <v>126</v>
+      </c>
+      <c r="H5" t="str">
+        <f t="shared" si="1"/>
+        <v>Air|Air|Fire</v>
+      </c>
+      <c r="I5" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A6" t="s">
+        <v>235</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="2"/>
+        <v>Spark</v>
+      </c>
+      <c r="C6" t="s">
+        <v>228</v>
+      </c>
+      <c r="D6" t="s">
+        <v>234</v>
+      </c>
+      <c r="E6" t="s">
+        <v>126</v>
+      </c>
+      <c r="F6" t="s">
+        <v>126</v>
+      </c>
+      <c r="G6" t="s">
+        <v>126</v>
+      </c>
+      <c r="H6" t="str">
+        <f t="shared" si="1"/>
+        <v>Fire|Fire|Fire</v>
+      </c>
+      <c r="I6" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H7" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H8" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H9" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H10" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H11" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H12" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H13" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H14" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H15" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="H16" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="17" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H17" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="18" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H18" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="19" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H19" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="20" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H20" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="21" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H21" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="22" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H22" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="23" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H23" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="24" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H24" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="25" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H25" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="26" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H26" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="27" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H27" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="28" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H28" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="29" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H29" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="30" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H30" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="31" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H31" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="32" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H32" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="33" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H33" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="34" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H34" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="35" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H35" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="36" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H36" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="37" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H37" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="38" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H38" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="39" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H39" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="40" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H40" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="41" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H41" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="42" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H42" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="43" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H43" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="44" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H44" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="45" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H45" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="46" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H46" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="47" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H47" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="48" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H48" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="49" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H49" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="50" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H50" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="51" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H51" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="52" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H52" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="53" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H53" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="54" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H54" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="55" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H55" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="56" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H56" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="57" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H57" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="58" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H58" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="59" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H59" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="60" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H60" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="61" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H61" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="62" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H62" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="63" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H63" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="64" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H64" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="65" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H65" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="66" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H66" t="str">
+        <f t="shared" si="1"/>
+        <v/>
+      </c>
+    </row>
+    <row r="67" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H67" t="str">
+        <f t="shared" ref="H67:H106" si="3">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(E67:G67))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="68" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H68" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="69" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H69" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="70" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H70" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="71" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H71" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="72" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H72" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="73" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H73" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="74" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H74" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="75" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H75" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="76" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H76" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="77" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H77" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="78" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H78" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="79" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H79" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="80" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H80" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="81" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H81" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="82" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H82" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="83" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H83" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="84" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H84" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="85" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H85" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="86" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H86" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="87" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H87" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="88" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H88" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="89" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H89" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="90" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H90" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="91" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H91" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="92" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H92" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="93" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H93" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="94" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H94" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="95" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H95" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="96" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H96" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="97" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H97" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="98" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H98" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="99" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H99" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="100" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H100" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="101" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H101" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="102" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H102" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="103" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H103" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="104" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H104" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="105" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H105" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+    <row r="106" spans="8:8" x14ac:dyDescent="0.25">
+      <c r="H106" t="str">
+        <f t="shared" si="3"/>
+        <v/>
+      </c>
+    </row>
+  </sheetData>
+  <conditionalFormatting sqref="E1:G5 I1">
+    <cfRule type="cellIs" dxfId="8" priority="5" operator="equal">
+      <formula>"Earth"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="7" priority="6" operator="equal">
+      <formula>"Water"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
+      <formula>"Fire"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="5" priority="8" operator="equal">
+      <formula>"Air"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="E6:G89">
+    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+      <formula>"Earth"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+      <formula>"Water"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+      <formula>"Fire"</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="1" priority="4" operator="equal">
+      <formula>"Air"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B44CB842-296D-43B5-8EC4-12AD766FB2C3}">
+          <x14:formula1>
+            <xm:f>input!$C$2:$F$2</xm:f>
+          </x14:formula1>
+          <xm:sqref>E2:G89</xm:sqref>
+        </x14:dataValidation>
+      </x14:dataValidations>
+    </ext>
+  </extLst>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C3C10F13-8E40-4AB2-9849-0A8DFD3352A1}">
   <sheetPr>
     <tabColor theme="4" tint="0.59999389629810485"/>
@@ -2088,7 +4076,7 @@
         <v>167</v>
       </c>
       <c r="B2" t="str">
-        <f t="shared" ref="B2" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
+        <f t="shared" ref="B2:B18" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Wayward</v>
       </c>
       <c r="C2" t="s">
@@ -2097,130 +4085,194 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>225</v>
+      </c>
+      <c r="B3" t="str">
+        <f t="shared" si="0"/>
+        <v>Attracted</v>
+      </c>
+      <c r="C3" t="s">
         <v>170</v>
-      </c>
-      <c r="C3" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>Spite</v>
+      </c>
+      <c r="C4" t="s">
         <v>172</v>
-      </c>
-      <c r="C4" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>173</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>Rooted</v>
+      </c>
+      <c r="C5" t="s">
         <v>174</v>
-      </c>
-      <c r="C5" t="s">
-        <v>175</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>177</v>
+        <v>176</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>Patrol</v>
       </c>
       <c r="C6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>177</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>Familiar</v>
+      </c>
+      <c r="C7" t="s">
         <v>178</v>
-      </c>
-      <c r="C7" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>179</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>Rail</v>
+      </c>
+      <c r="C8" t="s">
         <v>180</v>
-      </c>
-      <c r="C8" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>181</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>Tide</v>
+      </c>
+      <c r="C9" t="s">
         <v>182</v>
-      </c>
-      <c r="C9" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>183</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>Blink</v>
+      </c>
+      <c r="C10" t="s">
         <v>184</v>
-      </c>
-      <c r="C10" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>185</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>Loyal</v>
+      </c>
+      <c r="C11" t="s">
         <v>186</v>
-      </c>
-      <c r="C11" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>187</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>Hexed</v>
+      </c>
+      <c r="C12" t="s">
         <v>188</v>
-      </c>
-      <c r="C12" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>189</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>Stalker</v>
+      </c>
+      <c r="C13" t="s">
         <v>190</v>
-      </c>
-      <c r="C13" t="s">
-        <v>191</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>192</v>
+        <v>191</v>
+      </c>
+      <c r="B14" t="str">
+        <f t="shared" si="0"/>
+        <v>Herd</v>
       </c>
       <c r="C14" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>192</v>
+      </c>
+      <c r="B15" t="str">
+        <f t="shared" si="0"/>
+        <v>Greedy</v>
+      </c>
+      <c r="C15" t="s">
         <v>193</v>
-      </c>
-      <c r="C15" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>195</v>
+      </c>
+      <c r="B16" t="str">
+        <f t="shared" si="0"/>
+        <v>Oathbound</v>
+      </c>
+      <c r="C16" t="s">
         <v>196</v>
-      </c>
-      <c r="C16" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>197</v>
+      </c>
+      <c r="B17" t="str">
+        <f t="shared" si="0"/>
+        <v>Echo</v>
+      </c>
+      <c r="C17" t="s">
         <v>198</v>
-      </c>
-      <c r="C17" t="s">
-        <v>199</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>199</v>
+      </c>
+      <c r="B18" t="str">
+        <f t="shared" si="0"/>
+        <v>Phasing</v>
+      </c>
+      <c r="C18" t="s">
         <v>200</v>
-      </c>
-      <c r="C18" t="s">
-        <v>201</v>
       </c>
     </row>
   </sheetData>
@@ -2228,7 +4280,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <sheetPr>
     <tabColor theme="8" tint="0.59999389629810485"/>
@@ -3912,26 +5964,35 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0C00-000000000000}">
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A2:D2"/>
+  <dimension ref="A2:F2"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <cols>
+    <col min="2" max="2" width="17.28515625" customWidth="1"/>
+  </cols>
   <sheetData>
-    <row r="2" spans="1:4" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:6" ht="15.6" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A2" s="5" t="s">
         <v>123</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>5</v>
+        <v>215</v>
       </c>
       <c r="C2" t="s">
-        <v>18</v>
+        <v>126</v>
       </c>
       <c r="D2" t="s">
-        <v>95</v>
+        <v>130</v>
+      </c>
+      <c r="E2" t="s">
+        <v>133</v>
+      </c>
+      <c r="F2" t="s">
+        <v>137</v>
       </c>
     </row>
   </sheetData>
@@ -3939,12 +6000,12 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0D00-000000000000}">
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:C30"/>
+  <dimension ref="A1:C41"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="14.7109375" customWidth="1"/>
@@ -3999,7 +6060,7 @@
         <v>123</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>168</v>
+        <v>216</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>119</v>
@@ -4010,10 +6071,10 @@
         <v>123</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>156</v>
+        <v>217</v>
       </c>
       <c r="C6" s="11" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
@@ -4021,10 +6082,10 @@
         <v>123</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>157</v>
+        <v>218</v>
       </c>
       <c r="C7" s="11" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
@@ -4032,10 +6093,10 @@
         <v>123</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>158</v>
+        <v>168</v>
       </c>
       <c r="C8" s="11" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
@@ -4043,7 +6104,7 @@
         <v>123</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>122</v>
@@ -4054,7 +6115,7 @@
         <v>123</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>122</v>
@@ -4065,7 +6126,7 @@
         <v>123</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>122</v>
@@ -4076,7 +6137,7 @@
         <v>123</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>122</v>
@@ -4087,7 +6148,7 @@
         <v>123</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>215</v>
+        <v>160</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>122</v>
@@ -4098,10 +6159,10 @@
         <v>123</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C14" s="11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -4109,10 +6170,10 @@
         <v>123</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="C15" s="11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
@@ -4120,10 +6181,10 @@
         <v>123</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>165</v>
+        <v>213</v>
       </c>
       <c r="C16" s="11" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
@@ -4131,7 +6192,7 @@
         <v>123</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>120</v>
@@ -4142,10 +6203,10 @@
         <v>123</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>109</v>
+        <v>164</v>
       </c>
       <c r="C18" s="11" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
     </row>
     <row r="19" spans="1:3" x14ac:dyDescent="0.25">
@@ -4153,51 +6214,51 @@
         <v>123</v>
       </c>
       <c r="B19" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="C19" s="11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B20" s="11" t="s">
+        <v>166</v>
+      </c>
+      <c r="C20" s="11" t="s">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B21" s="11" t="s">
+        <v>109</v>
+      </c>
+      <c r="C21" s="11" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="11" t="s">
+        <v>123</v>
+      </c>
+      <c r="B22" s="11" t="s">
         <v>14</v>
       </c>
-      <c r="C19" s="11" t="s">
+      <c r="C22" s="11" t="s">
         <v>121</v>
-      </c>
-    </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A20" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="B20" s="12" t="s">
-        <v>0</v>
-      </c>
-      <c r="C20" s="12" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A21" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="B21" s="12" t="s">
-        <v>1</v>
-      </c>
-      <c r="C21" s="12" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A22" s="12" t="s">
-        <v>209</v>
-      </c>
-      <c r="B22" s="12" t="s">
-        <v>2</v>
-      </c>
-      <c r="C22" s="12" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B23" s="12" t="s">
-        <v>154</v>
+        <v>0</v>
       </c>
       <c r="C23" s="12" t="s">
         <v>119</v>
@@ -4205,10 +6266,10 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B24" s="12" t="s">
-        <v>214</v>
+        <v>1</v>
       </c>
       <c r="C24" s="12" t="s">
         <v>119</v>
@@ -4216,67 +6277,188 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B25" s="12" t="s">
-        <v>140</v>
+        <v>2</v>
       </c>
       <c r="C25" s="12" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>141</v>
+        <v>154</v>
       </c>
       <c r="C26" s="12" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B27" s="12" t="s">
+        <v>212</v>
+      </c>
+      <c r="C27" s="12" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="B28" s="12" t="s">
+        <v>140</v>
+      </c>
+      <c r="C28" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="B29" s="12" t="s">
+        <v>141</v>
+      </c>
+      <c r="C29" s="12" t="s">
+        <v>122</v>
+      </c>
+    </row>
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="12" t="s">
+        <v>207</v>
+      </c>
+      <c r="B30" s="12" t="s">
         <v>142</v>
       </c>
-      <c r="C27" s="12" t="s">
+      <c r="C30" s="12" t="s">
         <v>122</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A28" s="14" t="s">
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="B31" s="15" t="s">
+        <v>0</v>
+      </c>
+      <c r="C31" s="15" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="B32" s="15" t="s">
+        <v>1</v>
+      </c>
+      <c r="C32" s="15" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="B33" s="15" t="s">
+        <v>221</v>
+      </c>
+      <c r="C33" s="15" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="B34" s="15" t="s">
+        <v>2</v>
+      </c>
+      <c r="C34" s="15" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="B35" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="C35" s="15" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="B36" s="15" t="s">
+        <v>217</v>
+      </c>
+      <c r="C36" s="15" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="37" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A37" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="B37" s="15" t="s">
+        <v>218</v>
+      </c>
+      <c r="C37" s="15" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="38" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A38" s="15" t="s">
+        <v>222</v>
+      </c>
+      <c r="B38" s="15" t="s">
+        <v>14</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="B28" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="C28" s="14" t="s">
+      <c r="B39" s="14" t="s">
+        <v>0</v>
+      </c>
+      <c r="C39" s="14" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A29" s="14" t="s">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="B29" s="14" t="s">
+      <c r="B40" s="14" t="s">
         <v>1</v>
       </c>
-      <c r="C29" s="14" t="s">
+      <c r="C40" s="14" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A30" s="14" t="s">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="14" t="s">
         <v>168</v>
       </c>
-      <c r="B30" s="14" t="s">
+      <c r="B41" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C30" s="14" t="s">
+      <c r="C41" s="14" t="s">
         <v>119</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Implement Blank Orb mechanics and update game design documentation
- Introduced the **Blank Orb** as the starting weapon for players, launching from the summoning circle in a random direction.
- Revised game design documents to reflect changes in gameplay mechanics, including the new orb attributes and glyph integration.
- Enhanced the ritual menu UI to facilitate orb upgrades and glyph socketing, improving player interaction.
- Updated `GAME_BRIEF.md` to clarify the gameplay loop and player strategies involving the Blank Orb and glyphs.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\One Last Bullet\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2511F6C2-22E4-4F9C-BBC2-CF77A815396F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ABF32D9-303A-45E6-A6D4-93FEE1D1B812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -417,9 +417,6 @@
     <t>orbs</t>
   </si>
   <si>
-    <t>Standard orb with no effect</t>
-  </si>
-  <si>
     <t>Burn on enemy hit</t>
   </si>
   <si>
@@ -714,9 +711,6 @@
     <t>attunements</t>
   </si>
   <si>
-    <t>Enters and haunts enemies and deal its impact damage per second to them. Once dead, exits in a random direction</t>
-  </si>
-  <si>
     <t>possesion</t>
   </si>
   <si>
@@ -751,6 +745,12 @@
   </si>
   <si>
     <t>spark</t>
+  </si>
+  <si>
+    <t>Enters and haunts enemies and deal its impact damage per second to them. Once dead, exits in a random direction.</t>
+  </si>
+  <si>
+    <t>No effect</t>
   </si>
 </sst>
 </file>
@@ -862,7 +862,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -881,7 +881,6 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1293,10 +1292,10 @@
     <col min="9" max="9" width="15" customWidth="1"/>
     <col min="10" max="10" width="10.42578125" customWidth="1"/>
     <col min="11" max="11" width="15.42578125" customWidth="1"/>
-    <col min="12" max="12" width="8.85546875" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="8.5703125" customWidth="1"/>
-    <col min="14" max="14" width="9.140625" customWidth="1"/>
-    <col min="15" max="17" width="14.5703125" customWidth="1"/>
+    <col min="12" max="13" width="14.5703125" customWidth="1"/>
+    <col min="14" max="14" width="8.5703125" customWidth="1"/>
+    <col min="16" max="16" width="8.85546875" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="14.5703125" customWidth="1"/>
     <col min="18" max="18" width="8.85546875" customWidth="1"/>
     <col min="19" max="19" width="8.42578125" customWidth="1"/>
     <col min="20" max="20" width="8.5703125" customWidth="1"/>
@@ -1312,58 +1311,58 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>218</v>
       </c>
-      <c r="H1" s="4" t="s">
-        <v>219</v>
-      </c>
       <c r="I1" s="10" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="J1" s="9" t="s">
+        <v>155</v>
+      </c>
+      <c r="K1" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>161</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="O1" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="P1" s="9" t="s">
         <v>157</v>
       </c>
-      <c r="L1" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="M1" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="N1" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="O1" s="9" t="s">
-        <v>161</v>
-      </c>
-      <c r="P1" s="9" t="s">
+      <c r="Q1" s="9" t="s">
+        <v>212</v>
+      </c>
+      <c r="R1" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="Q1" s="9" t="s">
-        <v>213</v>
-      </c>
-      <c r="R1" s="9" t="s">
+      <c r="S1" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="T1" s="9" t="s">
         <v>164</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="U1" s="9" t="s">
         <v>165</v>
-      </c>
-      <c r="U1" s="9" t="s">
-        <v>166</v>
       </c>
       <c r="V1" s="13" t="s">
         <v>109</v>
@@ -1374,21 +1373,21 @@
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B26" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Blank</v>
       </c>
       <c r="C2" t="s">
-        <v>124</v>
+        <v>235</v>
       </c>
       <c r="H2" t="str">
         <f t="shared" ref="H2:H5" si="1">IF(ISBLANK(F2),"",IF(COUNTIF($G$2:$G$101,G2)=1,"Yes","No"))</f>
         <v/>
       </c>
       <c r="I2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J2">
         <v>10</v>
@@ -1397,19 +1396,19 @@
         <v>10</v>
       </c>
       <c r="L2" s="8">
-        <v>0</v>
-      </c>
-      <c r="M2">
+        <v>0.05</v>
+      </c>
+      <c r="M2" s="8">
+        <v>2</v>
+      </c>
+      <c r="N2">
         <v>100</v>
       </c>
-      <c r="N2">
+      <c r="O2">
         <v>5</v>
       </c>
-      <c r="O2" s="8">
-        <v>0.05</v>
-      </c>
       <c r="P2" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q2" s="8">
         <v>0.2</v>
@@ -1427,7 +1426,7 @@
         <v>0</v>
       </c>
       <c r="V2" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="W2" t="b">
         <v>1</v>
@@ -1435,23 +1434,23 @@
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Conduit</v>
       </c>
       <c r="C3" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G3" t="str">
         <f>_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(D3:F3))</f>
@@ -1462,7 +1461,7 @@
         <v>Yes</v>
       </c>
       <c r="I3" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J3">
         <v>10</v>
@@ -1471,19 +1470,19 @@
         <v>10</v>
       </c>
       <c r="L3" s="8">
-        <v>0</v>
-      </c>
-      <c r="M3">
+        <v>0.05</v>
+      </c>
+      <c r="M3" s="8">
+        <v>2</v>
+      </c>
+      <c r="N3">
         <v>130</v>
       </c>
-      <c r="N3">
+      <c r="O3">
         <v>5</v>
       </c>
-      <c r="O3" s="8">
-        <v>0.05</v>
-      </c>
       <c r="P3" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q3" s="8">
         <v>0.2</v>
@@ -1501,7 +1500,7 @@
         <v>0</v>
       </c>
       <c r="V3" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="W3" t="b">
         <v>1</v>
@@ -1509,23 +1508,23 @@
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Rot</v>
       </c>
       <c r="C4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="D4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F4" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="G4" t="str">
         <f t="shared" ref="G4:G67" si="2">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(D4:F4))</f>
@@ -1536,7 +1535,7 @@
         <v>Yes</v>
       </c>
       <c r="I4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J4">
         <v>5</v>
@@ -1545,19 +1544,19 @@
         <v>10</v>
       </c>
       <c r="L4" s="8">
+        <v>0.05</v>
+      </c>
+      <c r="M4" s="8">
+        <v>2</v>
+      </c>
+      <c r="N4">
+        <v>80</v>
+      </c>
+      <c r="O4">
+        <v>7</v>
+      </c>
+      <c r="P4" s="8">
         <v>0.01</v>
-      </c>
-      <c r="M4">
-        <v>80</v>
-      </c>
-      <c r="N4">
-        <v>7</v>
-      </c>
-      <c r="O4" s="8">
-        <v>0.05</v>
-      </c>
-      <c r="P4" s="8">
-        <v>2</v>
       </c>
       <c r="Q4" s="8">
         <v>0.2</v>
@@ -1575,7 +1574,7 @@
         <v>3</v>
       </c>
       <c r="V4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="W4" t="b">
         <v>1</v>
@@ -1583,23 +1582,23 @@
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Ghost</v>
       </c>
       <c r="C5" t="s">
-        <v>223</v>
+        <v>234</v>
       </c>
       <c r="D5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F5" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="G5" t="str">
         <f t="shared" si="2"/>
@@ -1610,7 +1609,7 @@
         <v>Yes</v>
       </c>
       <c r="I5" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J5">
         <v>10</v>
@@ -1619,19 +1618,19 @@
         <v>10</v>
       </c>
       <c r="L5" s="8">
-        <v>0</v>
-      </c>
-      <c r="M5">
+        <v>0.05</v>
+      </c>
+      <c r="M5" s="8">
+        <v>2</v>
+      </c>
+      <c r="N5">
         <v>110</v>
       </c>
-      <c r="N5">
+      <c r="O5">
         <v>2</v>
       </c>
-      <c r="O5" s="8">
-        <v>0.05</v>
-      </c>
       <c r="P5" s="8">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="Q5" s="8">
         <v>0.2</v>
@@ -1649,7 +1648,7 @@
         <v>0</v>
       </c>
       <c r="V5" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="W5" t="b">
         <v>1</v>
@@ -1657,23 +1656,23 @@
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Inferno</v>
       </c>
       <c r="C6" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="D6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G6" t="str">
         <f t="shared" si="2"/>
@@ -1684,7 +1683,7 @@
         <v>Yes</v>
       </c>
       <c r="I6" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J6">
         <v>10</v>
@@ -1695,17 +1694,17 @@
       <c r="L6" s="8">
         <v>0.05</v>
       </c>
-      <c r="M6">
+      <c r="M6" s="8">
+        <v>2</v>
+      </c>
+      <c r="N6">
         <v>90</v>
       </c>
-      <c r="N6">
+      <c r="O6">
         <v>3</v>
       </c>
-      <c r="O6" s="8">
+      <c r="P6" s="8">
         <v>0.05</v>
-      </c>
-      <c r="P6" s="8">
-        <v>2</v>
       </c>
       <c r="Q6" s="8">
         <v>0.2</v>
@@ -2817,7 +2816,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DFC42C69-7304-40C7-BA02-8A3EB2712138}">
           <x14:formula1>
             <xm:f>motion!$A$2:$A$30</xm:f>
@@ -2862,37 +2861,37 @@
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F1" s="4" t="s">
+        <v>139</v>
+      </c>
+      <c r="G1" s="4" t="s">
         <v>140</v>
       </c>
-      <c r="G1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>141</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>142</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="B2" t="str">
         <f>PROPER(A2)</f>
         <v>Coal</v>
       </c>
       <c r="C2" t="s">
+        <v>124</v>
+      </c>
+      <c r="D2" t="s">
         <v>125</v>
       </c>
-      <c r="D2" t="s">
-        <v>126</v>
-      </c>
       <c r="E2" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -2906,20 +2905,20 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" ref="B3:B13" si="0">PROPER(A3)</f>
         <v>Fury</v>
       </c>
       <c r="C3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E3" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -2933,20 +2932,20 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Blast</v>
       </c>
       <c r="C4" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
       <c r="D4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="E4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F4" s="6">
         <v>0.05</v>
@@ -2960,20 +2959,20 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Rime</v>
       </c>
       <c r="C5" t="s">
+        <v>128</v>
+      </c>
+      <c r="D5" t="s">
         <v>129</v>
       </c>
-      <c r="D5" t="s">
-        <v>130</v>
-      </c>
       <c r="E5" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -2987,20 +2986,20 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Soft</v>
       </c>
       <c r="C6" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="D6" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E6" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F6">
         <v>-10</v>
@@ -3014,20 +3013,20 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Bounty</v>
       </c>
       <c r="C7" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="D7" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="F7" s="8">
         <v>0.01</v>
@@ -3041,20 +3040,20 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
         <v>Static</v>
       </c>
       <c r="C8" t="s">
+        <v>131</v>
+      </c>
+      <c r="D8" t="s">
         <v>132</v>
       </c>
-      <c r="D8" t="s">
-        <v>133</v>
-      </c>
       <c r="E8" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -3068,20 +3067,20 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
         <v>Shear</v>
       </c>
       <c r="C9" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D9" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E9" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F9" s="6">
         <v>0.01</v>
@@ -3095,20 +3094,20 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
         <v>Drag</v>
       </c>
       <c r="C10" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D10" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E10" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F10">
         <v>-10</v>
@@ -3122,20 +3121,20 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
         <v>Blight</v>
       </c>
       <c r="C11" t="s">
+        <v>135</v>
+      </c>
+      <c r="D11" t="s">
         <v>136</v>
       </c>
-      <c r="D11" t="s">
-        <v>137</v>
-      </c>
       <c r="E11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -3149,20 +3148,20 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
         <v>Dense</v>
       </c>
       <c r="C12" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D12" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E12" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F12">
         <v>1</v>
@@ -3176,20 +3175,20 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
         <v>Crush</v>
       </c>
       <c r="C13" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="D13" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E13" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F13" s="6">
         <v>0.1</v>
@@ -3229,46 +3228,46 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>215</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="G1" s="4" t="s">
-        <v>218</v>
-      </c>
-      <c r="I1" s="16" t="s">
+      <c r="I1" s="4" t="s">
         <v>14</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B4" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Haunt</v>
       </c>
       <c r="C2" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D2" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="E2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="H2" t="str">
         <f>_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(E2:G2))</f>
@@ -3280,26 +3279,26 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Possesion</v>
       </c>
       <c r="C3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D3" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="E3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="H3" t="str">
         <f t="shared" ref="H3:H66" si="1">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(E3:G3))</f>
@@ -3311,26 +3310,26 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>230</v>
+        <v>228</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Trail</v>
       </c>
       <c r="C4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="E4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F4" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G4" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="H4" t="str">
         <f t="shared" si="1"/>
@@ -3342,26 +3341,26 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" ref="B5:B6" si="2">PROPER(SUBSTITUTE(A5,"_"," "))</f>
         <v>Kindling</v>
       </c>
       <c r="C5" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D5" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="E5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F5" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="G5" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H5" t="str">
         <f t="shared" si="1"/>
@@ -3373,26 +3372,26 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="2"/>
         <v>Spark</v>
       </c>
       <c r="C6" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D6" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="E6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="F6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="G6" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="H6" t="str">
         <f t="shared" si="1"/>
@@ -4003,31 +4002,31 @@
       </c>
     </row>
   </sheetData>
-  <conditionalFormatting sqref="E1:G5 I1">
-    <cfRule type="cellIs" dxfId="8" priority="5" operator="equal">
+  <conditionalFormatting sqref="E1:G89">
+    <cfRule type="cellIs" dxfId="8" priority="1" operator="equal">
       <formula>"Earth"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="7" priority="6" operator="equal">
+    <cfRule type="cellIs" dxfId="7" priority="2" operator="equal">
       <formula>"Water"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="6" priority="7" operator="equal">
+    <cfRule type="cellIs" dxfId="6" priority="3" operator="equal">
       <formula>"Fire"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="5" priority="8" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="4" operator="equal">
       <formula>"Air"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="E6:G89">
-    <cfRule type="cellIs" dxfId="4" priority="1" operator="equal">
+  <conditionalFormatting sqref="I1">
+    <cfRule type="cellIs" dxfId="4" priority="5" operator="equal">
       <formula>"Earth"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="3" priority="2" operator="equal">
+    <cfRule type="cellIs" dxfId="3" priority="6" operator="equal">
       <formula>"Water"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="2" priority="3" operator="equal">
+    <cfRule type="cellIs" dxfId="2" priority="7" operator="equal">
       <formula>"Fire"</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="1" priority="4" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="8" operator="equal">
       <formula>"Air"</formula>
     </cfRule>
   </conditionalFormatting>
@@ -4073,206 +4072,206 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B18" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Wayward</v>
       </c>
       <c r="C2" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Attracted</v>
       </c>
       <c r="C3" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>Spite</v>
+      </c>
+      <c r="C4" t="s">
         <v>171</v>
-      </c>
-      <c r="B4" t="str">
-        <f t="shared" si="0"/>
-        <v>Spite</v>
-      </c>
-      <c r="C4" t="s">
-        <v>172</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>Rooted</v>
+      </c>
+      <c r="C5" t="s">
         <v>173</v>
-      </c>
-      <c r="B5" t="str">
-        <f t="shared" si="0"/>
-        <v>Rooted</v>
-      </c>
-      <c r="C5" t="s">
-        <v>174</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Patrol</v>
       </c>
       <c r="C6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>176</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>Familiar</v>
+      </c>
+      <c r="C7" t="s">
         <v>177</v>
-      </c>
-      <c r="B7" t="str">
-        <f t="shared" si="0"/>
-        <v>Familiar</v>
-      </c>
-      <c r="C7" t="s">
-        <v>178</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>178</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>Rail</v>
+      </c>
+      <c r="C8" t="s">
         <v>179</v>
-      </c>
-      <c r="B8" t="str">
-        <f t="shared" si="0"/>
-        <v>Rail</v>
-      </c>
-      <c r="C8" t="s">
-        <v>180</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>180</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>Tide</v>
+      </c>
+      <c r="C9" t="s">
         <v>181</v>
-      </c>
-      <c r="B9" t="str">
-        <f t="shared" si="0"/>
-        <v>Tide</v>
-      </c>
-      <c r="C9" t="s">
-        <v>182</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>182</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>Blink</v>
+      </c>
+      <c r="C10" t="s">
         <v>183</v>
-      </c>
-      <c r="B10" t="str">
-        <f t="shared" si="0"/>
-        <v>Blink</v>
-      </c>
-      <c r="C10" t="s">
-        <v>184</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>184</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>Loyal</v>
+      </c>
+      <c r="C11" t="s">
         <v>185</v>
-      </c>
-      <c r="B11" t="str">
-        <f t="shared" si="0"/>
-        <v>Loyal</v>
-      </c>
-      <c r="C11" t="s">
-        <v>186</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>186</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>Hexed</v>
+      </c>
+      <c r="C12" t="s">
         <v>187</v>
-      </c>
-      <c r="B12" t="str">
-        <f t="shared" si="0"/>
-        <v>Hexed</v>
-      </c>
-      <c r="C12" t="s">
-        <v>188</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>188</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>Stalker</v>
+      </c>
+      <c r="C13" t="s">
         <v>189</v>
-      </c>
-      <c r="B13" t="str">
-        <f t="shared" si="0"/>
-        <v>Stalker</v>
-      </c>
-      <c r="C13" t="s">
-        <v>190</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v>Herd</v>
       </c>
       <c r="C14" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>191</v>
+      </c>
+      <c r="B15" t="str">
+        <f t="shared" si="0"/>
+        <v>Greedy</v>
+      </c>
+      <c r="C15" t="s">
         <v>192</v>
-      </c>
-      <c r="B15" t="str">
-        <f t="shared" si="0"/>
-        <v>Greedy</v>
-      </c>
-      <c r="C15" t="s">
-        <v>193</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>194</v>
+      </c>
+      <c r="B16" t="str">
+        <f t="shared" si="0"/>
+        <v>Oathbound</v>
+      </c>
+      <c r="C16" t="s">
         <v>195</v>
-      </c>
-      <c r="B16" t="str">
-        <f t="shared" si="0"/>
-        <v>Oathbound</v>
-      </c>
-      <c r="C16" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>196</v>
+      </c>
+      <c r="B17" t="str">
+        <f t="shared" si="0"/>
+        <v>Echo</v>
+      </c>
+      <c r="C17" t="s">
         <v>197</v>
-      </c>
-      <c r="B17" t="str">
-        <f t="shared" si="0"/>
-        <v>Echo</v>
-      </c>
-      <c r="C17" t="s">
-        <v>198</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>198</v>
+      </c>
+      <c r="B18" t="str">
+        <f t="shared" si="0"/>
+        <v>Phasing</v>
+      </c>
+      <c r="C18" t="s">
         <v>199</v>
-      </c>
-      <c r="B18" t="str">
-        <f t="shared" si="0"/>
-        <v>Phasing</v>
-      </c>
-      <c r="C18" t="s">
-        <v>200</v>
       </c>
     </row>
   </sheetData>
@@ -5980,19 +5979,19 @@
         <v>123</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="D2" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="F2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
   </sheetData>
@@ -6049,7 +6048,7 @@
         <v>123</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>119</v>
@@ -6060,7 +6059,7 @@
         <v>123</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>119</v>
@@ -6071,7 +6070,7 @@
         <v>123</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>119</v>
@@ -6082,7 +6081,7 @@
         <v>123</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>119</v>
@@ -6093,7 +6092,7 @@
         <v>123</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>119</v>
@@ -6104,7 +6103,7 @@
         <v>123</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>122</v>
@@ -6115,7 +6114,7 @@
         <v>123</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>122</v>
@@ -6126,7 +6125,7 @@
         <v>123</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>122</v>
@@ -6137,7 +6136,7 @@
         <v>123</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>122</v>
@@ -6148,7 +6147,7 @@
         <v>123</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>122</v>
@@ -6159,7 +6158,7 @@
         <v>123</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>122</v>
@@ -6170,7 +6169,7 @@
         <v>123</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>122</v>
@@ -6181,7 +6180,7 @@
         <v>123</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>122</v>
@@ -6192,7 +6191,7 @@
         <v>123</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>120</v>
@@ -6203,7 +6202,7 @@
         <v>123</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>120</v>
@@ -6214,7 +6213,7 @@
         <v>123</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>120</v>
@@ -6225,7 +6224,7 @@
         <v>123</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>120</v>
@@ -6255,7 +6254,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B23" s="12" t="s">
         <v>0</v>
@@ -6266,7 +6265,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B24" s="12" t="s">
         <v>1</v>
@@ -6277,7 +6276,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B25" s="12" t="s">
         <v>2</v>
@@ -6288,10 +6287,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="C26" s="12" t="s">
         <v>119</v>
@@ -6299,10 +6298,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C27" s="12" t="s">
         <v>119</v>
@@ -6310,10 +6309,10 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B28" s="12" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="C28" s="12" t="s">
         <v>122</v>
@@ -6321,10 +6320,10 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B29" s="12" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="C29" s="12" t="s">
         <v>122</v>
@@ -6332,10 +6331,10 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B30" s="12" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="C30" s="12" t="s">
         <v>122</v>
@@ -6343,7 +6342,7 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B31" s="15" t="s">
         <v>0</v>
@@ -6354,7 +6353,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>1</v>
@@ -6365,10 +6364,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="C33" s="15" t="s">
         <v>119</v>
@@ -6376,7 +6375,7 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B34" s="15" t="s">
         <v>2</v>
@@ -6387,10 +6386,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C35" s="15" t="s">
         <v>119</v>
@@ -6398,10 +6397,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C36" s="15" t="s">
         <v>119</v>
@@ -6409,10 +6408,10 @@
     </row>
     <row r="37" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="C37" s="15" t="s">
         <v>119</v>
@@ -6420,7 +6419,7 @@
     </row>
     <row r="38" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B38" s="15" t="s">
         <v>14</v>
@@ -6431,7 +6430,7 @@
     </row>
     <row r="39" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A39" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B39" s="14" t="s">
         <v>0</v>
@@ -6442,7 +6441,7 @@
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B40" s="14" t="s">
         <v>1</v>
@@ -6453,7 +6452,7 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B41" s="14" t="s">
         <v>2</v>

</xml_diff>

<commit_message>
Remove unused glyph assets and update particle effects
- Deleted unused glyph images (air, earth, fire, water) and their associated import files to streamline project assets.
- Updated the `glyph_rarity_particles.tscn` and `glyph.gd` files to refine particle effects and adjust rarity particle amounts for better visual feedback.
- Enhanced the `glyph.tscn` file to improve visibility settings for rarity particles, ensuring a more cohesive visual experience.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\One Last Bullet\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ABF32D9-303A-45E6-A6D4-93FEE1D1B812}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70D06406-E171-452E-A467-330327620DAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="489" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="236">
   <si>
     <t>id</t>
   </si>
@@ -483,9 +483,6 @@
     <t>rime</t>
   </si>
   <si>
-    <t>soft</t>
-  </si>
-  <si>
     <t>bounty</t>
   </si>
   <si>
@@ -751,6 +748,9 @@
   </si>
   <si>
     <t>No effect</t>
+  </si>
+  <si>
+    <t>sooth</t>
   </si>
 </sst>
 </file>
@@ -862,7 +862,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="17">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -881,6 +881,7 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1314,55 +1315,55 @@
         <v>4</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="E1" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="E1" s="4" t="s">
+      <c r="F1" s="4" t="s">
         <v>216</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="H1" s="4" t="s">
         <v>217</v>
       </c>
-      <c r="H1" s="4" t="s">
-        <v>218</v>
-      </c>
       <c r="I1" s="10" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="J1" s="9" t="s">
+        <v>154</v>
+      </c>
+      <c r="K1" s="9" t="s">
         <v>155</v>
       </c>
-      <c r="K1" s="9" t="s">
+      <c r="L1" s="9" t="s">
+        <v>159</v>
+      </c>
+      <c r="M1" s="9" t="s">
+        <v>160</v>
+      </c>
+      <c r="N1" s="9" t="s">
+        <v>157</v>
+      </c>
+      <c r="O1" s="9" t="s">
+        <v>158</v>
+      </c>
+      <c r="P1" s="9" t="s">
         <v>156</v>
       </c>
-      <c r="L1" s="9" t="s">
-        <v>160</v>
-      </c>
-      <c r="M1" s="9" t="s">
+      <c r="Q1" s="9" t="s">
+        <v>211</v>
+      </c>
+      <c r="R1" s="9" t="s">
         <v>161</v>
       </c>
-      <c r="N1" s="9" t="s">
-        <v>158</v>
-      </c>
-      <c r="O1" s="9" t="s">
-        <v>159</v>
-      </c>
-      <c r="P1" s="9" t="s">
-        <v>157</v>
-      </c>
-      <c r="Q1" s="9" t="s">
-        <v>212</v>
-      </c>
-      <c r="R1" s="9" t="s">
+      <c r="S1" s="9" t="s">
         <v>162</v>
       </c>
-      <c r="S1" s="9" t="s">
+      <c r="T1" s="9" t="s">
         <v>163</v>
       </c>
-      <c r="T1" s="9" t="s">
+      <c r="U1" s="9" t="s">
         <v>164</v>
-      </c>
-      <c r="U1" s="9" t="s">
-        <v>165</v>
       </c>
       <c r="V1" s="13" t="s">
         <v>109</v>
@@ -1373,21 +1374,21 @@
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B26" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Blank</v>
       </c>
       <c r="C2" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="H2" t="str">
         <f t="shared" ref="H2:H5" si="1">IF(ISBLANK(F2),"",IF(COUNTIF($G$2:$G$101,G2)=1,"Yes","No"))</f>
         <v/>
       </c>
       <c r="I2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J2">
         <v>10</v>
@@ -1426,7 +1427,7 @@
         <v>0</v>
       </c>
       <c r="V2" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="W2" t="b">
         <v>1</v>
@@ -1434,14 +1435,14 @@
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Conduit</v>
       </c>
       <c r="C3" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="D3" t="s">
         <v>132</v>
@@ -1461,7 +1462,7 @@
         <v>Yes</v>
       </c>
       <c r="I3" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J3">
         <v>10</v>
@@ -1500,7 +1501,7 @@
         <v>0</v>
       </c>
       <c r="V3" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="W3" t="b">
         <v>1</v>
@@ -1508,14 +1509,14 @@
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Rot</v>
       </c>
       <c r="C4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="D4" t="s">
         <v>136</v>
@@ -1535,7 +1536,7 @@
         <v>Yes</v>
       </c>
       <c r="I4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J4">
         <v>5</v>
@@ -1574,7 +1575,7 @@
         <v>3</v>
       </c>
       <c r="V4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="W4" t="b">
         <v>1</v>
@@ -1582,14 +1583,14 @@
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Ghost</v>
       </c>
       <c r="C5" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="D5" t="s">
         <v>132</v>
@@ -1609,7 +1610,7 @@
         <v>Yes</v>
       </c>
       <c r="I5" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J5">
         <v>10</v>
@@ -1648,7 +1649,7 @@
         <v>0</v>
       </c>
       <c r="V5" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="W5" t="b">
         <v>1</v>
@@ -1656,14 +1657,14 @@
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>225</v>
+      </c>
+      <c r="B6" t="str">
+        <f t="shared" si="0"/>
+        <v>Inferno</v>
+      </c>
+      <c r="C6" t="s">
         <v>226</v>
-      </c>
-      <c r="B6" t="str">
-        <f t="shared" si="0"/>
-        <v>Inferno</v>
-      </c>
-      <c r="C6" t="s">
-        <v>227</v>
       </c>
       <c r="D6" t="s">
         <v>125</v>
@@ -1683,7 +1684,7 @@
         <v>Yes</v>
       </c>
       <c r="I6" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="J6">
         <v>10</v>
@@ -2840,7 +2841,7 @@
   <sheetPr>
     <tabColor theme="7" tint="0.59999389629810485"/>
   </sheetPr>
-  <dimension ref="A1:H13"/>
+  <dimension ref="A1:I13"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="3" max="3" width="49.85546875" bestFit="1" customWidth="1"/>
@@ -2848,9 +2849,10 @@
     <col min="6" max="6" width="16.85546875" customWidth="1"/>
     <col min="7" max="7" width="12.85546875" customWidth="1"/>
     <col min="8" max="8" width="15.7109375" customWidth="1"/>
+    <col min="9" max="9" width="38" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A1" s="4" t="s">
         <v>0</v>
       </c>
@@ -2861,10 +2863,10 @@
         <v>2</v>
       </c>
       <c r="D1" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>139</v>
@@ -2875,8 +2877,11 @@
       <c r="H1" s="4" t="s">
         <v>141</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I1" s="16" t="s">
+        <v>109</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>142</v>
       </c>
@@ -2891,7 +2896,7 @@
         <v>125</v>
       </c>
       <c r="E2" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="F2">
         <v>1</v>
@@ -2902,8 +2907,12 @@
       <c r="H2">
         <v>3</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I2" t="str">
+        <f>"res://items/glyphs/"&amp;A2&amp;"_glyph.png"</f>
+        <v>res://items/glyphs/coal_glyph.png</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>143</v>
       </c>
@@ -2918,7 +2927,7 @@
         <v>125</v>
       </c>
       <c r="E3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="F3">
         <v>5</v>
@@ -2929,8 +2938,12 @@
       <c r="H3">
         <v>15</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I3" t="str">
+        <f t="shared" ref="I3:I13" si="1">"res://items/glyphs/"&amp;A3&amp;"_glyph.png"</f>
+        <v>res://items/glyphs/fury_glyph.png</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>144</v>
       </c>
@@ -2945,7 +2958,7 @@
         <v>125</v>
       </c>
       <c r="E4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="F4" s="6">
         <v>0.05</v>
@@ -2956,8 +2969,12 @@
       <c r="H4" s="6">
         <v>0.15</v>
       </c>
-    </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I4" t="str">
+        <f t="shared" si="1"/>
+        <v>res://items/glyphs/blast_glyph.png</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>145</v>
       </c>
@@ -2972,7 +2989,7 @@
         <v>129</v>
       </c>
       <c r="E5" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="F5">
         <v>1</v>
@@ -2983,14 +3000,18 @@
       <c r="H5">
         <v>3</v>
       </c>
-    </row>
-    <row r="6" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I5" t="str">
+        <f t="shared" si="1"/>
+        <v>res://items/glyphs/rime_glyph.png</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>146</v>
+        <v>235</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
-        <v>Soft</v>
+        <v>Sooth</v>
       </c>
       <c r="C6" t="s">
         <v>130</v>
@@ -2999,7 +3020,7 @@
         <v>129</v>
       </c>
       <c r="E6" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="F6">
         <v>-10</v>
@@ -3010,23 +3031,27 @@
       <c r="H6">
         <v>-30</v>
       </c>
-    </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I6" t="str">
+        <f t="shared" si="1"/>
+        <v>res://items/glyphs/sooth_glyph.png</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Bounty</v>
       </c>
       <c r="C7" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="D7" t="s">
         <v>129</v>
       </c>
       <c r="E7" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="F7" s="8">
         <v>0.01</v>
@@ -3037,10 +3062,14 @@
       <c r="H7" s="8">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="8" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I7" t="str">
+        <f t="shared" si="1"/>
+        <v>res://items/glyphs/bounty_glyph.png</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
@@ -3053,7 +3082,7 @@
         <v>132</v>
       </c>
       <c r="E8" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="F8">
         <v>1</v>
@@ -3064,10 +3093,14 @@
       <c r="H8">
         <v>3</v>
       </c>
-    </row>
-    <row r="9" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I8" t="str">
+        <f t="shared" si="1"/>
+        <v>res://items/glyphs/static_glyph.png</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
@@ -3080,7 +3113,7 @@
         <v>132</v>
       </c>
       <c r="E9" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="F9" s="6">
         <v>0.01</v>
@@ -3091,10 +3124,14 @@
       <c r="H9" s="6">
         <v>0.03</v>
       </c>
-    </row>
-    <row r="10" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I9" t="str">
+        <f t="shared" si="1"/>
+        <v>res://items/glyphs/shear_glyph.png</v>
+      </c>
+    </row>
+    <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
@@ -3107,7 +3144,7 @@
         <v>132</v>
       </c>
       <c r="E10" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="F10">
         <v>-10</v>
@@ -3118,10 +3155,14 @@
       <c r="H10">
         <v>-30</v>
       </c>
-    </row>
-    <row r="11" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I10" t="str">
+        <f t="shared" si="1"/>
+        <v>res://items/glyphs/drag_glyph.png</v>
+      </c>
+    </row>
+    <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
@@ -3134,7 +3175,7 @@
         <v>136</v>
       </c>
       <c r="E11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="F11">
         <v>1</v>
@@ -3145,10 +3186,14 @@
       <c r="H11">
         <v>3</v>
       </c>
-    </row>
-    <row r="12" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I11" t="str">
+        <f t="shared" si="1"/>
+        <v>res://items/glyphs/blight_glyph.png</v>
+      </c>
+    </row>
+    <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="0"/>
@@ -3161,7 +3206,7 @@
         <v>136</v>
       </c>
       <c r="E12" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="F12">
         <v>1</v>
@@ -3172,10 +3217,14 @@
       <c r="H12">
         <v>3</v>
       </c>
-    </row>
-    <row r="13" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="I12" t="str">
+        <f t="shared" si="1"/>
+        <v>res://items/glyphs/dense_glyph.png</v>
+      </c>
+    </row>
+    <row r="13" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B13" t="str">
         <f t="shared" si="0"/>
@@ -3188,7 +3237,7 @@
         <v>136</v>
       </c>
       <c r="E13" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="F13" s="6">
         <v>0.1</v>
@@ -3198,6 +3247,10 @@
       </c>
       <c r="H13" s="6">
         <v>0.3</v>
+      </c>
+      <c r="I13" t="str">
+        <f t="shared" si="1"/>
+        <v>res://items/glyphs/crush_glyph.png</v>
       </c>
     </row>
   </sheetData>
@@ -3228,19 +3281,19 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="F1" s="4" t="s">
         <v>215</v>
       </c>
-      <c r="F1" s="4" t="s">
+      <c r="G1" s="4" t="s">
         <v>216</v>
-      </c>
-      <c r="G1" s="4" t="s">
-        <v>217</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>14</v>
@@ -3248,17 +3301,17 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B4" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Haunt</v>
       </c>
       <c r="C2" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D2" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="E2" t="s">
         <v>132</v>
@@ -3279,17 +3332,17 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Possesion</v>
       </c>
       <c r="C3" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="D3" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="E3" t="s">
         <v>125</v>
@@ -3310,17 +3363,17 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>Trail</v>
+      </c>
+      <c r="C4" t="s">
+        <v>225</v>
+      </c>
+      <c r="D4" t="s">
         <v>228</v>
-      </c>
-      <c r="B4" t="str">
-        <f t="shared" si="0"/>
-        <v>Trail</v>
-      </c>
-      <c r="C4" t="s">
-        <v>226</v>
-      </c>
-      <c r="D4" t="s">
-        <v>229</v>
       </c>
       <c r="E4" t="s">
         <v>125</v>
@@ -3341,17 +3394,17 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" ref="B5:B6" si="2">PROPER(SUBSTITUTE(A5,"_"," "))</f>
         <v>Kindling</v>
       </c>
       <c r="C5" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D5" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="E5" t="s">
         <v>132</v>
@@ -3372,17 +3425,17 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="2"/>
         <v>Spark</v>
       </c>
       <c r="C6" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="D6" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="E6" t="s">
         <v>125</v>
@@ -4072,206 +4125,206 @@
     </row>
     <row r="2" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B18" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Wayward</v>
       </c>
       <c r="C2" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Attracted</v>
       </c>
       <c r="C3" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
     </row>
     <row r="4" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B4" t="str">
+        <f t="shared" si="0"/>
+        <v>Spite</v>
+      </c>
+      <c r="C4" t="s">
         <v>170</v>
-      </c>
-      <c r="B4" t="str">
-        <f t="shared" si="0"/>
-        <v>Spite</v>
-      </c>
-      <c r="C4" t="s">
-        <v>171</v>
       </c>
     </row>
     <row r="5" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>171</v>
+      </c>
+      <c r="B5" t="str">
+        <f t="shared" si="0"/>
+        <v>Rooted</v>
+      </c>
+      <c r="C5" t="s">
         <v>172</v>
-      </c>
-      <c r="B5" t="str">
-        <f t="shared" si="0"/>
-        <v>Rooted</v>
-      </c>
-      <c r="C5" t="s">
-        <v>173</v>
       </c>
     </row>
     <row r="6" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Patrol</v>
       </c>
       <c r="C6" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
     </row>
     <row r="7" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
+        <v>175</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="0"/>
+        <v>Familiar</v>
+      </c>
+      <c r="C7" t="s">
         <v>176</v>
-      </c>
-      <c r="B7" t="str">
-        <f t="shared" si="0"/>
-        <v>Familiar</v>
-      </c>
-      <c r="C7" t="s">
-        <v>177</v>
       </c>
     </row>
     <row r="8" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
+        <v>177</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="0"/>
+        <v>Rail</v>
+      </c>
+      <c r="C8" t="s">
         <v>178</v>
-      </c>
-      <c r="B8" t="str">
-        <f t="shared" si="0"/>
-        <v>Rail</v>
-      </c>
-      <c r="C8" t="s">
-        <v>179</v>
       </c>
     </row>
     <row r="9" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
+        <v>179</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="0"/>
+        <v>Tide</v>
+      </c>
+      <c r="C9" t="s">
         <v>180</v>
-      </c>
-      <c r="B9" t="str">
-        <f t="shared" si="0"/>
-        <v>Tide</v>
-      </c>
-      <c r="C9" t="s">
-        <v>181</v>
       </c>
     </row>
     <row r="10" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
+        <v>181</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="0"/>
+        <v>Blink</v>
+      </c>
+      <c r="C10" t="s">
         <v>182</v>
-      </c>
-      <c r="B10" t="str">
-        <f t="shared" si="0"/>
-        <v>Blink</v>
-      </c>
-      <c r="C10" t="s">
-        <v>183</v>
       </c>
     </row>
     <row r="11" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
+        <v>183</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="0"/>
+        <v>Loyal</v>
+      </c>
+      <c r="C11" t="s">
         <v>184</v>
-      </c>
-      <c r="B11" t="str">
-        <f t="shared" si="0"/>
-        <v>Loyal</v>
-      </c>
-      <c r="C11" t="s">
-        <v>185</v>
       </c>
     </row>
     <row r="12" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
+        <v>185</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="0"/>
+        <v>Hexed</v>
+      </c>
+      <c r="C12" t="s">
         <v>186</v>
-      </c>
-      <c r="B12" t="str">
-        <f t="shared" si="0"/>
-        <v>Hexed</v>
-      </c>
-      <c r="C12" t="s">
-        <v>187</v>
       </c>
     </row>
     <row r="13" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
+        <v>187</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="0"/>
+        <v>Stalker</v>
+      </c>
+      <c r="C13" t="s">
         <v>188</v>
-      </c>
-      <c r="B13" t="str">
-        <f t="shared" si="0"/>
-        <v>Stalker</v>
-      </c>
-      <c r="C13" t="s">
-        <v>189</v>
       </c>
     </row>
     <row r="14" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B14" t="str">
         <f t="shared" si="0"/>
         <v>Herd</v>
       </c>
       <c r="C14" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
+        <v>190</v>
+      </c>
+      <c r="B15" t="str">
+        <f t="shared" si="0"/>
+        <v>Greedy</v>
+      </c>
+      <c r="C15" t="s">
         <v>191</v>
-      </c>
-      <c r="B15" t="str">
-        <f t="shared" si="0"/>
-        <v>Greedy</v>
-      </c>
-      <c r="C15" t="s">
-        <v>192</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>193</v>
+      </c>
+      <c r="B16" t="str">
+        <f t="shared" si="0"/>
+        <v>Oathbound</v>
+      </c>
+      <c r="C16" t="s">
         <v>194</v>
-      </c>
-      <c r="B16" t="str">
-        <f t="shared" si="0"/>
-        <v>Oathbound</v>
-      </c>
-      <c r="C16" t="s">
-        <v>195</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>195</v>
+      </c>
+      <c r="B17" t="str">
+        <f t="shared" si="0"/>
+        <v>Echo</v>
+      </c>
+      <c r="C17" t="s">
         <v>196</v>
-      </c>
-      <c r="B17" t="str">
-        <f t="shared" si="0"/>
-        <v>Echo</v>
-      </c>
-      <c r="C17" t="s">
-        <v>197</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>197</v>
+      </c>
+      <c r="B18" t="str">
+        <f t="shared" si="0"/>
+        <v>Phasing</v>
+      </c>
+      <c r="C18" t="s">
         <v>198</v>
-      </c>
-      <c r="B18" t="str">
-        <f t="shared" si="0"/>
-        <v>Phasing</v>
-      </c>
-      <c r="C18" t="s">
-        <v>199</v>
       </c>
     </row>
   </sheetData>
@@ -5979,7 +6032,7 @@
         <v>123</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="C2" t="s">
         <v>125</v>
@@ -6004,7 +6057,7 @@
   <sheetPr>
     <tabColor theme="6" tint="-0.249977111117893"/>
   </sheetPr>
-  <dimension ref="A1:C41"/>
+  <dimension ref="A1:C42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="2" width="14.7109375" customWidth="1"/>
@@ -6059,7 +6112,7 @@
         <v>123</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>119</v>
@@ -6070,7 +6123,7 @@
         <v>123</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>119</v>
@@ -6081,7 +6134,7 @@
         <v>123</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>119</v>
@@ -6092,7 +6145,7 @@
         <v>123</v>
       </c>
       <c r="B8" s="11" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="C8" s="11" t="s">
         <v>119</v>
@@ -6103,7 +6156,7 @@
         <v>123</v>
       </c>
       <c r="B9" s="11" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="C9" s="11" t="s">
         <v>122</v>
@@ -6114,7 +6167,7 @@
         <v>123</v>
       </c>
       <c r="B10" s="11" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="C10" s="11" t="s">
         <v>122</v>
@@ -6125,7 +6178,7 @@
         <v>123</v>
       </c>
       <c r="B11" s="11" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="C11" s="11" t="s">
         <v>122</v>
@@ -6136,7 +6189,7 @@
         <v>123</v>
       </c>
       <c r="B12" s="11" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="C12" s="11" t="s">
         <v>122</v>
@@ -6147,7 +6200,7 @@
         <v>123</v>
       </c>
       <c r="B13" s="11" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="C13" s="11" t="s">
         <v>122</v>
@@ -6158,7 +6211,7 @@
         <v>123</v>
       </c>
       <c r="B14" s="11" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="C14" s="11" t="s">
         <v>122</v>
@@ -6169,7 +6222,7 @@
         <v>123</v>
       </c>
       <c r="B15" s="11" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="C15" s="11" t="s">
         <v>122</v>
@@ -6180,7 +6233,7 @@
         <v>123</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>122</v>
@@ -6191,7 +6244,7 @@
         <v>123</v>
       </c>
       <c r="B17" s="11" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="C17" s="11" t="s">
         <v>120</v>
@@ -6202,7 +6255,7 @@
         <v>123</v>
       </c>
       <c r="B18" s="11" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="C18" s="11" t="s">
         <v>120</v>
@@ -6213,7 +6266,7 @@
         <v>123</v>
       </c>
       <c r="B19" s="11" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="C19" s="11" t="s">
         <v>120</v>
@@ -6224,7 +6277,7 @@
         <v>123</v>
       </c>
       <c r="B20" s="11" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="C20" s="11" t="s">
         <v>120</v>
@@ -6254,7 +6307,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B23" s="12" t="s">
         <v>0</v>
@@ -6265,7 +6318,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B24" s="12" t="s">
         <v>1</v>
@@ -6276,7 +6329,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B25" s="12" t="s">
         <v>2</v>
@@ -6287,10 +6340,10 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B26" s="12" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="C26" s="12" t="s">
         <v>119</v>
@@ -6298,10 +6351,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="C27" s="12" t="s">
         <v>119</v>
@@ -6309,7 +6362,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B28" s="12" t="s">
         <v>139</v>
@@ -6320,7 +6373,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B29" s="12" t="s">
         <v>140</v>
@@ -6331,7 +6384,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B30" s="12" t="s">
         <v>141</v>
@@ -6341,22 +6394,22 @@
       </c>
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A31" s="15" t="s">
-        <v>221</v>
-      </c>
-      <c r="B31" s="15" t="s">
-        <v>0</v>
-      </c>
-      <c r="C31" s="15" t="s">
+      <c r="A31" s="12" t="s">
+        <v>205</v>
+      </c>
+      <c r="B31" s="12" t="s">
+        <v>109</v>
+      </c>
+      <c r="C31" s="12" t="s">
         <v>119</v>
       </c>
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B32" s="15" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C32" s="15" t="s">
         <v>119</v>
@@ -6364,10 +6417,10 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B33" s="15" t="s">
-        <v>220</v>
+        <v>1</v>
       </c>
       <c r="C33" s="15" t="s">
         <v>119</v>
@@ -6375,10 +6428,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>2</v>
+        <v>219</v>
       </c>
       <c r="C34" s="15" t="s">
         <v>119</v>
@@ -6386,10 +6439,10 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B35" s="15" t="s">
-        <v>215</v>
+        <v>2</v>
       </c>
       <c r="C35" s="15" t="s">
         <v>119</v>
@@ -6397,21 +6450,21 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="C36" s="15" t="s">
         <v>119</v>
       </c>
     </row>
-    <row r="37" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="C37" s="15" t="s">
         <v>119</v>
@@ -6419,32 +6472,32 @@
     </row>
     <row r="38" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B38" s="15" t="s">
+        <v>216</v>
+      </c>
+      <c r="C38" s="15" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="39" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A39" s="15" t="s">
+        <v>220</v>
+      </c>
+      <c r="B39" s="15" t="s">
         <v>14</v>
       </c>
-      <c r="C38" s="15" t="s">
+      <c r="C39" s="15" t="s">
         <v>121</v>
-      </c>
-    </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A39" s="14" t="s">
-        <v>167</v>
-      </c>
-      <c r="B39" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="C39" s="14" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="40" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A40" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B40" s="14" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C40" s="14" t="s">
         <v>119</v>
@@ -6452,12 +6505,23 @@
     </row>
     <row r="41" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A41" s="14" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B41" s="14" t="s">
+        <v>1</v>
+      </c>
+      <c r="C41" s="14" t="s">
+        <v>119</v>
+      </c>
+    </row>
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="14" t="s">
+        <v>166</v>
+      </c>
+      <c r="B42" s="14" t="s">
         <v>2</v>
       </c>
-      <c r="C41" s="14" t="s">
+      <c r="C42" s="14" t="s">
         <v>119</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update glyph mechanics and asset management
- Enhanced the glyph system to utilize per-id PNG textures from GameData, improving visual consistency and reducing hardcoded references.
- Updated the `Glyph` class to implement a caching mechanism for glyph textures, optimizing performance during gameplay.
- Revised project documentation to reflect the new texture management approach and updated glyph attributes, ensuring clarity for future development.
- Removed outdated references to elemental textures in favor of the new system, streamlining the codebase.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\One Last Bullet\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{70D06406-E171-452E-A467-330327620DAF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3323BB91-B6B3-42C1-8EA1-62FFBD700DB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -862,7 +862,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" quotePrefix="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -881,7 +881,6 @@
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2877,7 +2876,7 @@
       <c r="H1" s="4" t="s">
         <v>141</v>
       </c>
-      <c r="I1" s="16" t="s">
+      <c r="I1" s="4" t="s">
         <v>109</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update attribute icons and fix display formatting in ritual menu
- Renamed texture resources for critical chance and self-damage icons to improve clarity and consistency.
- Updated icon identifiers for various stats in the ritual menu, enhancing the user interface.
- Adjusted the display format for critical chance values to ensure consistent decimal representation.
- Replaced outdated references to damage icons with specific icons for each stat, streamlining the UI experience.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\One Last Bullet\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3323BB91-B6B3-42C1-8EA1-62FFBD700DB9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180A1645-971E-448D-B710-321AD7C2315F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="696" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4050" yWindow="5535" windowWidth="28800" windowHeight="15345" tabRatio="696" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="493" uniqueCount="236">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="250">
   <si>
     <t>id</t>
   </si>
@@ -751,6 +751,48 @@
   </si>
   <si>
     <t>sooth</t>
+  </si>
+  <si>
+    <t>shard</t>
+  </si>
+  <si>
+    <t>Shoots ice chards around every 3 seconds, doing 30 damage and inflicting 2 Frost</t>
+  </si>
+  <si>
+    <t>Beam now chains to enemies between you and the orb</t>
+  </si>
+  <si>
+    <t>More beams connect to other orbs and players</t>
+  </si>
+  <si>
+    <t>Range of the tether greatly increases</t>
+  </si>
+  <si>
+    <t>When a shard breaks, two smaller shards shoot out dealing 10 damage and inflicting 1 Chill</t>
+  </si>
+  <si>
+    <t>Shoots twice as many shards</t>
+  </si>
+  <si>
+    <t>If orb hits an enemy with 10 or more chill, kill it instantly</t>
+  </si>
+  <si>
+    <t>shatter</t>
+  </si>
+  <si>
+    <t>splinter</t>
+  </si>
+  <si>
+    <t>lethal</t>
+  </si>
+  <si>
+    <t>chain</t>
+  </si>
+  <si>
+    <t>conductor</t>
+  </si>
+  <si>
+    <t>reach</t>
   </si>
 </sst>
 </file>
@@ -1726,17 +1768,32 @@
       </c>
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>236</v>
+      </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>Shard</v>
+      </c>
+      <c r="C7" t="s">
+        <v>237</v>
+      </c>
+      <c r="D7" t="s">
+        <v>129</v>
+      </c>
+      <c r="E7" t="s">
+        <v>129</v>
+      </c>
+      <c r="F7" t="s">
+        <v>132</v>
       </c>
       <c r="G7" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Water|Water|Air</v>
       </c>
       <c r="H7" t="str">
         <f t="shared" ref="H7:H70" si="3">IF(ISBLANK(F7),"",IF(COUNTIF($G$2:$G$101,G7)=1,"Yes","No"))</f>
-        <v/>
+        <v>Yes</v>
       </c>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
@@ -2816,7 +2873,7 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" disablePrompts="1" count="2">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{DFC42C69-7304-40C7-BA02-8A3EB2712138}">
           <x14:formula1>
             <xm:f>motion!$A$2:$A$30</xm:f>
@@ -3396,7 +3453,7 @@
         <v>229</v>
       </c>
       <c r="B5" t="str">
-        <f t="shared" ref="B5:B6" si="2">PROPER(SUBSTITUTE(A5,"_"," "))</f>
+        <f t="shared" ref="B5:B12" si="2">PROPER(SUBSTITUTE(A5,"_"," "))</f>
         <v>Kindling</v>
       </c>
       <c r="C5" t="s">
@@ -3454,36 +3511,141 @@
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A7" t="s">
+        <v>247</v>
+      </c>
+      <c r="B7" t="str">
+        <f t="shared" si="2"/>
+        <v>Chain</v>
+      </c>
+      <c r="C7" t="s">
+        <v>200</v>
+      </c>
+      <c r="D7" t="s">
+        <v>238</v>
+      </c>
+      <c r="E7" t="s">
+        <v>129</v>
+      </c>
+      <c r="F7" t="s">
+        <v>132</v>
+      </c>
+      <c r="G7" t="s">
+        <v>125</v>
+      </c>
       <c r="H7" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Water|Air|Fire</v>
       </c>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>248</v>
+      </c>
+      <c r="B8" t="str">
+        <f t="shared" si="2"/>
+        <v>Conductor</v>
+      </c>
+      <c r="C8" t="s">
+        <v>200</v>
+      </c>
+      <c r="D8" t="s">
+        <v>239</v>
+      </c>
+      <c r="E8" t="s">
+        <v>132</v>
+      </c>
+      <c r="F8" t="s">
+        <v>129</v>
+      </c>
+      <c r="G8" t="s">
+        <v>129</v>
+      </c>
       <c r="H8" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Air|Water|Water</v>
       </c>
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>249</v>
+      </c>
+      <c r="B9" t="str">
+        <f t="shared" si="2"/>
+        <v>Reach</v>
+      </c>
+      <c r="C9" t="s">
+        <v>200</v>
+      </c>
+      <c r="D9" t="s">
+        <v>240</v>
+      </c>
+      <c r="E9" t="s">
+        <v>132</v>
+      </c>
+      <c r="F9" t="s">
+        <v>136</v>
+      </c>
+      <c r="G9" t="s">
+        <v>136</v>
+      </c>
       <c r="H9" t="str">
         <f t="shared" si="1"/>
-        <v/>
+        <v>Air|Earth|Earth</v>
       </c>
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>245</v>
+      </c>
+      <c r="B10" t="str">
+        <f t="shared" si="2"/>
+        <v>Splinter</v>
+      </c>
+      <c r="C10" t="s">
+        <v>236</v>
+      </c>
+      <c r="D10" t="s">
+        <v>241</v>
+      </c>
       <c r="H10" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>246</v>
+      </c>
+      <c r="B11" t="str">
+        <f t="shared" si="2"/>
+        <v>Lethal</v>
+      </c>
+      <c r="C11" t="s">
+        <v>236</v>
+      </c>
+      <c r="D11" t="s">
+        <v>242</v>
+      </c>
       <c r="H11" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A12" t="s">
+        <v>244</v>
+      </c>
+      <c r="B12" t="str">
+        <f t="shared" si="2"/>
+        <v>Shatter</v>
+      </c>
+      <c r="C12" t="s">
+        <v>236</v>
+      </c>
+      <c r="D12" t="s">
+        <v>243</v>
+      </c>
       <c r="H12" t="str">
         <f t="shared" si="1"/>
         <v/>

</xml_diff>

<commit_message>
Enhance dash mechanics and resolve collision issues
- Updated the dash component to include a new end-of-dash collision resolution mechanism, ensuring players do not end their dash inside world geometry.
- Implemented a stuck watchdog for players, allowing them to unstick from obstacles after a set number of overlapping frames.
- Revised project documentation to reflect changes in dash mechanics and collision handling, improving clarity for future development.
- Removed the outdated rot orb and updated orb references in the level configuration to streamline asset management.
</commit_message>
<xml_diff>
--- a/project/data/game_data.xlsx
+++ b/project/data/game_data.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Programming Projects\Game Dev\One Last Bullet\project\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{180A1645-971E-448D-B710-321AD7C2315F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F88551BE-FB3D-4078-9BD6-52BD9070121E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4050" yWindow="5535" windowWidth="28800" windowHeight="15345" tabRatio="696" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4050" yWindow="5535" windowWidth="28800" windowHeight="15345" tabRatio="696" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="orbs" sheetId="1" r:id="rId1"/>
@@ -43,7 +43,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="525" uniqueCount="250">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="589" uniqueCount="276">
   <si>
     <t>id</t>
   </si>
@@ -618,9 +618,6 @@
     <t>greedy</t>
   </si>
   <si>
-    <t>Steers towards mana crystals</t>
-  </si>
-  <si>
     <t>Steer towards other orbs</t>
   </si>
   <si>
@@ -648,18 +645,12 @@
     <t>conduit</t>
   </si>
   <si>
-    <t>rot</t>
-  </si>
-  <si>
     <t>ghost</t>
   </si>
   <si>
     <t>When you are within 120 meters of the orb, create a tether between you dealing 3 DPS to enemies touching it</t>
   </si>
   <si>
-    <t>Inflict poison on hit</t>
-  </si>
-  <si>
     <t>glyphs</t>
   </si>
   <si>
@@ -793,6 +784,93 @@
   </si>
   <si>
     <t>reach</t>
+  </si>
+  <si>
+    <t>contagion</t>
+  </si>
+  <si>
+    <t>On enemy death, a putrid cloud is left inflicting 1 poison on passing enemies</t>
+  </si>
+  <si>
+    <t>All poison stacks spread on death</t>
+  </si>
+  <si>
+    <t>virulence</t>
+  </si>
+  <si>
+    <t>carrion</t>
+  </si>
+  <si>
+    <t>outbreak</t>
+  </si>
+  <si>
+    <t>runic</t>
+  </si>
+  <si>
+    <t>Picks up glyphs instead of damaging them. Gets 5% damage increase for each deposited.</t>
+  </si>
+  <si>
+    <t>improve</t>
+  </si>
+  <si>
+    <t>Any picked up glyph goes up in rarity</t>
+  </si>
+  <si>
+    <t>Gets 5% damage increase for each deposited glyph</t>
+  </si>
+  <si>
+    <t>hoarder</t>
+  </si>
+  <si>
+    <t>mend</t>
+  </si>
+  <si>
+    <t>Does no self-damage. Players hit heal 10 hp instead</t>
+  </si>
+  <si>
+    <t>Creates a shield around the orb. Any players within it take 50% less damage.</t>
+  </si>
+  <si>
+    <t>guardian</t>
+  </si>
+  <si>
+    <t>destroyer</t>
+  </si>
+  <si>
+    <t>High damage. Inflicts Burn, Frost and Poison. Chases the nearest player</t>
+  </si>
+  <si>
+    <t>While holding a glyph, inflict 5 of that glyphs corresponding elemental status to any hit enemies (burn, chill, shock or poison)</t>
+  </si>
+  <si>
+    <t>affinity</t>
+  </si>
+  <si>
+    <t>Shield reflects enemy projectiles back at them</t>
+  </si>
+  <si>
+    <t>retribution</t>
+  </si>
+  <si>
+    <t>Greatly extends the shields area</t>
+  </si>
+  <si>
+    <t>shield</t>
+  </si>
+  <si>
+    <t>While in the shield, players can dash with no cooldown</t>
+  </si>
+  <si>
+    <t>flexible</t>
+  </si>
+  <si>
+    <t>Steers towards glyphs</t>
+  </si>
+  <si>
+    <t>Nearby enemies also get Disease status along with the poison</t>
+  </si>
+  <si>
+    <t>20% chance of adding Disease status to enemies. On death half their poison spreads to other nearby enemies</t>
   </si>
 </sst>
 </file>
@@ -1356,16 +1434,16 @@
         <v>4</v>
       </c>
       <c r="D1" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="E1" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="F1" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="H1" s="4" t="s">
         <v>214</v>
-      </c>
-      <c r="E1" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="F1" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="H1" s="4" t="s">
-        <v>217</v>
       </c>
       <c r="I1" s="10" t="s">
         <v>166</v>
@@ -1392,7 +1470,7 @@
         <v>156</v>
       </c>
       <c r="Q1" s="9" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="R1" s="9" t="s">
         <v>161</v>
@@ -1415,14 +1493,14 @@
     </row>
     <row r="2" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B26" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Blank</v>
       </c>
       <c r="C2" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="H2" t="str">
         <f t="shared" ref="H2:H5" si="1">IF(ISBLANK(F2),"",IF(COUNTIF($G$2:$G$101,G2)=1,"Yes","No"))</f>
@@ -1468,7 +1546,7 @@
         <v>0</v>
       </c>
       <c r="V2" t="s">
-        <v>206</v>
+        <v>203</v>
       </c>
       <c r="W2" t="b">
         <v>1</v>
@@ -1476,14 +1554,14 @@
     </row>
     <row r="3" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
         <v>Conduit</v>
       </c>
       <c r="C3" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D3" t="s">
         <v>132</v>
@@ -1542,7 +1620,7 @@
         <v>0</v>
       </c>
       <c r="V3" t="s">
-        <v>207</v>
+        <v>204</v>
       </c>
       <c r="W3" t="b">
         <v>1</v>
@@ -1550,14 +1628,14 @@
     </row>
     <row r="4" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>201</v>
+        <v>247</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
-        <v>Rot</v>
+        <v>Contagion</v>
       </c>
       <c r="C4" t="s">
-        <v>204</v>
+        <v>275</v>
       </c>
       <c r="D4" t="s">
         <v>136</v>
@@ -1566,11 +1644,11 @@
         <v>136</v>
       </c>
       <c r="F4" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="G4" t="str">
         <f t="shared" ref="G4:G67" si="2">_xlfn.TEXTJOIN("|",TRUE,_xlfn._xlws.SORT(D4:F4))</f>
-        <v>Earth|Earth|Water</v>
+        <v>Earth|Earth|Air</v>
       </c>
       <c r="H4" t="str">
         <f t="shared" si="1"/>
@@ -1616,7 +1694,7 @@
         <v>3</v>
       </c>
       <c r="V4" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="W4" t="b">
         <v>1</v>
@@ -1624,14 +1702,14 @@
     </row>
     <row r="5" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B5" t="str">
         <f t="shared" si="0"/>
         <v>Ghost</v>
       </c>
       <c r="C5" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D5" t="s">
         <v>132</v>
@@ -1690,7 +1768,7 @@
         <v>0</v>
       </c>
       <c r="V5" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="W5" t="b">
         <v>1</v>
@@ -1698,14 +1776,14 @@
     </row>
     <row r="6" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
         <v>Inferno</v>
       </c>
       <c r="C6" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="D6" t="s">
         <v>125</v>
@@ -1769,14 +1847,14 @@
     </row>
     <row r="7" spans="1:23" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="0"/>
         <v>Shard</v>
       </c>
       <c r="C7" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D7" t="s">
         <v>129</v>
@@ -1797,59 +1875,131 @@
       </c>
     </row>
     <row r="8" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A8" t="s">
+        <v>253</v>
+      </c>
       <c r="B8" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>Runic</v>
+      </c>
+      <c r="C8" t="s">
+        <v>254</v>
+      </c>
+      <c r="D8" t="s">
+        <v>129</v>
+      </c>
+      <c r="E8" t="s">
+        <v>129</v>
+      </c>
+      <c r="F8" t="s">
+        <v>129</v>
       </c>
       <c r="G8" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Water|Water|Water</v>
       </c>
       <c r="H8" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>Yes</v>
       </c>
     </row>
     <row r="9" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A9" t="s">
+        <v>262</v>
+      </c>
       <c r="B9" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>Guardian</v>
+      </c>
+      <c r="C9" t="s">
+        <v>261</v>
+      </c>
+      <c r="D9" t="s">
+        <v>129</v>
+      </c>
+      <c r="E9" t="s">
+        <v>129</v>
+      </c>
+      <c r="F9" t="s">
+        <v>136</v>
       </c>
       <c r="G9" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Water|Water|Earth</v>
       </c>
       <c r="H9" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>Yes</v>
       </c>
     </row>
     <row r="10" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A10" t="s">
+        <v>259</v>
+      </c>
       <c r="B10" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>Mend</v>
+      </c>
+      <c r="C10" t="s">
+        <v>260</v>
+      </c>
+      <c r="D10" t="s">
+        <v>136</v>
+      </c>
+      <c r="E10" t="s">
+        <v>136</v>
+      </c>
+      <c r="F10" t="s">
+        <v>129</v>
       </c>
       <c r="G10" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Earth|Earth|Water</v>
       </c>
       <c r="H10" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>Yes</v>
+      </c>
+      <c r="I10" t="s">
+        <v>165</v>
       </c>
     </row>
     <row r="11" spans="1:23" x14ac:dyDescent="0.25">
+      <c r="A11" t="s">
+        <v>263</v>
+      </c>
       <c r="B11" t="str">
         <f t="shared" si="0"/>
-        <v/>
+        <v>Destroyer</v>
+      </c>
+      <c r="C11" t="s">
+        <v>264</v>
+      </c>
+      <c r="D11" t="s">
+        <v>125</v>
+      </c>
+      <c r="E11" t="s">
+        <v>132</v>
+      </c>
+      <c r="F11" t="s">
+        <v>136</v>
       </c>
       <c r="G11" t="str">
         <f t="shared" si="2"/>
-        <v/>
+        <v>Fire|Air|Earth</v>
       </c>
       <c r="H11" t="str">
         <f t="shared" si="3"/>
-        <v/>
+        <v>Yes</v>
+      </c>
+      <c r="I11" t="s">
+        <v>169</v>
+      </c>
+      <c r="J11">
+        <v>50</v>
+      </c>
+      <c r="K11">
+        <v>50</v>
       </c>
     </row>
     <row r="12" spans="1:23" x14ac:dyDescent="0.25">
@@ -2922,7 +3072,7 @@
         <v>152</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="F1" s="4" t="s">
         <v>139</v>
@@ -3063,7 +3213,7 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="0"/>
@@ -3101,13 +3251,13 @@
         <v>Bounty</v>
       </c>
       <c r="C7" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D7" t="s">
         <v>129</v>
       </c>
       <c r="E7" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="F7" s="8">
         <v>0.01</v>
@@ -3324,6 +3474,7 @@
   <cols>
     <col min="1" max="1" width="12.7109375" customWidth="1"/>
     <col min="2" max="2" width="13.7109375" customWidth="1"/>
+    <col min="3" max="3" width="9.7109375" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="94.140625" bestFit="1" customWidth="1"/>
     <col min="5" max="7" width="10.5703125" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="0" hidden="1" customWidth="1"/>
@@ -3337,19 +3488,19 @@
         <v>1</v>
       </c>
       <c r="C1" s="4" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D1" s="4" t="s">
         <v>2</v>
       </c>
       <c r="E1" s="4" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="F1" s="4" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="G1" s="4" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="I1" s="4" t="s">
         <v>14</v>
@@ -3357,17 +3508,17 @@
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="B2" t="str">
         <f t="shared" ref="B2:B4" si="0">PROPER(SUBSTITUTE(A2,"_"," "))</f>
         <v>Haunt</v>
       </c>
       <c r="C2" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D2" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="E2" t="s">
         <v>132</v>
@@ -3388,17 +3539,17 @@
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
+        <v>218</v>
+      </c>
+      <c r="B3" t="str">
+        <f t="shared" si="0"/>
+        <v>Possesion</v>
+      </c>
+      <c r="C3" t="s">
+        <v>200</v>
+      </c>
+      <c r="D3" t="s">
         <v>221</v>
-      </c>
-      <c r="B3" t="str">
-        <f t="shared" si="0"/>
-        <v>Possesion</v>
-      </c>
-      <c r="C3" t="s">
-        <v>202</v>
-      </c>
-      <c r="D3" t="s">
-        <v>224</v>
       </c>
       <c r="E3" t="s">
         <v>125</v>
@@ -3419,17 +3570,17 @@
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>227</v>
+        <v>224</v>
       </c>
       <c r="B4" t="str">
         <f t="shared" si="0"/>
         <v>Trail</v>
       </c>
       <c r="C4" t="s">
+        <v>222</v>
+      </c>
+      <c r="D4" t="s">
         <v>225</v>
-      </c>
-      <c r="D4" t="s">
-        <v>228</v>
       </c>
       <c r="E4" t="s">
         <v>125</v>
@@ -3450,17 +3601,17 @@
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>229</v>
+        <v>226</v>
       </c>
       <c r="B5" t="str">
-        <f t="shared" ref="B5:B12" si="2">PROPER(SUBSTITUTE(A5,"_"," "))</f>
+        <f t="shared" ref="B5:B20" si="2">PROPER(SUBSTITUTE(A5,"_"," "))</f>
         <v>Kindling</v>
       </c>
       <c r="C5" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D5" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="E5" t="s">
         <v>132</v>
@@ -3481,17 +3632,17 @@
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="B6" t="str">
         <f t="shared" si="2"/>
         <v>Spark</v>
       </c>
       <c r="C6" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D6" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="E6" t="s">
         <v>125</v>
@@ -3512,17 +3663,17 @@
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="B7" t="str">
         <f t="shared" si="2"/>
         <v>Chain</v>
       </c>
       <c r="C7" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D7" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="E7" t="s">
         <v>129</v>
@@ -3540,17 +3691,17 @@
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="B8" t="str">
         <f t="shared" si="2"/>
         <v>Conductor</v>
       </c>
       <c r="C8" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D8" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="E8" t="s">
         <v>132</v>
@@ -3568,17 +3719,17 @@
     </row>
     <row r="9" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="B9" t="str">
         <f t="shared" si="2"/>
         <v>Reach</v>
       </c>
       <c r="C9" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="D9" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="E9" t="s">
         <v>132</v>
@@ -3596,17 +3747,17 @@
     </row>
     <row r="10" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="B10" t="str">
         <f t="shared" si="2"/>
         <v>Splinter</v>
       </c>
       <c r="C10" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D10" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="H10" t="str">
         <f t="shared" si="1"/>
@@ -3615,17 +3766,17 @@
     </row>
     <row r="11" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="B11" t="str">
         <f t="shared" si="2"/>
         <v>Lethal</v>
       </c>
       <c r="C11" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D11" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="H11" t="str">
         <f t="shared" si="1"/>
@@ -3634,17 +3785,17 @@
     </row>
     <row r="12" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="B12" t="str">
         <f t="shared" si="2"/>
         <v>Shatter</v>
       </c>
       <c r="C12" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D12" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="H12" t="str">
         <f t="shared" si="1"/>
@@ -3652,120 +3803,278 @@
       </c>
     </row>
     <row r="13" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A13" t="s">
+        <v>251</v>
+      </c>
+      <c r="B13" t="str">
+        <f t="shared" si="2"/>
+        <v>Carrion</v>
+      </c>
+      <c r="C13" t="s">
+        <v>247</v>
+      </c>
+      <c r="D13" t="s">
+        <v>248</v>
+      </c>
       <c r="H13" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="14" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A14" t="s">
+        <v>252</v>
+      </c>
+      <c r="B14" t="str">
+        <f t="shared" si="2"/>
+        <v>Outbreak</v>
+      </c>
+      <c r="C14" t="s">
+        <v>247</v>
+      </c>
+      <c r="D14" t="s">
+        <v>274</v>
+      </c>
       <c r="H14" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="15" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A15" t="s">
+        <v>250</v>
+      </c>
+      <c r="B15" t="str">
+        <f t="shared" si="2"/>
+        <v>Virulence</v>
+      </c>
+      <c r="C15" t="s">
+        <v>247</v>
+      </c>
+      <c r="D15" t="s">
+        <v>249</v>
+      </c>
       <c r="H15" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
     <row r="16" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A16" t="s">
+        <v>255</v>
+      </c>
+      <c r="B16" t="str">
+        <f t="shared" si="2"/>
+        <v>Improve</v>
+      </c>
+      <c r="C16" t="s">
+        <v>253</v>
+      </c>
+      <c r="D16" t="s">
+        <v>256</v>
+      </c>
+      <c r="E16" t="s">
+        <v>129</v>
+      </c>
+      <c r="F16" t="s">
+        <v>129</v>
+      </c>
+      <c r="G16" t="s">
+        <v>136</v>
+      </c>
       <c r="H16" t="str">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="17" spans="8:8" x14ac:dyDescent="0.25">
+        <v>Water|Water|Earth</v>
+      </c>
+    </row>
+    <row r="17" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A17" t="s">
+        <v>258</v>
+      </c>
+      <c r="B17" t="str">
+        <f t="shared" si="2"/>
+        <v>Hoarder</v>
+      </c>
+      <c r="C17" t="s">
+        <v>253</v>
+      </c>
+      <c r="D17" t="s">
+        <v>257</v>
+      </c>
+      <c r="E17" t="s">
+        <v>125</v>
+      </c>
+      <c r="F17" t="s">
+        <v>125</v>
+      </c>
+      <c r="G17" t="s">
+        <v>125</v>
+      </c>
       <c r="H17" t="str">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="18" spans="8:8" x14ac:dyDescent="0.25">
+        <v>Fire|Fire|Fire</v>
+      </c>
+    </row>
+    <row r="18" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A18" t="s">
+        <v>266</v>
+      </c>
+      <c r="B18" t="str">
+        <f t="shared" si="2"/>
+        <v>Affinity</v>
+      </c>
+      <c r="C18" t="s">
+        <v>253</v>
+      </c>
+      <c r="D18" t="s">
+        <v>265</v>
+      </c>
+      <c r="E18" t="s">
+        <v>136</v>
+      </c>
+      <c r="F18" t="s">
+        <v>136</v>
+      </c>
+      <c r="G18" t="s">
+        <v>125</v>
+      </c>
       <c r="H18" t="str">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="19" spans="8:8" x14ac:dyDescent="0.25">
+        <v>Earth|Earth|Fire</v>
+      </c>
+    </row>
+    <row r="19" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A19" t="s">
+        <v>268</v>
+      </c>
+      <c r="B19" t="str">
+        <f t="shared" si="2"/>
+        <v>Retribution</v>
+      </c>
+      <c r="C19" t="s">
+        <v>262</v>
+      </c>
+      <c r="D19" t="s">
+        <v>267</v>
+      </c>
+      <c r="E19" t="s">
+        <v>125</v>
+      </c>
+      <c r="F19" t="s">
+        <v>125</v>
+      </c>
+      <c r="G19" t="s">
+        <v>136</v>
+      </c>
       <c r="H19" t="str">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="8:8" x14ac:dyDescent="0.25">
+        <v>Fire|Fire|Earth</v>
+      </c>
+    </row>
+    <row r="20" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A20" t="s">
+        <v>272</v>
+      </c>
+      <c r="B20" t="str">
+        <f t="shared" si="2"/>
+        <v>Flexible</v>
+      </c>
+      <c r="C20" t="s">
+        <v>262</v>
+      </c>
+      <c r="D20" t="s">
+        <v>271</v>
+      </c>
+      <c r="E20" t="s">
+        <v>132</v>
+      </c>
+      <c r="F20" t="s">
+        <v>132</v>
+      </c>
+      <c r="G20" t="s">
+        <v>129</v>
+      </c>
       <c r="H20" t="str">
         <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="8:8" x14ac:dyDescent="0.25">
+        <v>Air|Air|Water</v>
+      </c>
+    </row>
+    <row r="21" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="A21" t="s">
+        <v>270</v>
+      </c>
+      <c r="C21" t="s">
+        <v>262</v>
+      </c>
+      <c r="D21" t="s">
+        <v>269</v>
+      </c>
       <c r="H21" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="22" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H22" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="23" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H23" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="24" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H24" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="25" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H25" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="26" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H26" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="27" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H27" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="28" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H28" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="29" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H29" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="30" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H30" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="31" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H31" t="str">
         <f t="shared" si="1"/>
         <v/>
       </c>
     </row>
-    <row r="32" spans="8:8" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:8" x14ac:dyDescent="0.25">
       <c r="H32" t="str">
         <f t="shared" si="1"/>
         <v/>
@@ -4247,12 +4556,18 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{CCE6A557-97BC-4b89-ADB6-D9C93CAAB3DF}">
-      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="1">
+      <x14:dataValidations xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main" count="2">
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{B44CB842-296D-43B5-8EC4-12AD766FB2C3}">
           <x14:formula1>
             <xm:f>input!$C$2:$F$2</xm:f>
           </x14:formula1>
           <xm:sqref>E2:G89</xm:sqref>
+        </x14:dataValidation>
+        <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" xr:uid="{55B61686-C713-47B1-9060-9045630E3352}">
+          <x14:formula1>
+            <xm:f>orbs!$A$2:$A$43</xm:f>
+          </x14:formula1>
+          <xm:sqref>C2:C100</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -4268,7 +4583,7 @@
   <dimension ref="A1:C18"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="9.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" customWidth="1"/>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="46.42578125" customWidth="1"/>
   </cols>
@@ -4298,7 +4613,7 @@
     </row>
     <row r="3" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="B3" t="str">
         <f t="shared" si="0"/>
@@ -4437,7 +4752,7 @@
         <v>Herd</v>
       </c>
       <c r="C14" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
     </row>
     <row r="15" spans="1:3" x14ac:dyDescent="0.25">
@@ -4449,43 +4764,43 @@
         <v>Greedy</v>
       </c>
       <c r="C15" t="s">
-        <v>191</v>
+        <v>273</v>
       </c>
     </row>
     <row r="16" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>192</v>
+      </c>
+      <c r="B16" t="str">
+        <f t="shared" si="0"/>
+        <v>Oathbound</v>
+      </c>
+      <c r="C16" t="s">
         <v>193</v>
-      </c>
-      <c r="B16" t="str">
-        <f t="shared" si="0"/>
-        <v>Oathbound</v>
-      </c>
-      <c r="C16" t="s">
-        <v>194</v>
       </c>
     </row>
     <row r="17" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
+        <v>194</v>
+      </c>
+      <c r="B17" t="str">
+        <f t="shared" si="0"/>
+        <v>Echo</v>
+      </c>
+      <c r="C17" t="s">
         <v>195</v>
-      </c>
-      <c r="B17" t="str">
-        <f t="shared" si="0"/>
-        <v>Echo</v>
-      </c>
-      <c r="C17" t="s">
-        <v>196</v>
       </c>
     </row>
     <row r="18" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>196</v>
+      </c>
+      <c r="B18" t="str">
+        <f t="shared" si="0"/>
+        <v>Phasing</v>
+      </c>
+      <c r="C18" t="s">
         <v>197</v>
-      </c>
-      <c r="B18" t="str">
-        <f t="shared" si="0"/>
-        <v>Phasing</v>
-      </c>
-      <c r="C18" t="s">
-        <v>198</v>
       </c>
     </row>
   </sheetData>
@@ -6193,7 +6508,7 @@
         <v>123</v>
       </c>
       <c r="B2" s="3" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="C2" t="s">
         <v>125</v>
@@ -6273,7 +6588,7 @@
         <v>123</v>
       </c>
       <c r="B5" s="11" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C5" s="11" t="s">
         <v>119</v>
@@ -6284,7 +6599,7 @@
         <v>123</v>
       </c>
       <c r="B6" s="11" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C6" s="11" t="s">
         <v>119</v>
@@ -6295,7 +6610,7 @@
         <v>123</v>
       </c>
       <c r="B7" s="11" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C7" s="11" t="s">
         <v>119</v>
@@ -6394,7 +6709,7 @@
         <v>123</v>
       </c>
       <c r="B16" s="11" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="C16" s="11" t="s">
         <v>122</v>
@@ -6468,7 +6783,7 @@
     </row>
     <row r="23" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A23" s="12" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B23" s="12" t="s">
         <v>0</v>
@@ -6479,7 +6794,7 @@
     </row>
     <row r="24" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A24" s="12" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B24" s="12" t="s">
         <v>1</v>
@@ -6490,7 +6805,7 @@
     </row>
     <row r="25" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A25" s="12" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B25" s="12" t="s">
         <v>2</v>
@@ -6501,7 +6816,7 @@
     </row>
     <row r="26" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A26" s="12" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B26" s="12" t="s">
         <v>152</v>
@@ -6512,10 +6827,10 @@
     </row>
     <row r="27" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A27" s="12" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B27" s="12" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="C27" s="12" t="s">
         <v>119</v>
@@ -6523,7 +6838,7 @@
     </row>
     <row r="28" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A28" s="12" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B28" s="12" t="s">
         <v>139</v>
@@ -6534,7 +6849,7 @@
     </row>
     <row r="29" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A29" s="12" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B29" s="12" t="s">
         <v>140</v>
@@ -6545,7 +6860,7 @@
     </row>
     <row r="30" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A30" s="12" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B30" s="12" t="s">
         <v>141</v>
@@ -6556,7 +6871,7 @@
     </row>
     <row r="31" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A31" s="12" t="s">
-        <v>205</v>
+        <v>202</v>
       </c>
       <c r="B31" s="12" t="s">
         <v>109</v>
@@ -6567,7 +6882,7 @@
     </row>
     <row r="32" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A32" s="15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B32" s="15" t="s">
         <v>0</v>
@@ -6578,7 +6893,7 @@
     </row>
     <row r="33" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A33" s="15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B33" s="15" t="s">
         <v>1</v>
@@ -6589,10 +6904,10 @@
     </row>
     <row r="34" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A34" s="15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B34" s="15" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="C34" s="15" t="s">
         <v>119</v>
@@ -6600,7 +6915,7 @@
     </row>
     <row r="35" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A35" s="15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B35" s="15" t="s">
         <v>2</v>
@@ -6611,10 +6926,10 @@
     </row>
     <row r="36" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A36" s="15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B36" s="15" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="C36" s="15" t="s">
         <v>119</v>
@@ -6622,10 +6937,10 @@
     </row>
     <row r="37" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A37" s="15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B37" s="15" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C37" s="15" t="s">
         <v>119</v>
@@ -6633,10 +6948,10 @@
     </row>
     <row r="38" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A38" s="15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B38" s="15" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="C38" s="15" t="s">
         <v>119</v>
@@ -6644,7 +6959,7 @@
     </row>
     <row r="39" spans="1:3" ht="15.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A39" s="15" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B39" s="15" t="s">
         <v>14</v>

</xml_diff>